<commit_message>
MIA: run automatico 2026-07-29 18:51 UTC
</commit_message>
<xml_diff>
--- a/database/ASAI3.xlsx
+++ b/database/ASAI3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1352"/>
+  <dimension ref="A1:F1353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,16 +512,16 @@
         <v>44259</v>
       </c>
       <c r="B5" t="n">
-        <v>13.90097713470459</v>
+        <v>13.90097618103027</v>
       </c>
       <c r="C5" t="n">
-        <v>14.04340481356423</v>
+        <v>14.04340385011868</v>
       </c>
       <c r="D5" t="n">
-        <v>13.44330802948757</v>
+        <v>13.44330710721157</v>
       </c>
       <c r="E5" t="n">
-        <v>13.53256280482981</v>
+        <v>13.53256187643049</v>
       </c>
       <c r="F5" t="n">
         <v>12300000</v>
@@ -692,16 +692,16 @@
         <v>44272</v>
       </c>
       <c r="B14" t="n">
-        <v>14.05289936065674</v>
+        <v>14.05290031433105</v>
       </c>
       <c r="C14" t="n">
-        <v>14.07188929407625</v>
+        <v>14.07189024903928</v>
       </c>
       <c r="D14" t="n">
-        <v>13.49458119180776</v>
+        <v>13.49458210759284</v>
       </c>
       <c r="E14" t="n">
-        <v>13.58763467271578</v>
+        <v>13.58763559481576</v>
       </c>
       <c r="F14" t="n">
         <v>4753000</v>
@@ -732,16 +732,16 @@
         <v>44274</v>
       </c>
       <c r="B16" t="n">
-        <v>13.54775238037109</v>
+        <v>13.54775428771973</v>
       </c>
       <c r="C16" t="n">
-        <v>14.03580565118024</v>
+        <v>14.03580762724047</v>
       </c>
       <c r="D16" t="n">
-        <v>13.46419523502917</v>
+        <v>13.46419713061404</v>
       </c>
       <c r="E16" t="n">
-        <v>13.95414740838706</v>
+        <v>13.95414937295086</v>
       </c>
       <c r="F16" t="n">
         <v>14098000</v>
@@ -752,16 +752,16 @@
         <v>44277</v>
       </c>
       <c r="B17" t="n">
-        <v>13.29328346252441</v>
+        <v>13.2932825088501</v>
       </c>
       <c r="C17" t="n">
-        <v>13.63511042556885</v>
+        <v>13.6351094473715</v>
       </c>
       <c r="D17" t="n">
-        <v>13.15655249620002</v>
+        <v>13.15655155233494</v>
       </c>
       <c r="E17" t="n">
-        <v>13.63511042556885</v>
+        <v>13.6351094473715</v>
       </c>
       <c r="F17" t="n">
         <v>5803000</v>
@@ -772,16 +772,16 @@
         <v>44278</v>
       </c>
       <c r="B18" t="n">
-        <v>13.44140815734863</v>
+        <v>13.44140911102295</v>
       </c>
       <c r="C18" t="n">
-        <v>13.44140815734863</v>
+        <v>13.44140911102295</v>
       </c>
       <c r="D18" t="n">
-        <v>13.01982095435623</v>
+        <v>13.01982187811874</v>
       </c>
       <c r="E18" t="n">
-        <v>13.29328287491709</v>
+        <v>13.29328381808184</v>
       </c>
       <c r="F18" t="n">
         <v>7916000</v>
@@ -812,16 +812,16 @@
         <v>44280</v>
       </c>
       <c r="B20" t="n">
-        <v>13.64840412139893</v>
+        <v>13.64840221405029</v>
       </c>
       <c r="C20" t="n">
-        <v>13.67309167041285</v>
+        <v>13.67308975961416</v>
       </c>
       <c r="D20" t="n">
-        <v>12.83941352376278</v>
+        <v>12.83941172946964</v>
       </c>
       <c r="E20" t="n">
-        <v>12.91347617080455</v>
+        <v>12.91347436616125</v>
       </c>
       <c r="F20" t="n">
         <v>6602000</v>
@@ -832,16 +832,16 @@
         <v>44281</v>
       </c>
       <c r="B21" t="n">
-        <v>13.8060245513916</v>
+        <v>13.80602359771729</v>
       </c>
       <c r="C21" t="n">
-        <v>14.1269626819656</v>
+        <v>14.12696170612194</v>
       </c>
       <c r="D21" t="n">
-        <v>13.48888513211062</v>
+        <v>13.48888420034324</v>
       </c>
       <c r="E21" t="n">
-        <v>13.54965455193487</v>
+        <v>13.54965361596974</v>
       </c>
       <c r="F21" t="n">
         <v>4396500</v>
@@ -912,16 +912,16 @@
         <v>44287</v>
       </c>
       <c r="B25" t="n">
-        <v>14.25419902801514</v>
+        <v>14.25419807434082</v>
       </c>
       <c r="C25" t="n">
-        <v>14.40232432733938</v>
+        <v>14.40232336375477</v>
       </c>
       <c r="D25" t="n">
-        <v>14.02631437007006</v>
+        <v>14.02631343164232</v>
       </c>
       <c r="E25" t="n">
-        <v>14.09088159926785</v>
+        <v>14.09088065652025</v>
       </c>
       <c r="F25" t="n">
         <v>9940000</v>
@@ -932,16 +932,16 @@
         <v>44291</v>
       </c>
       <c r="B26" t="n">
-        <v>14.71756267547607</v>
+        <v>14.71756362915039</v>
       </c>
       <c r="C26" t="n">
-        <v>14.88657769361247</v>
+        <v>14.88657865823869</v>
       </c>
       <c r="D26" t="n">
-        <v>14.2997741979616</v>
+        <v>14.29977512456389</v>
       </c>
       <c r="E26" t="n">
-        <v>14.2997741979616</v>
+        <v>14.29977512456389</v>
       </c>
       <c r="F26" t="n">
         <v>6073500</v>
@@ -952,16 +952,16 @@
         <v>44292</v>
       </c>
       <c r="B27" t="n">
-        <v>14.58653163909912</v>
+        <v>14.58652973175049</v>
       </c>
       <c r="C27" t="n">
-        <v>14.72136280773917</v>
+        <v>14.72136088275989</v>
       </c>
       <c r="D27" t="n">
-        <v>14.52766111829865</v>
+        <v>14.52765921864798</v>
       </c>
       <c r="E27" t="n">
-        <v>14.71756500173048</v>
+        <v>14.7175630772478</v>
       </c>
       <c r="F27" t="n">
         <v>5821500</v>
@@ -972,16 +972,16 @@
         <v>44293</v>
       </c>
       <c r="B28" t="n">
-        <v>14.49347686767578</v>
+        <v>14.4934778213501</v>
       </c>
       <c r="C28" t="n">
-        <v>14.78023202327058</v>
+        <v>14.78023299581345</v>
       </c>
       <c r="D28" t="n">
-        <v>13.92756307336586</v>
+        <v>13.92756398980291</v>
       </c>
       <c r="E28" t="n">
-        <v>14.45359719150692</v>
+        <v>14.45359814255714</v>
       </c>
       <c r="F28" t="n">
         <v>10992000</v>
@@ -992,16 +992,16 @@
         <v>44294</v>
       </c>
       <c r="B29" t="n">
-        <v>14.70237159729004</v>
+        <v>14.70237064361572</v>
       </c>
       <c r="C29" t="n">
-        <v>14.74035237068301</v>
+        <v>14.74035141454506</v>
       </c>
       <c r="D29" t="n">
-        <v>14.26559225050429</v>
+        <v>14.26559132516181</v>
       </c>
       <c r="E29" t="n">
-        <v>14.43270747232676</v>
+        <v>14.4327065361443</v>
       </c>
       <c r="F29" t="n">
         <v>6395000</v>
@@ -1012,16 +1012,16 @@
         <v>44295</v>
       </c>
       <c r="B30" t="n">
-        <v>14.71756267547607</v>
+        <v>14.71756362915039</v>
       </c>
       <c r="C30" t="n">
-        <v>14.73655351358414</v>
+        <v>14.73655446848903</v>
       </c>
       <c r="D30" t="n">
-        <v>14.40801889636538</v>
+        <v>14.40801982998176</v>
       </c>
       <c r="E30" t="n">
-        <v>14.63210571505577</v>
+        <v>14.63210666319261</v>
       </c>
       <c r="F30" t="n">
         <v>7012500</v>
@@ -1032,16 +1032,16 @@
         <v>44298</v>
       </c>
       <c r="B31" t="n">
-        <v>14.69857215881348</v>
+        <v>14.69857311248779</v>
       </c>
       <c r="C31" t="n">
-        <v>14.8011210568803</v>
+        <v>14.8011220172082</v>
       </c>
       <c r="D31" t="n">
-        <v>14.52765913976815</v>
+        <v>14.52766008235327</v>
       </c>
       <c r="E31" t="n">
-        <v>14.69857215881348</v>
+        <v>14.69857311248779</v>
       </c>
       <c r="F31" t="n">
         <v>4711000</v>
@@ -1072,16 +1072,16 @@
         <v>44300</v>
       </c>
       <c r="B33" t="n">
-        <v>14.93785285949707</v>
+        <v>14.93785381317139</v>
       </c>
       <c r="C33" t="n">
-        <v>14.9454484709092</v>
+        <v>14.94544942506844</v>
       </c>
       <c r="D33" t="n">
-        <v>14.62261144203403</v>
+        <v>14.62261237558245</v>
       </c>
       <c r="E33" t="n">
-        <v>14.65109770142871</v>
+        <v>14.65109863679578</v>
       </c>
       <c r="F33" t="n">
         <v>5841000</v>
@@ -1092,16 +1092,16 @@
         <v>44301</v>
       </c>
       <c r="B34" t="n">
-        <v>15.1866283416748</v>
+        <v>15.18662643432617</v>
       </c>
       <c r="C34" t="n">
-        <v>15.20371846858745</v>
+        <v>15.2037165590924</v>
       </c>
       <c r="D34" t="n">
-        <v>14.84100264251348</v>
+        <v>14.84100077857334</v>
       </c>
       <c r="E34" t="n">
-        <v>14.84100264251348</v>
+        <v>14.84100077857334</v>
       </c>
       <c r="F34" t="n">
         <v>11554500</v>
@@ -1132,16 +1132,16 @@
         <v>44305</v>
       </c>
       <c r="B36" t="n">
-        <v>15.28727626800537</v>
+        <v>15.28727722167969</v>
       </c>
       <c r="C36" t="n">
-        <v>15.50756529752376</v>
+        <v>15.50756626494049</v>
       </c>
       <c r="D36" t="n">
-        <v>15.00431891696419</v>
+        <v>15.00431985298662</v>
       </c>
       <c r="E36" t="n">
-        <v>15.14484768829616</v>
+        <v>15.14484863308528</v>
       </c>
       <c r="F36" t="n">
         <v>5017000</v>
@@ -1152,16 +1152,16 @@
         <v>44306</v>
       </c>
       <c r="B37" t="n">
-        <v>15.47717952728271</v>
+        <v>15.4771785736084</v>
       </c>
       <c r="C37" t="n">
-        <v>15.65569088659348</v>
+        <v>15.65568992191963</v>
       </c>
       <c r="D37" t="n">
-        <v>15.06698752800291</v>
+        <v>15.06698659960384</v>
       </c>
       <c r="E37" t="n">
-        <v>15.35944030441754</v>
+        <v>15.35943935799809</v>
       </c>
       <c r="F37" t="n">
         <v>6029000</v>
@@ -1232,16 +1232,16 @@
         <v>44313</v>
       </c>
       <c r="B41" t="n">
-        <v>15.12775707244873</v>
+        <v>15.12775611877441</v>
       </c>
       <c r="C41" t="n">
-        <v>15.29677210768214</v>
+        <v>15.29677114335289</v>
       </c>
       <c r="D41" t="n">
-        <v>15.10117062083444</v>
+        <v>15.10116966883617</v>
       </c>
       <c r="E41" t="n">
-        <v>15.24929500760934</v>
+        <v>15.24929404627311</v>
       </c>
       <c r="F41" t="n">
         <v>4986500</v>
@@ -1252,16 +1252,16 @@
         <v>44314</v>
       </c>
       <c r="B42" t="n">
-        <v>15.18852615356445</v>
+        <v>15.18852519989014</v>
       </c>
       <c r="C42" t="n">
-        <v>15.35564228216909</v>
+        <v>15.35564131800169</v>
       </c>
       <c r="D42" t="n">
-        <v>15.04799647598031</v>
+        <v>15.04799553112973</v>
       </c>
       <c r="E42" t="n">
-        <v>15.14864647703371</v>
+        <v>15.14864552586341</v>
       </c>
       <c r="F42" t="n">
         <v>5371500</v>
@@ -1272,16 +1272,16 @@
         <v>44315</v>
       </c>
       <c r="B43" t="n">
-        <v>15.21646499633789</v>
+        <v>15.21646404266357</v>
       </c>
       <c r="C43" t="n">
-        <v>15.32323336252505</v>
+        <v>15.32323240215915</v>
       </c>
       <c r="D43" t="n">
-        <v>14.90950503441863</v>
+        <v>14.90950409998268</v>
       </c>
       <c r="E43" t="n">
-        <v>15.26222338706449</v>
+        <v>15.26222243052232</v>
       </c>
       <c r="F43" t="n">
         <v>5343000</v>
@@ -1312,16 +1312,16 @@
         <v>44319</v>
       </c>
       <c r="B45" t="n">
-        <v>15.53295803070068</v>
+        <v>15.532958984375</v>
       </c>
       <c r="C45" t="n">
-        <v>15.67023137590184</v>
+        <v>15.6702323380043</v>
       </c>
       <c r="D45" t="n">
-        <v>15.29463476087267</v>
+        <v>15.29463569991469</v>
       </c>
       <c r="E45" t="n">
-        <v>15.44334861216023</v>
+        <v>15.44334956033281</v>
       </c>
       <c r="F45" t="n">
         <v>8474000</v>
@@ -1332,16 +1332,16 @@
         <v>44320</v>
       </c>
       <c r="B46" t="n">
-        <v>15.72933578491211</v>
+        <v>15.72933769226074</v>
       </c>
       <c r="C46" t="n">
-        <v>15.74840208285252</v>
+        <v>15.74840399251314</v>
       </c>
       <c r="D46" t="n">
-        <v>15.35945760522207</v>
+        <v>15.35945946771906</v>
       </c>
       <c r="E46" t="n">
-        <v>15.63400611347231</v>
+        <v>15.63400800926121</v>
       </c>
       <c r="F46" t="n">
         <v>9407500</v>
@@ -1352,16 +1352,16 @@
         <v>44321</v>
       </c>
       <c r="B47" t="n">
-        <v>16.32228469848633</v>
+        <v>16.32228660583496</v>
       </c>
       <c r="C47" t="n">
-        <v>16.58730007183393</v>
+        <v>16.58730201015107</v>
       </c>
       <c r="D47" t="n">
-        <v>16.01532383109572</v>
+        <v>16.01532570257429</v>
       </c>
       <c r="E47" t="n">
-        <v>16.08396141636727</v>
+        <v>16.08396329586652</v>
       </c>
       <c r="F47" t="n">
         <v>17262500</v>
@@ -1372,16 +1372,16 @@
         <v>44322</v>
       </c>
       <c r="B48" t="n">
-        <v>16.61971473693848</v>
+        <v>16.61971282958984</v>
       </c>
       <c r="C48" t="n">
-        <v>16.64449947442742</v>
+        <v>16.64449756423438</v>
       </c>
       <c r="D48" t="n">
-        <v>16.16022705029641</v>
+        <v>16.16022519568053</v>
       </c>
       <c r="E48" t="n">
-        <v>16.31847408082518</v>
+        <v>16.31847220804819</v>
       </c>
       <c r="F48" t="n">
         <v>9404500</v>
@@ -1392,16 +1392,16 @@
         <v>44323</v>
       </c>
       <c r="B49" t="n">
-        <v>16.96290016174316</v>
+        <v>16.96289825439453</v>
       </c>
       <c r="C49" t="n">
-        <v>17.04488198227947</v>
+        <v>17.0448800657126</v>
       </c>
       <c r="D49" t="n">
-        <v>16.4290546491212</v>
+        <v>16.42905280179942</v>
       </c>
       <c r="E49" t="n">
-        <v>16.663565057737</v>
+        <v>16.66356318404632</v>
       </c>
       <c r="F49" t="n">
         <v>8422500</v>
@@ -1412,16 +1412,16 @@
         <v>44326</v>
       </c>
       <c r="B50" t="n">
-        <v>16.81418609619141</v>
+        <v>16.81418418884277</v>
       </c>
       <c r="C50" t="n">
-        <v>17.0162841548014</v>
+        <v>17.01628222452739</v>
       </c>
       <c r="D50" t="n">
-        <v>16.55298359675715</v>
+        <v>16.55298171903851</v>
       </c>
       <c r="E50" t="n">
-        <v>16.97052576072697</v>
+        <v>16.97052383564365</v>
       </c>
       <c r="F50" t="n">
         <v>7669500</v>
@@ -1432,16 +1432,16 @@
         <v>44327</v>
       </c>
       <c r="B51" t="n">
-        <v>16.58729934692383</v>
+        <v>16.5872974395752</v>
       </c>
       <c r="C51" t="n">
-        <v>16.78367894467991</v>
+        <v>16.78367701474988</v>
       </c>
       <c r="D51" t="n">
-        <v>16.4919696745899</v>
+        <v>16.49196777820309</v>
       </c>
       <c r="E51" t="n">
-        <v>16.6254319431623</v>
+        <v>16.62543003142886</v>
       </c>
       <c r="F51" t="n">
         <v>6191000</v>
@@ -1452,16 +1452,16 @@
         <v>44328</v>
       </c>
       <c r="B52" t="n">
-        <v>16.12590980529785</v>
+        <v>16.12590789794922</v>
       </c>
       <c r="C52" t="n">
-        <v>16.57776989836218</v>
+        <v>16.57776793756821</v>
       </c>
       <c r="D52" t="n">
-        <v>16.04201880215192</v>
+        <v>16.04201690472579</v>
       </c>
       <c r="E52" t="n">
-        <v>16.49006781665641</v>
+        <v>16.49006586623571</v>
       </c>
       <c r="F52" t="n">
         <v>6728500</v>
@@ -1492,16 +1492,16 @@
         <v>44330</v>
       </c>
       <c r="B54" t="n">
-        <v>16.52628898620605</v>
+        <v>16.52629089355469</v>
       </c>
       <c r="C54" t="n">
-        <v>16.66356232925931</v>
+        <v>16.66356425245107</v>
       </c>
       <c r="D54" t="n">
-        <v>16.13734451407442</v>
+        <v>16.13734637653381</v>
       </c>
       <c r="E54" t="n">
-        <v>16.54726082268666</v>
+        <v>16.54726273245572</v>
       </c>
       <c r="F54" t="n">
         <v>5923000</v>
@@ -1512,16 +1512,16 @@
         <v>44333</v>
       </c>
       <c r="B55" t="n">
-        <v>16.34706878662109</v>
+        <v>16.34707069396973</v>
       </c>
       <c r="C55" t="n">
-        <v>16.52819314458002</v>
+        <v>16.52819507306194</v>
       </c>
       <c r="D55" t="n">
-        <v>16.06107980023078</v>
+        <v>16.06108167421069</v>
       </c>
       <c r="E55" t="n">
-        <v>16.50531395293831</v>
+        <v>16.50531587875072</v>
       </c>
       <c r="F55" t="n">
         <v>4728000</v>
@@ -1552,16 +1552,16 @@
         <v>44335</v>
       </c>
       <c r="B57" t="n">
-        <v>15.82847881317139</v>
+        <v>15.82847690582275</v>
       </c>
       <c r="C57" t="n">
-        <v>16.36804269641236</v>
+        <v>16.3680407240457</v>
       </c>
       <c r="D57" t="n">
-        <v>15.67595206173143</v>
+        <v>15.67595017276244</v>
       </c>
       <c r="E57" t="n">
-        <v>15.98481846065799</v>
+        <v>15.98481653447027</v>
       </c>
       <c r="F57" t="n">
         <v>6358000</v>
@@ -1572,16 +1572,16 @@
         <v>44336</v>
       </c>
       <c r="B58" t="n">
-        <v>16.03248596191406</v>
+        <v>16.03248405456543</v>
       </c>
       <c r="C58" t="n">
-        <v>16.03248596191406</v>
+        <v>16.03248405456543</v>
       </c>
       <c r="D58" t="n">
-        <v>15.69692561740377</v>
+        <v>15.69692374997599</v>
       </c>
       <c r="E58" t="n">
-        <v>15.90283657256179</v>
+        <v>15.90283468063725</v>
       </c>
       <c r="F58" t="n">
         <v>7278000</v>
@@ -1592,16 +1592,16 @@
         <v>44337</v>
       </c>
       <c r="B59" t="n">
-        <v>16.43477249145508</v>
+        <v>16.43477439880371</v>
       </c>
       <c r="C59" t="n">
-        <v>16.62543183488117</v>
+        <v>16.6254337643569</v>
       </c>
       <c r="D59" t="n">
-        <v>15.75984081583289</v>
+        <v>15.75984264485187</v>
       </c>
       <c r="E59" t="n">
-        <v>16.03438932487009</v>
+        <v>16.03439118575198</v>
       </c>
       <c r="F59" t="n">
         <v>10145000</v>
@@ -1632,16 +1632,16 @@
         <v>44341</v>
       </c>
       <c r="B61" t="n">
-        <v>16.88472747802734</v>
+        <v>16.88472938537598</v>
       </c>
       <c r="C61" t="n">
-        <v>17.06394632104241</v>
+        <v>17.06394824863613</v>
       </c>
       <c r="D61" t="n">
-        <v>16.77986465398696</v>
+        <v>16.77986654948997</v>
       </c>
       <c r="E61" t="n">
-        <v>17.0162823928035</v>
+        <v>17.01628431501296</v>
       </c>
       <c r="F61" t="n">
         <v>5307000</v>
@@ -1652,16 +1652,16 @@
         <v>44342</v>
       </c>
       <c r="B62" t="n">
-        <v>16.94192695617676</v>
+        <v>16.94192504882812</v>
       </c>
       <c r="C62" t="n">
-        <v>17.11161449219801</v>
+        <v>17.11161256574568</v>
       </c>
       <c r="D62" t="n">
-        <v>16.65975260630318</v>
+        <v>16.65975073072218</v>
       </c>
       <c r="E62" t="n">
-        <v>17.02391059716581</v>
+        <v>17.02390868058733</v>
       </c>
       <c r="F62" t="n">
         <v>5462000</v>
@@ -1672,16 +1672,16 @@
         <v>44343</v>
       </c>
       <c r="B63" t="n">
-        <v>16.94955253601074</v>
+        <v>16.94955444335938</v>
       </c>
       <c r="C63" t="n">
-        <v>17.26223183953111</v>
+        <v>17.26223378206583</v>
       </c>
       <c r="D63" t="n">
-        <v>16.70550899973091</v>
+        <v>16.7055108796171</v>
       </c>
       <c r="E63" t="n">
-        <v>16.94955253601074</v>
+        <v>16.94955444335938</v>
       </c>
       <c r="F63" t="n">
         <v>5669000</v>
@@ -1692,16 +1692,16 @@
         <v>44344</v>
       </c>
       <c r="B64" t="n">
-        <v>16.98577690124512</v>
+        <v>16.98577880859375</v>
       </c>
       <c r="C64" t="n">
-        <v>17.14974233685488</v>
+        <v>17.14974426261534</v>
       </c>
       <c r="D64" t="n">
-        <v>16.56442007870208</v>
+        <v>16.56442193873616</v>
       </c>
       <c r="E64" t="n">
-        <v>16.91141906621777</v>
+        <v>16.91142096521669</v>
       </c>
       <c r="F64" t="n">
         <v>4590500</v>
@@ -1732,16 +1732,16 @@
         <v>44348</v>
       </c>
       <c r="B66" t="n">
-        <v>16.96861457824707</v>
+        <v>16.9686164855957</v>
       </c>
       <c r="C66" t="n">
-        <v>17.4109431969055</v>
+        <v>17.41094515397386</v>
       </c>
       <c r="D66" t="n">
-        <v>16.8256209926954</v>
+        <v>16.82562288397091</v>
       </c>
       <c r="E66" t="n">
-        <v>17.17834020076747</v>
+        <v>17.17834213169021</v>
       </c>
       <c r="F66" t="n">
         <v>13722000</v>
@@ -1772,16 +1772,16 @@
         <v>44351</v>
       </c>
       <c r="B68" t="n">
-        <v>16.77223587036133</v>
+        <v>16.77223968505859</v>
       </c>
       <c r="C68" t="n">
-        <v>16.81608689471135</v>
+        <v>16.81609071938215</v>
       </c>
       <c r="D68" t="n">
-        <v>16.40617063922488</v>
+        <v>16.40617437066384</v>
       </c>
       <c r="E68" t="n">
-        <v>16.72266459379896</v>
+        <v>16.72266839722167</v>
       </c>
       <c r="F68" t="n">
         <v>8097000</v>
@@ -1852,16 +1852,16 @@
         <v>44357</v>
       </c>
       <c r="B72" t="n">
-        <v>16.30321884155273</v>
+        <v>16.30321502685547</v>
       </c>
       <c r="C72" t="n">
-        <v>16.34707169398488</v>
+        <v>16.34706786902673</v>
       </c>
       <c r="D72" t="n">
-        <v>15.97719348463267</v>
+        <v>15.97718974622022</v>
       </c>
       <c r="E72" t="n">
-        <v>16.15641233581547</v>
+        <v>16.15640855546862</v>
       </c>
       <c r="F72" t="n">
         <v>4720000</v>
@@ -1892,16 +1892,16 @@
         <v>44361</v>
       </c>
       <c r="B74" t="n">
-        <v>16.01532173156738</v>
+        <v>16.01532554626465</v>
       </c>
       <c r="C74" t="n">
-        <v>16.19263501570841</v>
+        <v>16.19263887264001</v>
       </c>
       <c r="D74" t="n">
-        <v>15.85135630955313</v>
+        <v>15.8513600851954</v>
       </c>
       <c r="E74" t="n">
-        <v>16.16403557102893</v>
+        <v>16.16403942114841</v>
       </c>
       <c r="F74" t="n">
         <v>4317000</v>
@@ -1912,16 +1912,16 @@
         <v>44362</v>
       </c>
       <c r="B75" t="n">
-        <v>15.85898494720459</v>
+        <v>15.85898303985596</v>
       </c>
       <c r="C75" t="n">
-        <v>16.02676511323235</v>
+        <v>16.02676318570492</v>
       </c>
       <c r="D75" t="n">
-        <v>15.48720119095393</v>
+        <v>15.48719932831946</v>
       </c>
       <c r="E75" t="n">
-        <v>16.01532460600237</v>
+        <v>16.01532267985088</v>
       </c>
       <c r="F75" t="n">
         <v>8432500</v>
@@ -1932,16 +1932,16 @@
         <v>44363</v>
       </c>
       <c r="B76" t="n">
-        <v>15.89902305603027</v>
+        <v>15.89902114868164</v>
       </c>
       <c r="C76" t="n">
-        <v>16.11446715307724</v>
+        <v>16.11446521988256</v>
       </c>
       <c r="D76" t="n">
-        <v>15.66260712011776</v>
+        <v>15.6626052411311</v>
       </c>
       <c r="E76" t="n">
-        <v>15.7026452588224</v>
+        <v>15.70264337503251</v>
       </c>
       <c r="F76" t="n">
         <v>10606500</v>
@@ -1952,16 +1952,16 @@
         <v>44364</v>
       </c>
       <c r="B77" t="n">
-        <v>15.97719383239746</v>
+        <v>15.97719192504883</v>
       </c>
       <c r="C77" t="n">
-        <v>16.00769882125508</v>
+        <v>16.00769691026478</v>
       </c>
       <c r="D77" t="n">
-        <v>15.69120478891841</v>
+        <v>15.691202915711</v>
       </c>
       <c r="E77" t="n">
-        <v>15.8971175547978</v>
+        <v>15.89711565700863</v>
       </c>
       <c r="F77" t="n">
         <v>7246000</v>
@@ -1972,16 +1972,16 @@
         <v>44365</v>
       </c>
       <c r="B78" t="n">
-        <v>16.2078914642334</v>
+        <v>16.20789337158203</v>
       </c>
       <c r="C78" t="n">
-        <v>16.36423112436919</v>
+        <v>16.36423305011592</v>
       </c>
       <c r="D78" t="n">
-        <v>15.67976622640263</v>
+        <v>15.67976807160136</v>
       </c>
       <c r="E78" t="n">
-        <v>15.98863265031907</v>
+        <v>15.98863453186528</v>
       </c>
       <c r="F78" t="n">
         <v>12012000</v>
@@ -1992,16 +1992,16 @@
         <v>44368</v>
       </c>
       <c r="B79" t="n">
-        <v>16.48434448242188</v>
+        <v>16.48434257507324</v>
       </c>
       <c r="C79" t="n">
-        <v>16.59302020374093</v>
+        <v>16.59301828381779</v>
       </c>
       <c r="D79" t="n">
-        <v>16.00007212945171</v>
+        <v>16.00007027813662</v>
       </c>
       <c r="E79" t="n">
-        <v>16.20789042268334</v>
+        <v>16.20788854732228</v>
       </c>
       <c r="F79" t="n">
         <v>6798000</v>
@@ -2012,16 +2012,16 @@
         <v>44369</v>
       </c>
       <c r="B80" t="n">
-        <v>16.47290420532227</v>
+        <v>16.4729061126709</v>
       </c>
       <c r="C80" t="n">
-        <v>16.49578339803871</v>
+        <v>16.49578530803645</v>
       </c>
       <c r="D80" t="n">
-        <v>16.13162548984007</v>
+        <v>16.13162735767305</v>
       </c>
       <c r="E80" t="n">
-        <v>16.46718395257762</v>
+        <v>16.46718585926392</v>
       </c>
       <c r="F80" t="n">
         <v>6518000</v>
@@ -2052,16 +2052,16 @@
         <v>44371</v>
       </c>
       <c r="B82" t="n">
-        <v>16.64640617370605</v>
+        <v>16.64640426635742</v>
       </c>
       <c r="C82" t="n">
-        <v>16.72648245540622</v>
+        <v>16.72648053888243</v>
       </c>
       <c r="D82" t="n">
-        <v>16.39664417817516</v>
+        <v>16.39664229944431</v>
       </c>
       <c r="E82" t="n">
-        <v>16.46909284857351</v>
+        <v>16.46909096154148</v>
       </c>
       <c r="F82" t="n">
         <v>8527500</v>
@@ -2092,16 +2092,16 @@
         <v>44375</v>
       </c>
       <c r="B84" t="n">
-        <v>16.3737621307373</v>
+        <v>16.37376403808594</v>
       </c>
       <c r="C84" t="n">
-        <v>16.37948056539015</v>
+        <v>16.37948247340491</v>
       </c>
       <c r="D84" t="n">
-        <v>15.9390592744375</v>
+        <v>15.93906113114842</v>
       </c>
       <c r="E84" t="n">
-        <v>16.2250482827814</v>
+        <v>16.22505017280664</v>
       </c>
       <c r="F84" t="n">
         <v>6202500</v>
@@ -2152,16 +2152,16 @@
         <v>44378</v>
       </c>
       <c r="B87" t="n">
-        <v>16.35851097106934</v>
+        <v>16.3585090637207</v>
       </c>
       <c r="C87" t="n">
-        <v>16.66356450050222</v>
+        <v>16.66356255758535</v>
       </c>
       <c r="D87" t="n">
-        <v>16.14878712414984</v>
+        <v>16.14878524125432</v>
       </c>
       <c r="E87" t="n">
-        <v>16.66356450050222</v>
+        <v>16.66356255758535</v>
       </c>
       <c r="F87" t="n">
         <v>8503000</v>
@@ -2192,16 +2192,16 @@
         <v>44382</v>
       </c>
       <c r="B89" t="n">
-        <v>16.41570854187012</v>
+        <v>16.41570663452148</v>
       </c>
       <c r="C89" t="n">
-        <v>16.54726347128895</v>
+        <v>16.54726154865489</v>
       </c>
       <c r="D89" t="n">
-        <v>16.25174308313778</v>
+        <v>16.25174119484036</v>
       </c>
       <c r="E89" t="n">
-        <v>16.40808274888606</v>
+        <v>16.40808084242347</v>
       </c>
       <c r="F89" t="n">
         <v>3871000</v>
@@ -2232,16 +2232,16 @@
         <v>44384</v>
       </c>
       <c r="B91" t="n">
-        <v>16.44430541992188</v>
+        <v>16.44430732727051</v>
       </c>
       <c r="C91" t="n">
-        <v>16.58348612054724</v>
+        <v>16.58348804403921</v>
       </c>
       <c r="D91" t="n">
-        <v>16.15069061682722</v>
+        <v>16.15069249011994</v>
       </c>
       <c r="E91" t="n">
-        <v>16.39664149383569</v>
+        <v>16.39664339565586</v>
       </c>
       <c r="F91" t="n">
         <v>12086500</v>
@@ -2252,16 +2252,16 @@
         <v>44385</v>
       </c>
       <c r="B92" t="n">
-        <v>16.43477249145508</v>
+        <v>16.43477439880371</v>
       </c>
       <c r="C92" t="n">
-        <v>16.79893041915436</v>
+        <v>16.79893236876558</v>
       </c>
       <c r="D92" t="n">
-        <v>16.24411496629124</v>
+        <v>16.24411685151298</v>
       </c>
       <c r="E92" t="n">
-        <v>16.26317944602405</v>
+        <v>16.26318133345833</v>
       </c>
       <c r="F92" t="n">
         <v>7435000</v>
@@ -2272,16 +2272,16 @@
         <v>44389</v>
       </c>
       <c r="B93" t="n">
-        <v>16.50150108337402</v>
+        <v>16.50150299072266</v>
       </c>
       <c r="C93" t="n">
-        <v>16.60255099813928</v>
+        <v>16.60255291716791</v>
       </c>
       <c r="D93" t="n">
-        <v>16.27461834177422</v>
+        <v>16.2746202228983</v>
       </c>
       <c r="E93" t="n">
-        <v>16.43095796968715</v>
+        <v>16.43095986888196</v>
       </c>
       <c r="F93" t="n">
         <v>4327500</v>
@@ -2292,16 +2292,16 @@
         <v>44390</v>
       </c>
       <c r="B94" t="n">
-        <v>16.78749084472656</v>
+        <v>16.7874927520752</v>
       </c>
       <c r="C94" t="n">
-        <v>16.91141813862505</v>
+        <v>16.91142006005396</v>
       </c>
       <c r="D94" t="n">
-        <v>16.43095872774974</v>
+        <v>16.43096059459017</v>
       </c>
       <c r="E94" t="n">
-        <v>16.45383792048305</v>
+        <v>16.45383978992295</v>
       </c>
       <c r="F94" t="n">
         <v>6446000</v>
@@ -2312,16 +2312,16 @@
         <v>44391</v>
       </c>
       <c r="B95" t="n">
-        <v>16.7226676940918</v>
+        <v>16.72266578674316</v>
       </c>
       <c r="C95" t="n">
-        <v>17.08873299309478</v>
+        <v>17.08873104399359</v>
       </c>
       <c r="D95" t="n">
-        <v>16.67309640833917</v>
+        <v>16.67309450664453</v>
       </c>
       <c r="E95" t="n">
-        <v>16.9304859864696</v>
+        <v>16.9304840554177</v>
       </c>
       <c r="F95" t="n">
         <v>5548000</v>
@@ -2332,16 +2332,16 @@
         <v>44392</v>
       </c>
       <c r="B96" t="n">
-        <v>16.45002555847168</v>
+        <v>16.45002746582031</v>
       </c>
       <c r="C96" t="n">
-        <v>16.86375476157448</v>
+        <v>16.86375671689422</v>
       </c>
       <c r="D96" t="n">
-        <v>16.44049240966831</v>
+        <v>16.44049431591159</v>
       </c>
       <c r="E96" t="n">
-        <v>16.72266670485169</v>
+        <v>16.72266864381253</v>
       </c>
       <c r="F96" t="n">
         <v>3746000</v>
@@ -2352,16 +2352,16 @@
         <v>44393</v>
       </c>
       <c r="B97" t="n">
-        <v>16.67119026184082</v>
+        <v>16.67119216918945</v>
       </c>
       <c r="C97" t="n">
-        <v>16.86947357936254</v>
+        <v>16.86947550939675</v>
       </c>
       <c r="D97" t="n">
-        <v>16.52247641000283</v>
+        <v>16.52247830033713</v>
       </c>
       <c r="E97" t="n">
-        <v>16.54154088978033</v>
+        <v>16.54154278229579</v>
       </c>
       <c r="F97" t="n">
         <v>7965000</v>
@@ -2372,16 +2372,16 @@
         <v>44396</v>
       </c>
       <c r="B98" t="n">
-        <v>16.65402984619141</v>
+        <v>16.65402793884277</v>
       </c>
       <c r="C98" t="n">
-        <v>16.79702526617702</v>
+        <v>16.79702334245145</v>
       </c>
       <c r="D98" t="n">
-        <v>16.40426788246265</v>
+        <v>16.4042660037187</v>
       </c>
       <c r="E98" t="n">
-        <v>16.58539408105208</v>
+        <v>16.58539218156415</v>
       </c>
       <c r="F98" t="n">
         <v>7763500</v>
@@ -2392,16 +2392,16 @@
         <v>44397</v>
       </c>
       <c r="B99" t="n">
-        <v>16.51103591918945</v>
+        <v>16.51103782653809</v>
       </c>
       <c r="C99" t="n">
-        <v>16.71694684707543</v>
+        <v>16.71694877821082</v>
       </c>
       <c r="D99" t="n">
-        <v>16.45955909634909</v>
+        <v>16.45956099775114</v>
       </c>
       <c r="E99" t="n">
-        <v>16.6540295180957</v>
+        <v>16.6540314419629</v>
       </c>
       <c r="F99" t="n">
         <v>3835500</v>
@@ -2432,16 +2432,16 @@
         <v>44399</v>
       </c>
       <c r="B101" t="n">
-        <v>16.64449501037598</v>
+        <v>16.64449691772461</v>
       </c>
       <c r="C101" t="n">
-        <v>16.68072024642313</v>
+        <v>16.68072215792294</v>
       </c>
       <c r="D101" t="n">
-        <v>16.44430435190125</v>
+        <v>16.44430623630937</v>
       </c>
       <c r="E101" t="n">
-        <v>16.58729793913493</v>
+        <v>16.58729983992916</v>
       </c>
       <c r="F101" t="n">
         <v>2829500</v>
@@ -2492,16 +2492,16 @@
         <v>44404</v>
       </c>
       <c r="B104" t="n">
-        <v>16.96861457824707</v>
+        <v>16.9686164855957</v>
       </c>
       <c r="C104" t="n">
-        <v>17.30036195137194</v>
+        <v>17.30036389601047</v>
       </c>
       <c r="D104" t="n">
-        <v>16.87328673338735</v>
+        <v>16.8732886300207</v>
       </c>
       <c r="E104" t="n">
-        <v>17.14402050381685</v>
+        <v>17.1440224308819</v>
       </c>
       <c r="F104" t="n">
         <v>6666500</v>
@@ -2512,16 +2512,16 @@
         <v>44405</v>
       </c>
       <c r="B105" t="n">
-        <v>16.793212890625</v>
+        <v>16.79321098327637</v>
       </c>
       <c r="C105" t="n">
-        <v>17.38044259996134</v>
+        <v>17.38044062591602</v>
       </c>
       <c r="D105" t="n">
-        <v>16.42333646812846</v>
+        <v>16.42333460278985</v>
       </c>
       <c r="E105" t="n">
-        <v>17.34993760917749</v>
+        <v>17.34993563859687</v>
       </c>
       <c r="F105" t="n">
         <v>14614500</v>
@@ -2552,16 +2552,16 @@
         <v>44407</v>
       </c>
       <c r="B107" t="n">
-        <v>16.52628898620605</v>
+        <v>16.52629089355469</v>
       </c>
       <c r="C107" t="n">
-        <v>16.73219990991705</v>
+        <v>16.73220184103048</v>
       </c>
       <c r="D107" t="n">
-        <v>16.30893755658766</v>
+        <v>16.30893943885111</v>
       </c>
       <c r="E107" t="n">
-        <v>16.62543155217983</v>
+        <v>16.6254334709708</v>
       </c>
       <c r="F107" t="n">
         <v>16469000</v>
@@ -2572,16 +2572,16 @@
         <v>44410</v>
       </c>
       <c r="B108" t="n">
-        <v>16.5224781036377</v>
+        <v>16.52247619628906</v>
       </c>
       <c r="C108" t="n">
-        <v>16.83897031953316</v>
+        <v>16.83896837564879</v>
       </c>
       <c r="D108" t="n">
-        <v>16.36232372925435</v>
+        <v>16.36232184039388</v>
       </c>
       <c r="E108" t="n">
-        <v>16.6826306597586</v>
+        <v>16.68262873392202</v>
       </c>
       <c r="F108" t="n">
         <v>8100500</v>
@@ -2592,16 +2592,16 @@
         <v>44411</v>
       </c>
       <c r="B109" t="n">
-        <v>16.53010368347168</v>
+        <v>16.53010559082031</v>
       </c>
       <c r="C109" t="n">
-        <v>16.68072308765598</v>
+        <v>16.68072501238404</v>
       </c>
       <c r="D109" t="n">
-        <v>16.26127540276083</v>
+        <v>16.26127727909034</v>
       </c>
       <c r="E109" t="n">
-        <v>16.68072308765598</v>
+        <v>16.68072501238404</v>
       </c>
       <c r="F109" t="n">
         <v>5450500</v>
@@ -2632,16 +2632,16 @@
         <v>44413</v>
       </c>
       <c r="B111" t="n">
-        <v>16.58729934692383</v>
+        <v>16.5872974395752</v>
       </c>
       <c r="C111" t="n">
-        <v>16.93811123196384</v>
+        <v>16.93810928427588</v>
       </c>
       <c r="D111" t="n">
-        <v>16.47481073358749</v>
+        <v>16.47480883917376</v>
       </c>
       <c r="E111" t="n">
-        <v>16.59301960001205</v>
+        <v>16.59301769200566</v>
       </c>
       <c r="F111" t="n">
         <v>13427000</v>
@@ -2652,16 +2652,16 @@
         <v>44414</v>
       </c>
       <c r="B112" t="n">
-        <v>16.73982620239258</v>
+        <v>16.73983001708984</v>
       </c>
       <c r="C112" t="n">
-        <v>16.78367905199969</v>
+        <v>16.78368287669021</v>
       </c>
       <c r="D112" t="n">
-        <v>16.37566826999301</v>
+        <v>16.37567200170541</v>
       </c>
       <c r="E112" t="n">
-        <v>16.63115048433273</v>
+        <v>16.63115427426481</v>
       </c>
       <c r="F112" t="n">
         <v>15424500</v>
@@ -2712,16 +2712,16 @@
         <v>44419</v>
       </c>
       <c r="B115" t="n">
-        <v>17.20884895324707</v>
+        <v>17.2088451385498</v>
       </c>
       <c r="C115" t="n">
-        <v>17.57872718168084</v>
+        <v>17.57872328499242</v>
       </c>
       <c r="D115" t="n">
-        <v>17.19741026393275</v>
+        <v>17.1974064517711</v>
       </c>
       <c r="E115" t="n">
-        <v>17.57872718168084</v>
+        <v>17.57872328499242</v>
       </c>
       <c r="F115" t="n">
         <v>6265000</v>
@@ -2752,16 +2752,16 @@
         <v>44421</v>
       </c>
       <c r="B117" t="n">
-        <v>16.91142082214355</v>
+        <v>16.91141891479492</v>
       </c>
       <c r="C117" t="n">
-        <v>17.27367324935177</v>
+        <v>17.27367130114663</v>
       </c>
       <c r="D117" t="n">
-        <v>16.53010391318421</v>
+        <v>16.53010204884227</v>
       </c>
       <c r="E117" t="n">
-        <v>16.82562429034489</v>
+        <v>16.82562239267279</v>
       </c>
       <c r="F117" t="n">
         <v>5547600</v>
@@ -2772,16 +2772,16 @@
         <v>44424</v>
       </c>
       <c r="B118" t="n">
-        <v>16.44430541992188</v>
+        <v>16.44430732727051</v>
       </c>
       <c r="C118" t="n">
-        <v>17.04487925261408</v>
+        <v>17.04488122962231</v>
       </c>
       <c r="D118" t="n">
-        <v>16.27271237679204</v>
+        <v>16.27271426423787</v>
       </c>
       <c r="E118" t="n">
-        <v>16.86375487887679</v>
+        <v>16.86375683487669</v>
       </c>
       <c r="F118" t="n">
         <v>7814500</v>
@@ -2812,16 +2812,16 @@
         <v>44426</v>
       </c>
       <c r="B120" t="n">
-        <v>15.88186264038086</v>
+        <v>15.88186454772949</v>
       </c>
       <c r="C120" t="n">
-        <v>16.30131210662337</v>
+        <v>16.30131406434622</v>
       </c>
       <c r="D120" t="n">
-        <v>15.64353936928479</v>
+        <v>15.64354124801175</v>
       </c>
       <c r="E120" t="n">
-        <v>16.16784983839123</v>
+        <v>16.16785178008579</v>
       </c>
       <c r="F120" t="n">
         <v>10736900</v>
@@ -2852,16 +2852,16 @@
         <v>44428</v>
       </c>
       <c r="B122" t="n">
-        <v>16.94955253601074</v>
+        <v>16.94955444335938</v>
       </c>
       <c r="C122" t="n">
-        <v>17.41666595234703</v>
+        <v>17.41666791226037</v>
       </c>
       <c r="D122" t="n">
-        <v>16.37757629334467</v>
+        <v>16.3775781363283</v>
       </c>
       <c r="E122" t="n">
-        <v>16.53963619846235</v>
+        <v>16.53963805968273</v>
       </c>
       <c r="F122" t="n">
         <v>9513400</v>
@@ -2872,16 +2872,16 @@
         <v>44431</v>
       </c>
       <c r="B123" t="n">
-        <v>16.69216537475586</v>
+        <v>16.69216346740723</v>
       </c>
       <c r="C123" t="n">
-        <v>17.16881200972343</v>
+        <v>17.16881004791025</v>
       </c>
       <c r="D123" t="n">
-        <v>16.52057229524551</v>
+        <v>16.52057040750415</v>
       </c>
       <c r="E123" t="n">
-        <v>16.97815262843136</v>
+        <v>16.97815068840407</v>
       </c>
       <c r="F123" t="n">
         <v>5050600</v>
@@ -2892,16 +2892,16 @@
         <v>44432</v>
       </c>
       <c r="B124" t="n">
-        <v>16.91142082214355</v>
+        <v>16.91141891479492</v>
       </c>
       <c r="C124" t="n">
-        <v>17.05441443572051</v>
+        <v>17.05441251224439</v>
       </c>
       <c r="D124" t="n">
-        <v>16.66356437675437</v>
+        <v>16.66356249736014</v>
       </c>
       <c r="E124" t="n">
-        <v>16.78749350858018</v>
+        <v>16.78749161520865</v>
       </c>
       <c r="F124" t="n">
         <v>4198100</v>
@@ -2912,16 +2912,16 @@
         <v>44433</v>
       </c>
       <c r="B125" t="n">
-        <v>17.01628494262695</v>
+        <v>17.01628303527832</v>
       </c>
       <c r="C125" t="n">
-        <v>17.19741116994805</v>
+        <v>17.19740924229705</v>
       </c>
       <c r="D125" t="n">
-        <v>16.78749477992469</v>
+        <v>16.78749289822105</v>
       </c>
       <c r="E125" t="n">
-        <v>17.0258180933557</v>
+        <v>17.0258161849385</v>
       </c>
       <c r="F125" t="n">
         <v>4269900</v>
@@ -2952,16 +2952,16 @@
         <v>44435</v>
       </c>
       <c r="B127" t="n">
-        <v>16.58729934692383</v>
+        <v>16.5872974395752</v>
       </c>
       <c r="C127" t="n">
-        <v>16.72076161549623</v>
+        <v>16.72075969280097</v>
       </c>
       <c r="D127" t="n">
-        <v>16.39664182051824</v>
+        <v>16.39663993509303</v>
       </c>
       <c r="E127" t="n">
-        <v>16.55870171800724</v>
+        <v>16.558699813947</v>
       </c>
       <c r="F127" t="n">
         <v>5662600</v>
@@ -2972,16 +2972,16 @@
         <v>44438</v>
       </c>
       <c r="B128" t="n">
-        <v>16.35851097106934</v>
+        <v>16.3585090637207</v>
       </c>
       <c r="C128" t="n">
-        <v>16.79702678332595</v>
+        <v>16.79702482484782</v>
       </c>
       <c r="D128" t="n">
-        <v>16.16785160604255</v>
+        <v>16.16784972092418</v>
       </c>
       <c r="E128" t="n">
-        <v>16.4729069537379</v>
+        <v>16.47290503305107</v>
       </c>
       <c r="F128" t="n">
         <v>16747200</v>
@@ -3032,16 +3032,16 @@
         <v>44441</v>
       </c>
       <c r="B131" t="n">
-        <v>16.72076416015625</v>
+        <v>16.72076225280762</v>
       </c>
       <c r="C131" t="n">
-        <v>17.03535085395019</v>
+        <v>17.03534891071645</v>
       </c>
       <c r="D131" t="n">
-        <v>16.10112210481625</v>
+        <v>16.10112026815059</v>
       </c>
       <c r="E131" t="n">
-        <v>16.1678523401267</v>
+        <v>16.16785049584908</v>
       </c>
       <c r="F131" t="n">
         <v>17566400</v>
@@ -3112,16 +3112,16 @@
         <v>44448</v>
       </c>
       <c r="B135" t="n">
-        <v>17.34993553161621</v>
+        <v>17.34993362426758</v>
       </c>
       <c r="C135" t="n">
-        <v>17.44526338911795</v>
+        <v>17.44526147128954</v>
       </c>
       <c r="D135" t="n">
-        <v>16.92095289980908</v>
+        <v>16.92095103962024</v>
       </c>
       <c r="E135" t="n">
-        <v>17.07347965372665</v>
+        <v>17.07347777676993</v>
       </c>
       <c r="F135" t="n">
         <v>12544000</v>
@@ -3132,16 +3132,16 @@
         <v>44449</v>
       </c>
       <c r="B136" t="n">
-        <v>17.33086776733398</v>
+        <v>17.33086967468262</v>
       </c>
       <c r="C136" t="n">
-        <v>17.6073218035846</v>
+        <v>17.60732374135838</v>
       </c>
       <c r="D136" t="n">
-        <v>17.01628113669726</v>
+        <v>17.01628300942406</v>
       </c>
       <c r="E136" t="n">
-        <v>17.33086776733398</v>
+        <v>17.33086967468262</v>
       </c>
       <c r="F136" t="n">
         <v>19125200</v>
@@ -3172,16 +3172,16 @@
         <v>44453</v>
       </c>
       <c r="B138" t="n">
-        <v>17.47386360168457</v>
+        <v>17.4738597869873</v>
       </c>
       <c r="C138" t="n">
-        <v>18.1507026927803</v>
+        <v>18.15069873032314</v>
       </c>
       <c r="D138" t="n">
-        <v>17.3976002213898</v>
+        <v>17.39759642334149</v>
       </c>
       <c r="E138" t="n">
-        <v>17.82658287196191</v>
+        <v>17.82657898026294</v>
       </c>
       <c r="F138" t="n">
         <v>6594500</v>
@@ -3192,16 +3192,16 @@
         <v>44454</v>
       </c>
       <c r="B139" t="n">
-        <v>17.72171783447266</v>
+        <v>17.72171974182129</v>
       </c>
       <c r="C139" t="n">
-        <v>17.82658065116278</v>
+        <v>17.82658256979756</v>
       </c>
       <c r="D139" t="n">
-        <v>17.27367075834045</v>
+        <v>17.27367261746679</v>
       </c>
       <c r="E139" t="n">
-        <v>17.46432827619446</v>
+        <v>17.46433015584083</v>
       </c>
       <c r="F139" t="n">
         <v>8756500</v>
@@ -3212,16 +3212,16 @@
         <v>44455</v>
       </c>
       <c r="B140" t="n">
-        <v>18.26509666442871</v>
+        <v>18.26509857177734</v>
       </c>
       <c r="C140" t="n">
-        <v>18.33182689421092</v>
+        <v>18.33182880852791</v>
       </c>
       <c r="D140" t="n">
-        <v>17.72171985818801</v>
+        <v>17.72172170879404</v>
       </c>
       <c r="E140" t="n">
-        <v>17.72171985818801</v>
+        <v>17.72172170879404</v>
       </c>
       <c r="F140" t="n">
         <v>17281800</v>
@@ -3232,16 +3232,16 @@
         <v>44456</v>
       </c>
       <c r="B141" t="n">
-        <v>18.11256980895996</v>
+        <v>18.11256790161133</v>
       </c>
       <c r="C141" t="n">
-        <v>18.44622277435644</v>
+        <v>18.4462208318724</v>
       </c>
       <c r="D141" t="n">
-        <v>18.11256980895996</v>
+        <v>18.11256790161133</v>
       </c>
       <c r="E141" t="n">
-        <v>18.28416286649314</v>
+        <v>18.28416094107486</v>
       </c>
       <c r="F141" t="n">
         <v>23104900</v>
@@ -3272,16 +3272,16 @@
         <v>44460</v>
       </c>
       <c r="B143" t="n">
-        <v>18.57968330383301</v>
+        <v>18.57968139648438</v>
       </c>
       <c r="C143" t="n">
-        <v>18.7417432123123</v>
+        <v>18.74174128832697</v>
       </c>
       <c r="D143" t="n">
-        <v>17.82658265967325</v>
+        <v>17.82658082963624</v>
       </c>
       <c r="E143" t="n">
-        <v>18.06490594753913</v>
+        <v>18.06490409303639</v>
       </c>
       <c r="F143" t="n">
         <v>17756900</v>
@@ -3352,16 +3352,16 @@
         <v>44466</v>
       </c>
       <c r="B147" t="n">
-        <v>18.35089302062988</v>
+        <v>18.35089492797852</v>
       </c>
       <c r="C147" t="n">
-        <v>18.46528899793678</v>
+        <v>18.46529091717547</v>
       </c>
       <c r="D147" t="n">
-        <v>17.83611385014238</v>
+        <v>17.83611570398607</v>
       </c>
       <c r="E147" t="n">
-        <v>18.01724005660232</v>
+        <v>18.01724192927185</v>
       </c>
       <c r="F147" t="n">
         <v>7788100</v>
@@ -3432,16 +3432,16 @@
         <v>44470</v>
       </c>
       <c r="B151" t="n">
-        <v>18.45575523376465</v>
+        <v>18.45575332641602</v>
       </c>
       <c r="C151" t="n">
-        <v>18.56061623968673</v>
+        <v>18.56061432150102</v>
       </c>
       <c r="D151" t="n">
-        <v>18.00770630734936</v>
+        <v>18.00770444630528</v>
       </c>
       <c r="E151" t="n">
-        <v>18.19836565709148</v>
+        <v>18.19836377634331</v>
       </c>
       <c r="F151" t="n">
         <v>5841800</v>
@@ -3452,16 +3452,16 @@
         <v>44473</v>
       </c>
       <c r="B152" t="n">
-        <v>18.41762733459473</v>
+        <v>18.41762542724609</v>
       </c>
       <c r="C152" t="n">
-        <v>18.49389073029286</v>
+        <v>18.49388881504631</v>
       </c>
       <c r="D152" t="n">
-        <v>18.07444114482175</v>
+        <v>18.07443927301384</v>
       </c>
       <c r="E152" t="n">
-        <v>18.38902969762216</v>
+        <v>18.38902779323513</v>
       </c>
       <c r="F152" t="n">
         <v>9789400</v>
@@ -3472,16 +3472,16 @@
         <v>44474</v>
       </c>
       <c r="B153" t="n">
-        <v>18.32229423522949</v>
+        <v>18.32229232788086</v>
       </c>
       <c r="C153" t="n">
-        <v>18.49388729827244</v>
+        <v>18.49388537306099</v>
       </c>
       <c r="D153" t="n">
-        <v>18.04584015897554</v>
+        <v>18.04583828040574</v>
       </c>
       <c r="E153" t="n">
-        <v>18.34136053518147</v>
+        <v>18.34135862584804</v>
       </c>
       <c r="F153" t="n">
         <v>8000200</v>
@@ -3492,16 +3492,16 @@
         <v>44475</v>
       </c>
       <c r="B154" t="n">
-        <v>18.27167701721191</v>
+        <v>18.27167892456055</v>
       </c>
       <c r="C154" t="n">
-        <v>18.63481622367532</v>
+        <v>18.63481816893143</v>
       </c>
       <c r="D154" t="n">
-        <v>18.06143689840233</v>
+        <v>18.06143878380436</v>
       </c>
       <c r="E154" t="n">
-        <v>18.11877428411284</v>
+        <v>18.11877617550022</v>
       </c>
       <c r="F154" t="n">
         <v>10611600</v>
@@ -3532,16 +3532,16 @@
         <v>44477</v>
       </c>
       <c r="B156" t="n">
-        <v>17.48805618286133</v>
+        <v>17.48805809020996</v>
       </c>
       <c r="C156" t="n">
-        <v>18.32901294579992</v>
+        <v>18.32901494486817</v>
       </c>
       <c r="D156" t="n">
-        <v>17.36382488657761</v>
+        <v>17.36382678037685</v>
       </c>
       <c r="E156" t="n">
-        <v>18.06143546255174</v>
+        <v>18.06143743243643</v>
       </c>
       <c r="F156" t="n">
         <v>14612800</v>
@@ -3552,16 +3552,16 @@
         <v>44480</v>
       </c>
       <c r="B157" t="n">
-        <v>16.62799072265625</v>
+        <v>16.62798690795898</v>
       </c>
       <c r="C157" t="n">
-        <v>17.52628500439614</v>
+        <v>17.5262809836174</v>
       </c>
       <c r="D157" t="n">
-        <v>16.47508980100556</v>
+        <v>16.47508602138593</v>
       </c>
       <c r="E157" t="n">
-        <v>17.42116493724025</v>
+        <v>17.42116094057755</v>
       </c>
       <c r="F157" t="n">
         <v>31512800</v>
@@ -3572,16 +3572,16 @@
         <v>44482</v>
       </c>
       <c r="B158" t="n">
-        <v>17.12491798400879</v>
+        <v>17.12491607666016</v>
       </c>
       <c r="C158" t="n">
-        <v>17.40205019435258</v>
+        <v>17.40204825613737</v>
       </c>
       <c r="D158" t="n">
-        <v>16.62798912502792</v>
+        <v>16.6279872730265</v>
       </c>
       <c r="E158" t="n">
-        <v>16.62798912502792</v>
+        <v>16.6279872730265</v>
       </c>
       <c r="F158" t="n">
         <v>10150700</v>
@@ -3592,16 +3592,16 @@
         <v>44483</v>
       </c>
       <c r="B159" t="n">
-        <v>17.06758308410645</v>
+        <v>17.06757926940918</v>
       </c>
       <c r="C159" t="n">
-        <v>17.14403354871527</v>
+        <v>17.14402971693091</v>
       </c>
       <c r="D159" t="n">
-        <v>16.60887847373064</v>
+        <v>16.60887476155634</v>
       </c>
       <c r="E159" t="n">
-        <v>16.96246301174824</v>
+        <v>16.96245922054588</v>
       </c>
       <c r="F159" t="n">
         <v>10051300</v>
@@ -3632,16 +3632,16 @@
         <v>44487</v>
       </c>
       <c r="B161" t="n">
-        <v>16.20751190185547</v>
+        <v>16.20750999450684</v>
       </c>
       <c r="C161" t="n">
-        <v>16.67577301414236</v>
+        <v>16.67577105168735</v>
       </c>
       <c r="D161" t="n">
-        <v>16.10239365985386</v>
+        <v>16.10239176487586</v>
       </c>
       <c r="E161" t="n">
-        <v>16.58976601986295</v>
+        <v>16.5897640675295</v>
       </c>
       <c r="F161" t="n">
         <v>13070300</v>
@@ -3672,16 +3672,16 @@
         <v>44489</v>
       </c>
       <c r="B163" t="n">
-        <v>15.987717628479</v>
+        <v>15.98771572113037</v>
       </c>
       <c r="C163" t="n">
-        <v>16.21706901380629</v>
+        <v>16.21706707909584</v>
       </c>
       <c r="D163" t="n">
-        <v>15.71058538806291</v>
+        <v>15.71058351377639</v>
       </c>
       <c r="E163" t="n">
-        <v>15.9399367733902</v>
+        <v>15.93993487174186</v>
       </c>
       <c r="F163" t="n">
         <v>11472200</v>
@@ -3692,16 +3692,16 @@
         <v>44490</v>
       </c>
       <c r="B164" t="n">
-        <v>15.70102691650391</v>
+        <v>15.70102882385254</v>
       </c>
       <c r="C164" t="n">
-        <v>16.21706701417989</v>
+        <v>16.21706898421667</v>
       </c>
       <c r="D164" t="n">
-        <v>15.31877465475826</v>
+        <v>15.31877651567118</v>
       </c>
       <c r="E164" t="n">
-        <v>15.81570168366632</v>
+        <v>15.81570360494555</v>
       </c>
       <c r="F164" t="n">
         <v>11995800</v>
@@ -3752,16 +3752,16 @@
         <v>44495</v>
       </c>
       <c r="B167" t="n">
-        <v>15.24232387542725</v>
+        <v>15.24232482910156</v>
       </c>
       <c r="C167" t="n">
-        <v>15.44300654837805</v>
+        <v>15.44300751460859</v>
       </c>
       <c r="D167" t="n">
-        <v>15.0129725095867</v>
+        <v>15.01297344891107</v>
       </c>
       <c r="E167" t="n">
-        <v>15.38566916259858</v>
+        <v>15.38567012524165</v>
       </c>
       <c r="F167" t="n">
         <v>7090300</v>
@@ -3872,16 +3872,16 @@
         <v>44504</v>
       </c>
       <c r="B173" t="n">
-        <v>14.52560043334961</v>
+        <v>14.52560138702393</v>
       </c>
       <c r="C173" t="n">
-        <v>14.73583964480952</v>
+        <v>14.73584061228703</v>
       </c>
       <c r="D173" t="n">
-        <v>14.30580559832982</v>
+        <v>14.30580653757357</v>
       </c>
       <c r="E173" t="n">
-        <v>14.69761441648602</v>
+        <v>14.69761538145387</v>
       </c>
       <c r="F173" t="n">
         <v>4262500</v>
@@ -3972,16 +3972,16 @@
         <v>44511</v>
       </c>
       <c r="B178" t="n">
-        <v>15.19454193115234</v>
+        <v>15.19454288482666</v>
       </c>
       <c r="C178" t="n">
-        <v>15.51945681788442</v>
+        <v>15.51945779195179</v>
       </c>
       <c r="D178" t="n">
-        <v>15.07986624960478</v>
+        <v>15.07986719608156</v>
       </c>
       <c r="E178" t="n">
-        <v>15.43344982888343</v>
+        <v>15.43345079755262</v>
       </c>
       <c r="F178" t="n">
         <v>5555700</v>
@@ -4012,16 +4012,16 @@
         <v>44516</v>
       </c>
       <c r="B180" t="n">
-        <v>14.18157291412354</v>
+        <v>14.18157196044922</v>
       </c>
       <c r="C180" t="n">
-        <v>14.86007137817213</v>
+        <v>14.86007037887054</v>
       </c>
       <c r="D180" t="n">
-        <v>14.00000240201066</v>
+        <v>14.0000014605465</v>
       </c>
       <c r="E180" t="n">
-        <v>14.81228961649183</v>
+        <v>14.81228862040344</v>
       </c>
       <c r="F180" t="n">
         <v>11424100</v>
@@ -4032,16 +4032,16 @@
         <v>44517</v>
       </c>
       <c r="B181" t="n">
-        <v>13.62730884552002</v>
+        <v>13.6273078918457</v>
       </c>
       <c r="C181" t="n">
-        <v>14.42048311764886</v>
+        <v>14.42048210846616</v>
       </c>
       <c r="D181" t="n">
-        <v>13.49352007368859</v>
+        <v>13.49351912937716</v>
       </c>
       <c r="E181" t="n">
-        <v>14.42048311764886</v>
+        <v>14.42048210846616</v>
       </c>
       <c r="F181" t="n">
         <v>10535200</v>
@@ -4052,16 +4052,16 @@
         <v>44518</v>
       </c>
       <c r="B182" t="n">
-        <v>13.35973072052002</v>
+        <v>13.3597297668457</v>
       </c>
       <c r="C182" t="n">
-        <v>13.69420217986363</v>
+        <v>13.69420120231332</v>
       </c>
       <c r="D182" t="n">
-        <v>13.13993586710555</v>
+        <v>13.13993492912112</v>
       </c>
       <c r="E182" t="n">
-        <v>13.65597694834105</v>
+        <v>13.65597597351942</v>
       </c>
       <c r="F182" t="n">
         <v>21252300</v>
@@ -4092,16 +4092,16 @@
         <v>44522</v>
       </c>
       <c r="B184" t="n">
-        <v>13.17815971374512</v>
+        <v>13.17816066741943</v>
       </c>
       <c r="C184" t="n">
-        <v>13.569968523517</v>
+        <v>13.56996950554565</v>
       </c>
       <c r="D184" t="n">
-        <v>13.12082141680619</v>
+        <v>13.12082236633105</v>
       </c>
       <c r="E184" t="n">
-        <v>13.52218676129477</v>
+        <v>13.52218773986557</v>
       </c>
       <c r="F184" t="n">
         <v>12046100</v>
@@ -4132,16 +4132,16 @@
         <v>44524</v>
       </c>
       <c r="B186" t="n">
-        <v>13.11126613616943</v>
+        <v>13.11126708984375</v>
       </c>
       <c r="C186" t="n">
-        <v>13.38839927066881</v>
+        <v>13.38840024450097</v>
       </c>
       <c r="D186" t="n">
-        <v>12.97747738072233</v>
+        <v>12.97747832466525</v>
       </c>
       <c r="E186" t="n">
-        <v>13.09215306623642</v>
+        <v>13.09215401852051</v>
       </c>
       <c r="F186" t="n">
         <v>5705900</v>
@@ -4192,16 +4192,16 @@
         <v>44529</v>
       </c>
       <c r="B189" t="n">
-        <v>12.47099208831787</v>
+        <v>12.47099304199219</v>
       </c>
       <c r="C189" t="n">
-        <v>13.11126530889348</v>
+        <v>13.11126631153039</v>
       </c>
       <c r="D189" t="n">
-        <v>12.42321032786153</v>
+        <v>12.42321127788191</v>
       </c>
       <c r="E189" t="n">
-        <v>12.88191304097531</v>
+        <v>12.88191402607333</v>
       </c>
       <c r="F189" t="n">
         <v>13464500</v>
@@ -4232,16 +4232,16 @@
         <v>44531</v>
       </c>
       <c r="B191" t="n">
-        <v>11.91672706604004</v>
+        <v>11.91672611236572</v>
       </c>
       <c r="C191" t="n">
-        <v>12.37542982579687</v>
+        <v>12.37542883541339</v>
       </c>
       <c r="D191" t="n">
-        <v>11.81160700007474</v>
+        <v>11.81160605481299</v>
       </c>
       <c r="E191" t="n">
-        <v>12.2989793658374</v>
+        <v>12.29897838157211</v>
       </c>
       <c r="F191" t="n">
         <v>5991300</v>
@@ -4252,16 +4252,16 @@
         <v>44532</v>
       </c>
       <c r="B192" t="n">
-        <v>11.89761257171631</v>
+        <v>11.89761447906494</v>
       </c>
       <c r="C192" t="n">
-        <v>12.14607699253434</v>
+        <v>12.14607893971519</v>
       </c>
       <c r="D192" t="n">
-        <v>11.71604297887929</v>
+        <v>11.71604485711986</v>
       </c>
       <c r="E192" t="n">
-        <v>12.14607699253434</v>
+        <v>12.14607893971519</v>
       </c>
       <c r="F192" t="n">
         <v>7306700</v>
@@ -4292,16 +4292,16 @@
         <v>44536</v>
       </c>
       <c r="B194" t="n">
-        <v>13.13993549346924</v>
+        <v>13.13993453979492</v>
       </c>
       <c r="C194" t="n">
-        <v>13.28327987976253</v>
+        <v>13.28327891568452</v>
       </c>
       <c r="D194" t="n">
-        <v>12.77679534865</v>
+        <v>12.77679442133178</v>
       </c>
       <c r="E194" t="n">
-        <v>12.83413364998414</v>
+        <v>12.83413271850441</v>
       </c>
       <c r="F194" t="n">
         <v>6605800</v>
@@ -4332,16 +4332,16 @@
         <v>44538</v>
       </c>
       <c r="B196" t="n">
-        <v>13.75153827667236</v>
+        <v>13.75153923034668</v>
       </c>
       <c r="C196" t="n">
-        <v>14.02867138859101</v>
+        <v>14.02867236148461</v>
       </c>
       <c r="D196" t="n">
-        <v>13.2737225036153</v>
+        <v>13.27372342415291</v>
       </c>
       <c r="E196" t="n">
-        <v>13.42662340517576</v>
+        <v>13.42662433631711</v>
       </c>
       <c r="F196" t="n">
         <v>14295000</v>
@@ -4372,16 +4372,16 @@
         <v>44540</v>
       </c>
       <c r="B198" t="n">
-        <v>13.91399574279785</v>
+        <v>13.91399669647217</v>
       </c>
       <c r="C198" t="n">
-        <v>14.19112885532154</v>
+        <v>14.19112982799074</v>
       </c>
       <c r="D198" t="n">
-        <v>13.74198177248616</v>
+        <v>13.74198271437053</v>
       </c>
       <c r="E198" t="n">
-        <v>13.74198177248616</v>
+        <v>13.74198271437053</v>
       </c>
       <c r="F198" t="n">
         <v>8247400</v>
@@ -4452,16 +4452,16 @@
         <v>44546</v>
       </c>
       <c r="B202" t="n">
-        <v>13.89488410949707</v>
+        <v>13.89488506317139</v>
       </c>
       <c r="C202" t="n">
-        <v>14.28669293890897</v>
+        <v>14.28669391947506</v>
       </c>
       <c r="D202" t="n">
-        <v>13.82799018584958</v>
+        <v>13.82799113493264</v>
       </c>
       <c r="E202" t="n">
-        <v>14.21024248006574</v>
+        <v>14.21024345538466</v>
       </c>
       <c r="F202" t="n">
         <v>5287600</v>
@@ -4472,16 +4472,16 @@
         <v>44547</v>
       </c>
       <c r="B203" t="n">
-        <v>13.818434715271</v>
+        <v>13.81843280792236</v>
       </c>
       <c r="C203" t="n">
-        <v>14.00956087710406</v>
+        <v>14.00955894337442</v>
       </c>
       <c r="D203" t="n">
-        <v>13.64642071394053</v>
+        <v>13.64641883033486</v>
       </c>
       <c r="E203" t="n">
-        <v>13.8471034117056</v>
+        <v>13.84710150039985</v>
       </c>
       <c r="F203" t="n">
         <v>8250000</v>
@@ -4492,16 +4492,16 @@
         <v>44550</v>
       </c>
       <c r="B204" t="n">
-        <v>13.47440719604492</v>
+        <v>13.47440624237061</v>
       </c>
       <c r="C204" t="n">
-        <v>13.8662160431998</v>
+        <v>13.86621506179454</v>
       </c>
       <c r="D204" t="n">
-        <v>13.29283666454885</v>
+        <v>13.29283572372549</v>
       </c>
       <c r="E204" t="n">
-        <v>13.81843427641866</v>
+        <v>13.81843329839523</v>
       </c>
       <c r="F204" t="n">
         <v>6680500</v>
@@ -4512,16 +4512,16 @@
         <v>44551</v>
       </c>
       <c r="B205" t="n">
-        <v>13.617751121521</v>
+        <v>13.61775016784668</v>
       </c>
       <c r="C205" t="n">
-        <v>13.6655328866758</v>
+        <v>13.66553192965524</v>
       </c>
       <c r="D205" t="n">
-        <v>13.36928667180511</v>
+        <v>13.36928573553119</v>
       </c>
       <c r="E205" t="n">
-        <v>13.48396236135982</v>
+        <v>13.48396141705496</v>
       </c>
       <c r="F205" t="n">
         <v>4083800</v>
@@ -4552,16 +4552,16 @@
         <v>44553</v>
       </c>
       <c r="B207" t="n">
-        <v>13.4648494720459</v>
+        <v>13.46484851837158</v>
       </c>
       <c r="C207" t="n">
-        <v>13.65597561094082</v>
+        <v>13.65597464372962</v>
       </c>
       <c r="D207" t="n">
-        <v>13.32150418435372</v>
+        <v>13.32150324083211</v>
       </c>
       <c r="E207" t="n">
-        <v>13.41706770948184</v>
+        <v>13.41706675919176</v>
       </c>
       <c r="F207" t="n">
         <v>4198000</v>
@@ -4572,16 +4572,16 @@
         <v>44557</v>
       </c>
       <c r="B208" t="n">
-        <v>13.03481578826904</v>
+        <v>13.03481483459473</v>
       </c>
       <c r="C208" t="n">
-        <v>13.56041245676783</v>
+        <v>13.56041146463896</v>
       </c>
       <c r="D208" t="n">
-        <v>12.90102703170205</v>
+        <v>12.9010260878162</v>
       </c>
       <c r="E208" t="n">
-        <v>13.46484984038684</v>
+        <v>13.46484885524968</v>
       </c>
       <c r="F208" t="n">
         <v>14666400</v>
@@ -4692,16 +4692,16 @@
         <v>44566</v>
       </c>
       <c r="B214" t="n">
-        <v>11.45802211761475</v>
+        <v>11.45802307128906</v>
       </c>
       <c r="C214" t="n">
-        <v>12.13652055763904</v>
+        <v>12.13652156778615</v>
       </c>
       <c r="D214" t="n">
-        <v>11.41024035762631</v>
+        <v>11.41024130732365</v>
       </c>
       <c r="E214" t="n">
-        <v>12.11740840046043</v>
+        <v>12.1174094090168</v>
       </c>
       <c r="F214" t="n">
         <v>11220000</v>
@@ -4732,16 +4732,16 @@
         <v>44568</v>
       </c>
       <c r="B216" t="n">
-        <v>10.85597515106201</v>
+        <v>10.85597610473633</v>
       </c>
       <c r="C216" t="n">
-        <v>11.11399613247418</v>
+        <v>11.11399710881509</v>
       </c>
       <c r="D216" t="n">
-        <v>10.71263076896282</v>
+        <v>10.71263171004464</v>
       </c>
       <c r="E216" t="n">
-        <v>11.0088769796922</v>
+        <v>11.00887794679861</v>
       </c>
       <c r="F216" t="n">
         <v>11641900</v>
@@ -4752,16 +4752,16 @@
         <v>44571</v>
       </c>
       <c r="B217" t="n">
-        <v>10.79863739013672</v>
+        <v>10.7986364364624</v>
       </c>
       <c r="C217" t="n">
-        <v>10.8559747764533</v>
+        <v>10.85597381771528</v>
       </c>
       <c r="D217" t="n">
-        <v>10.54061641762812</v>
+        <v>10.54061548674074</v>
       </c>
       <c r="E217" t="n">
-        <v>10.76041216213855</v>
+        <v>10.76041121184007</v>
       </c>
       <c r="F217" t="n">
         <v>8755800</v>
@@ -4812,16 +4812,16 @@
         <v>44574</v>
       </c>
       <c r="B220" t="n">
-        <v>11.48669338226318</v>
+        <v>11.48669147491455</v>
       </c>
       <c r="C220" t="n">
-        <v>11.57269946905179</v>
+        <v>11.57269754742197</v>
       </c>
       <c r="D220" t="n">
-        <v>11.15222192531568</v>
+        <v>11.15222007350554</v>
       </c>
       <c r="E220" t="n">
-        <v>11.27645415471443</v>
+        <v>11.27645228227571</v>
       </c>
       <c r="F220" t="n">
         <v>9668300</v>
@@ -4832,16 +4832,16 @@
         <v>44575</v>
       </c>
       <c r="B221" t="n">
-        <v>11.59181118011475</v>
+        <v>11.59181213378906</v>
       </c>
       <c r="C221" t="n">
-        <v>11.65870509911001</v>
+        <v>11.65870605828779</v>
       </c>
       <c r="D221" t="n">
-        <v>11.39112851176765</v>
+        <v>11.39112944893152</v>
       </c>
       <c r="E221" t="n">
-        <v>11.4102406694686</v>
+        <v>11.41024160820486</v>
       </c>
       <c r="F221" t="n">
         <v>7586600</v>
@@ -4872,16 +4872,16 @@
         <v>44579</v>
       </c>
       <c r="B223" t="n">
-        <v>11.3911304473877</v>
+        <v>11.39112949371338</v>
       </c>
       <c r="C223" t="n">
-        <v>11.49624961100837</v>
+        <v>11.49624864853339</v>
       </c>
       <c r="D223" t="n">
-        <v>11.29556690856058</v>
+        <v>11.29556596288691</v>
       </c>
       <c r="E223" t="n">
-        <v>11.47713745005981</v>
+        <v>11.47713648918492</v>
       </c>
       <c r="F223" t="n">
         <v>7771300</v>
@@ -4912,16 +4912,16 @@
         <v>44581</v>
       </c>
       <c r="B225" t="n">
-        <v>11.41979789733887</v>
+        <v>11.41979885101318</v>
       </c>
       <c r="C225" t="n">
-        <v>11.69693103603816</v>
+        <v>11.69693201285603</v>
       </c>
       <c r="D225" t="n">
-        <v>11.36246050939355</v>
+        <v>11.36246145827959</v>
       </c>
       <c r="E225" t="n">
-        <v>11.56314318992485</v>
+        <v>11.56314415557002</v>
       </c>
       <c r="F225" t="n">
         <v>7365800</v>
@@ -4932,16 +4932,16 @@
         <v>44582</v>
       </c>
       <c r="B226" t="n">
-        <v>11.48669338226318</v>
+        <v>11.48669147491455</v>
       </c>
       <c r="C226" t="n">
-        <v>11.6300377716056</v>
+        <v>11.63003584045484</v>
       </c>
       <c r="D226" t="n">
-        <v>11.21911585216062</v>
+        <v>11.21911398924284</v>
       </c>
       <c r="E226" t="n">
-        <v>11.37201677715557</v>
+        <v>11.37201488884882</v>
       </c>
       <c r="F226" t="n">
         <v>8537100</v>
@@ -4952,16 +4952,16 @@
         <v>44585</v>
       </c>
       <c r="B227" t="n">
-        <v>11.50580501556396</v>
+        <v>11.50580406188965</v>
       </c>
       <c r="C227" t="n">
-        <v>11.63959377449148</v>
+        <v>11.6395928097279</v>
       </c>
       <c r="D227" t="n">
-        <v>11.3242354032836</v>
+        <v>11.32423446465893</v>
       </c>
       <c r="E227" t="n">
-        <v>11.46757978606487</v>
+        <v>11.4675788355589</v>
       </c>
       <c r="F227" t="n">
         <v>6551900</v>
@@ -5012,16 +5012,16 @@
         <v>44588</v>
       </c>
       <c r="B230" t="n">
-        <v>11.99317646026611</v>
+        <v>11.99317741394043</v>
       </c>
       <c r="C230" t="n">
-        <v>12.13652083211196</v>
+        <v>12.13652179718475</v>
       </c>
       <c r="D230" t="n">
-        <v>11.66826157863015</v>
+        <v>11.66826250646786</v>
       </c>
       <c r="E230" t="n">
-        <v>11.85938771154504</v>
+        <v>11.85938865458074</v>
       </c>
       <c r="F230" t="n">
         <v>13761300</v>
@@ -5032,16 +5032,16 @@
         <v>44589</v>
       </c>
       <c r="B231" t="n">
-        <v>11.83071994781494</v>
+        <v>11.83072090148926</v>
       </c>
       <c r="C231" t="n">
-        <v>12.04095916619962</v>
+        <v>12.04096013682132</v>
       </c>
       <c r="D231" t="n">
-        <v>11.4580232758641</v>
+        <v>11.45802419949534</v>
       </c>
       <c r="E231" t="n">
-        <v>11.94539563656258</v>
+        <v>11.9453965994809</v>
       </c>
       <c r="F231" t="n">
         <v>14924100</v>
@@ -5072,16 +5072,16 @@
         <v>44593</v>
       </c>
       <c r="B233" t="n">
-        <v>12.0218448638916</v>
+        <v>12.02184581756592</v>
       </c>
       <c r="C233" t="n">
-        <v>12.09829531522309</v>
+        <v>12.0982962749621</v>
       </c>
       <c r="D233" t="n">
-        <v>11.83071873556289</v>
+        <v>11.83071967407547</v>
       </c>
       <c r="E233" t="n">
-        <v>11.93583787830337</v>
+        <v>11.93583882515488</v>
       </c>
       <c r="F233" t="n">
         <v>5991900</v>
@@ -5092,16 +5092,16 @@
         <v>44594</v>
       </c>
       <c r="B234" t="n">
-        <v>11.94539451599121</v>
+        <v>11.94539356231689</v>
       </c>
       <c r="C234" t="n">
-        <v>12.27986592698347</v>
+        <v>12.27986494660625</v>
       </c>
       <c r="D234" t="n">
-        <v>11.81160576932205</v>
+        <v>11.81160482632891</v>
       </c>
       <c r="E234" t="n">
-        <v>12.02184496798465</v>
+        <v>12.02184400820683</v>
       </c>
       <c r="F234" t="n">
         <v>9442200</v>
@@ -5112,16 +5112,16 @@
         <v>44595</v>
       </c>
       <c r="B235" t="n">
-        <v>11.94539451599121</v>
+        <v>11.94539356231689</v>
       </c>
       <c r="C235" t="n">
-        <v>12.21297109796826</v>
+        <v>12.21297012293166</v>
       </c>
       <c r="D235" t="n">
-        <v>11.89761275565499</v>
+        <v>11.89761180579539</v>
       </c>
       <c r="E235" t="n">
-        <v>12.04095803666365</v>
+        <v>12.04095707535991</v>
       </c>
       <c r="F235" t="n">
         <v>8796800</v>
@@ -5132,16 +5132,16 @@
         <v>44596</v>
       </c>
       <c r="B236" t="n">
-        <v>12.32764720916748</v>
+        <v>12.3276481628418</v>
       </c>
       <c r="C236" t="n">
-        <v>12.32764720916748</v>
+        <v>12.3276481628418</v>
       </c>
       <c r="D236" t="n">
-        <v>11.56314266236741</v>
+        <v>11.56314355689919</v>
       </c>
       <c r="E236" t="n">
-        <v>11.91672624310277</v>
+        <v>11.91672716498799</v>
       </c>
       <c r="F236" t="n">
         <v>17676100</v>
@@ -5152,16 +5152,16 @@
         <v>44599</v>
       </c>
       <c r="B237" t="n">
-        <v>12.20341682434082</v>
+        <v>12.2034158706665</v>
       </c>
       <c r="C237" t="n">
-        <v>12.60478128600524</v>
+        <v>12.60478030096504</v>
       </c>
       <c r="D237" t="n">
-        <v>12.20341682434082</v>
+        <v>12.2034158706665</v>
       </c>
       <c r="E237" t="n">
-        <v>12.29897944421849</v>
+        <v>12.29897848307614</v>
       </c>
       <c r="F237" t="n">
         <v>7212000</v>
@@ -5252,16 +5252,16 @@
         <v>44606</v>
       </c>
       <c r="B242" t="n">
-        <v>11.78293800354004</v>
+        <v>11.78293704986572</v>
       </c>
       <c r="C242" t="n">
-        <v>11.97406414854188</v>
+        <v>11.97406317939841</v>
       </c>
       <c r="D242" t="n">
-        <v>11.639593622629</v>
+        <v>11.63959268055653</v>
       </c>
       <c r="E242" t="n">
-        <v>11.79249453863047</v>
+        <v>11.79249358418268</v>
       </c>
       <c r="F242" t="n">
         <v>5445000</v>
@@ -5272,16 +5272,16 @@
         <v>44607</v>
       </c>
       <c r="B243" t="n">
-        <v>11.63959407806396</v>
+        <v>11.63959312438965</v>
       </c>
       <c r="C243" t="n">
-        <v>11.95495245749671</v>
+        <v>11.95495147798393</v>
       </c>
       <c r="D243" t="n">
-        <v>11.5344740106788</v>
+        <v>11.53447306561735</v>
       </c>
       <c r="E243" t="n">
-        <v>11.92628285110363</v>
+        <v>11.92628187393986</v>
       </c>
       <c r="F243" t="n">
         <v>11329100</v>
@@ -5292,16 +5292,16 @@
         <v>44608</v>
       </c>
       <c r="B244" t="n">
-        <v>12.47099208831787</v>
+        <v>12.47099304199219</v>
       </c>
       <c r="C244" t="n">
-        <v>12.6430051500549</v>
+        <v>12.6430061168833</v>
       </c>
       <c r="D244" t="n">
-        <v>11.56314228509255</v>
+        <v>11.56314316934232</v>
       </c>
       <c r="E244" t="n">
-        <v>11.65870489464395</v>
+        <v>11.65870578620152</v>
       </c>
       <c r="F244" t="n">
         <v>21489000</v>
@@ -5312,16 +5312,16 @@
         <v>44609</v>
       </c>
       <c r="B245" t="n">
-        <v>12.66211986541748</v>
+        <v>12.66211795806885</v>
       </c>
       <c r="C245" t="n">
-        <v>12.94880955407657</v>
+        <v>12.94880760354266</v>
       </c>
       <c r="D245" t="n">
-        <v>12.46143717449226</v>
+        <v>12.46143529737331</v>
       </c>
       <c r="E245" t="n">
-        <v>12.46143717449226</v>
+        <v>12.46143529737331</v>
       </c>
       <c r="F245" t="n">
         <v>10362100</v>
@@ -5332,16 +5332,16 @@
         <v>44610</v>
       </c>
       <c r="B246" t="n">
-        <v>12.13652229309082</v>
+        <v>12.1365213394165</v>
       </c>
       <c r="C246" t="n">
-        <v>12.83413390140938</v>
+        <v>12.83413289291753</v>
       </c>
       <c r="D246" t="n">
-        <v>12.13652229309082</v>
+        <v>12.1365213394165</v>
       </c>
       <c r="E246" t="n">
-        <v>12.80546429449997</v>
+        <v>12.80546328826094</v>
       </c>
       <c r="F246" t="n">
         <v>11604500</v>
@@ -5392,16 +5392,16 @@
         <v>44615</v>
       </c>
       <c r="B249" t="n">
-        <v>12.73856830596924</v>
+        <v>12.73857021331787</v>
       </c>
       <c r="C249" t="n">
-        <v>12.87235704914128</v>
+        <v>12.87235897652213</v>
       </c>
       <c r="D249" t="n">
-        <v>12.51877349007365</v>
+        <v>12.51877536451236</v>
       </c>
       <c r="E249" t="n">
-        <v>12.51877349007365</v>
+        <v>12.51877536451236</v>
       </c>
       <c r="F249" t="n">
         <v>5598100</v>
@@ -5452,16 +5452,16 @@
         <v>44622</v>
       </c>
       <c r="B252" t="n">
-        <v>12.68123245239258</v>
+        <v>12.68123149871826</v>
       </c>
       <c r="C252" t="n">
-        <v>12.95836559486294</v>
+        <v>12.95836462034722</v>
       </c>
       <c r="D252" t="n">
-        <v>12.64300631142708</v>
+        <v>12.6430053606275</v>
       </c>
       <c r="E252" t="n">
-        <v>12.86280206517191</v>
+        <v>12.8628010978429</v>
       </c>
       <c r="F252" t="n">
         <v>4196000</v>
@@ -5592,16 +5592,16 @@
         <v>44631</v>
       </c>
       <c r="B259" t="n">
-        <v>12.40409851074219</v>
+        <v>12.40409755706787</v>
       </c>
       <c r="C259" t="n">
-        <v>12.9296961060736</v>
+        <v>12.92969511198934</v>
       </c>
       <c r="D259" t="n">
-        <v>12.20341673702652</v>
+        <v>12.20341579878139</v>
       </c>
       <c r="E259" t="n">
-        <v>12.9296961060736</v>
+        <v>12.92969511198934</v>
       </c>
       <c r="F259" t="n">
         <v>7293900</v>
@@ -5632,16 +5632,16 @@
         <v>44635</v>
       </c>
       <c r="B261" t="n">
-        <v>12.82457447052002</v>
+        <v>12.82457542419434</v>
       </c>
       <c r="C261" t="n">
-        <v>12.90102491562967</v>
+        <v>12.90102587498907</v>
       </c>
       <c r="D261" t="n">
-        <v>12.29897697687028</v>
+        <v>12.29897789145957</v>
       </c>
       <c r="E261" t="n">
-        <v>12.29897697687028</v>
+        <v>12.29897789145957</v>
       </c>
       <c r="F261" t="n">
         <v>8181800</v>
@@ -5772,16 +5772,16 @@
         <v>44644</v>
       </c>
       <c r="B268" t="n">
-        <v>14.63071918487549</v>
+        <v>14.63072109222412</v>
       </c>
       <c r="C268" t="n">
-        <v>14.7453948595791</v>
+        <v>14.74539678187754</v>
       </c>
       <c r="D268" t="n">
-        <v>14.35358607650145</v>
+        <v>14.35358794772134</v>
       </c>
       <c r="E268" t="n">
-        <v>14.39181130140265</v>
+        <v>14.39181317760581</v>
       </c>
       <c r="F268" t="n">
         <v>7986800</v>
@@ -5792,16 +5792,16 @@
         <v>44645</v>
       </c>
       <c r="B269" t="n">
-        <v>15.13720512390137</v>
+        <v>15.13720417022705</v>
       </c>
       <c r="C269" t="n">
-        <v>15.24232427482575</v>
+        <v>15.24232331452872</v>
       </c>
       <c r="D269" t="n">
-        <v>14.64027624019771</v>
+        <v>14.64027531783091</v>
       </c>
       <c r="E269" t="n">
-        <v>14.71672669748114</v>
+        <v>14.71672577029781</v>
       </c>
       <c r="F269" t="n">
         <v>8426200</v>
@@ -5812,16 +5812,16 @@
         <v>44648</v>
       </c>
       <c r="B270" t="n">
-        <v>15.51945686340332</v>
+        <v>15.519455909729</v>
       </c>
       <c r="C270" t="n">
-        <v>15.7774778311631</v>
+        <v>15.77747686163333</v>
       </c>
       <c r="D270" t="n">
-        <v>14.97474714661442</v>
+        <v>14.97474622641265</v>
       </c>
       <c r="E270" t="n">
-        <v>15.19454197571826</v>
+        <v>15.19454104201004</v>
       </c>
       <c r="F270" t="n">
         <v>14496800</v>
@@ -5832,16 +5832,16 @@
         <v>44649</v>
       </c>
       <c r="B271" t="n">
-        <v>15.50034427642822</v>
+        <v>15.50034236907959</v>
       </c>
       <c r="C271" t="n">
-        <v>15.93037923607671</v>
+        <v>15.93037727581141</v>
       </c>
       <c r="D271" t="n">
-        <v>15.43345035442127</v>
+        <v>15.43344845530407</v>
       </c>
       <c r="E271" t="n">
-        <v>15.72969564733319</v>
+        <v>15.72969371176241</v>
       </c>
       <c r="F271" t="n">
         <v>7323700</v>
@@ -5852,16 +5852,16 @@
         <v>44650</v>
       </c>
       <c r="B272" t="n">
-        <v>15.45256423950195</v>
+        <v>15.45256328582764</v>
       </c>
       <c r="C272" t="n">
-        <v>15.82526000904275</v>
+        <v>15.82525903236704</v>
       </c>
       <c r="D272" t="n">
-        <v>15.3952268494317</v>
+        <v>15.39522589929603</v>
       </c>
       <c r="E272" t="n">
-        <v>15.51945816503771</v>
+        <v>15.51945720723495</v>
       </c>
       <c r="F272" t="n">
         <v>8944100</v>
@@ -5932,16 +5932,16 @@
         <v>44656</v>
       </c>
       <c r="B276" t="n">
-        <v>15.45256423950195</v>
+        <v>15.45256328582764</v>
       </c>
       <c r="C276" t="n">
-        <v>15.65324601610922</v>
+        <v>15.65324505004958</v>
       </c>
       <c r="D276" t="n">
-        <v>15.35700070756969</v>
+        <v>15.35699975979319</v>
       </c>
       <c r="E276" t="n">
-        <v>15.57679555510796</v>
+        <v>15.57679459376655</v>
       </c>
       <c r="F276" t="n">
         <v>10716200</v>
@@ -5972,16 +5972,16 @@
         <v>44658</v>
       </c>
       <c r="B278" t="n">
-        <v>15.38566970825195</v>
+        <v>15.38567066192627</v>
       </c>
       <c r="C278" t="n">
-        <v>15.52901408914568</v>
+        <v>15.52901505170514</v>
       </c>
       <c r="D278" t="n">
-        <v>15.25188095108615</v>
+        <v>15.25188189646763</v>
       </c>
       <c r="E278" t="n">
-        <v>15.3665566380734</v>
+        <v>15.366557590563</v>
       </c>
       <c r="F278" t="n">
         <v>6566700</v>
@@ -5992,16 +5992,16 @@
         <v>44659</v>
       </c>
       <c r="B279" t="n">
-        <v>15.40478134155273</v>
+        <v>15.40478420257568</v>
       </c>
       <c r="C279" t="n">
-        <v>15.5767934889472</v>
+        <v>15.57679638191676</v>
       </c>
       <c r="D279" t="n">
-        <v>15.07030993551665</v>
+        <v>15.07031273442055</v>
       </c>
       <c r="E279" t="n">
-        <v>15.32833089069213</v>
+        <v>15.32833373751647</v>
       </c>
       <c r="F279" t="n">
         <v>3069100</v>
@@ -6012,16 +6012,16 @@
         <v>44662</v>
       </c>
       <c r="B280" t="n">
-        <v>15.29010581970215</v>
+        <v>15.29010486602783</v>
       </c>
       <c r="C280" t="n">
-        <v>15.49078758367887</v>
+        <v>15.49078661748763</v>
       </c>
       <c r="D280" t="n">
-        <v>15.21365536351254</v>
+        <v>15.21365441460659</v>
       </c>
       <c r="E280" t="n">
-        <v>15.38566934561982</v>
+        <v>15.38566838598501</v>
       </c>
       <c r="F280" t="n">
         <v>10289300</v>
@@ -6032,16 +6032,16 @@
         <v>44663</v>
       </c>
       <c r="B281" t="n">
-        <v>15.72014236450195</v>
+        <v>15.72014045715332</v>
       </c>
       <c r="C281" t="n">
-        <v>15.82526061318996</v>
+        <v>15.82525869308717</v>
       </c>
       <c r="D281" t="n">
-        <v>15.39522743716192</v>
+        <v>15.3952255692357</v>
       </c>
       <c r="E281" t="n">
-        <v>15.48123443691209</v>
+        <v>15.48123255855052</v>
       </c>
       <c r="F281" t="n">
         <v>9798400</v>
@@ -6072,16 +6072,16 @@
         <v>44665</v>
       </c>
       <c r="B283" t="n">
-        <v>15.64369010925293</v>
+        <v>15.64368915557861</v>
       </c>
       <c r="C283" t="n">
-        <v>15.79659101958422</v>
+        <v>15.79659005658872</v>
       </c>
       <c r="D283" t="n">
-        <v>15.4812326641856</v>
+        <v>15.48123172041506</v>
       </c>
       <c r="E283" t="n">
-        <v>15.72014056441858</v>
+        <v>15.72013960608367</v>
       </c>
       <c r="F283" t="n">
         <v>4607000</v>
@@ -6092,16 +6092,16 @@
         <v>44669</v>
       </c>
       <c r="B284" t="n">
-        <v>15.31877517700195</v>
+        <v>15.31877422332764</v>
       </c>
       <c r="C284" t="n">
-        <v>15.67235784764996</v>
+        <v>15.67235687196327</v>
       </c>
       <c r="D284" t="n">
-        <v>15.31877517700195</v>
+        <v>15.31877422332764</v>
       </c>
       <c r="E284" t="n">
-        <v>15.56723961128785</v>
+        <v>15.56723864214531</v>
       </c>
       <c r="F284" t="n">
         <v>3539900</v>
@@ -6152,16 +6152,16 @@
         <v>44673</v>
       </c>
       <c r="B287" t="n">
-        <v>15.31877517700195</v>
+        <v>15.31877422332764</v>
       </c>
       <c r="C287" t="n">
-        <v>15.74880830260542</v>
+        <v>15.74880732215928</v>
       </c>
       <c r="D287" t="n">
-        <v>15.14676119767152</v>
+        <v>15.14676025470597</v>
       </c>
       <c r="E287" t="n">
-        <v>15.74880830260542</v>
+        <v>15.74880732215928</v>
       </c>
       <c r="F287" t="n">
         <v>8878800</v>
@@ -6292,16 +6292,16 @@
         <v>44684</v>
       </c>
       <c r="B294" t="n">
-        <v>14.62423324584961</v>
+        <v>14.62423419952393</v>
       </c>
       <c r="C294" t="n">
-        <v>14.85544619454671</v>
+        <v>14.85544716329886</v>
       </c>
       <c r="D294" t="n">
-        <v>14.47972446384498</v>
+        <v>14.4797254080956</v>
       </c>
       <c r="E294" t="n">
-        <v>14.70130422874864</v>
+        <v>14.70130518744891</v>
       </c>
       <c r="F294" t="n">
         <v>5388000</v>
@@ -6372,16 +6372,16 @@
         <v>44690</v>
       </c>
       <c r="B298" t="n">
-        <v>14.21961212158203</v>
+        <v>14.21961116790771</v>
       </c>
       <c r="C298" t="n">
-        <v>14.32558450824887</v>
+        <v>14.32558354746724</v>
       </c>
       <c r="D298" t="n">
-        <v>13.92096133187191</v>
+        <v>13.92096039822737</v>
       </c>
       <c r="E298" t="n">
-        <v>14.04620192634656</v>
+        <v>14.04620098430244</v>
       </c>
       <c r="F298" t="n">
         <v>11844800</v>
@@ -6452,16 +6452,16 @@
         <v>44694</v>
       </c>
       <c r="B302" t="n">
-        <v>14.91324996948242</v>
+        <v>14.91324901580811</v>
       </c>
       <c r="C302" t="n">
-        <v>15.09629425517541</v>
+        <v>15.09629328979575</v>
       </c>
       <c r="D302" t="n">
-        <v>14.62423422366596</v>
+        <v>14.62423328847366</v>
       </c>
       <c r="E302" t="n">
-        <v>14.7205724993519</v>
+        <v>14.72057155799894</v>
       </c>
       <c r="F302" t="n">
         <v>5016200</v>
@@ -6472,16 +6472,16 @@
         <v>44697</v>
       </c>
       <c r="B303" t="n">
-        <v>14.80727577209473</v>
+        <v>14.80727672576904</v>
       </c>
       <c r="C303" t="n">
-        <v>14.93251634198823</v>
+        <v>14.93251730372877</v>
       </c>
       <c r="D303" t="n">
-        <v>14.64349971290772</v>
+        <v>14.64350065603391</v>
       </c>
       <c r="E303" t="n">
-        <v>14.93251634198823</v>
+        <v>14.93251730372877</v>
       </c>
       <c r="F303" t="n">
         <v>6824600</v>
@@ -6532,16 +6532,16 @@
         <v>44700</v>
       </c>
       <c r="B306" t="n">
-        <v>14.88434791564941</v>
+        <v>14.88434886932373</v>
       </c>
       <c r="C306" t="n">
-        <v>14.95178571626016</v>
+        <v>14.95178667425537</v>
       </c>
       <c r="D306" t="n">
-        <v>14.6627690645589</v>
+        <v>14.66277000403615</v>
       </c>
       <c r="E306" t="n">
-        <v>14.92288340795901</v>
+        <v>14.92288436410238</v>
       </c>
       <c r="F306" t="n">
         <v>6219800</v>
@@ -6552,16 +6552,16 @@
         <v>44701</v>
       </c>
       <c r="B307" t="n">
-        <v>15.37567710876465</v>
+        <v>15.37567615509033</v>
       </c>
       <c r="C307" t="n">
-        <v>15.49128359304003</v>
+        <v>15.49128263219524</v>
       </c>
       <c r="D307" t="n">
-        <v>14.93251845966301</v>
+        <v>14.93251753347555</v>
       </c>
       <c r="E307" t="n">
-        <v>15.0288576559385</v>
+        <v>15.02885672377561</v>
       </c>
       <c r="F307" t="n">
         <v>8142900</v>
@@ -6752,16 +6752,16 @@
         <v>44715</v>
       </c>
       <c r="B317" t="n">
-        <v>14.88434791564941</v>
+        <v>14.88434886932373</v>
       </c>
       <c r="C317" t="n">
-        <v>15.23116826519437</v>
+        <v>15.23116924109026</v>
       </c>
       <c r="D317" t="n">
-        <v>14.78800964425473</v>
+        <v>14.78801059175644</v>
       </c>
       <c r="E317" t="n">
-        <v>15.17336456735067</v>
+        <v>15.17336553954295</v>
       </c>
       <c r="F317" t="n">
         <v>4184100</v>
@@ -6852,16 +6852,16 @@
         <v>44722</v>
       </c>
       <c r="B322" t="n">
-        <v>14.48935985565186</v>
+        <v>14.48935890197754</v>
       </c>
       <c r="C322" t="n">
-        <v>15.01922359929862</v>
+        <v>15.01922261074923</v>
       </c>
       <c r="D322" t="n">
-        <v>14.22924549491244</v>
+        <v>14.22924455835858</v>
       </c>
       <c r="E322" t="n">
-        <v>14.85544751637582</v>
+        <v>14.85544653860601</v>
       </c>
       <c r="F322" t="n">
         <v>15101900</v>
@@ -6912,16 +6912,16 @@
         <v>44727</v>
       </c>
       <c r="B325" t="n">
-        <v>14.91324996948242</v>
+        <v>14.91324901580811</v>
       </c>
       <c r="C325" t="n">
-        <v>15.06739286434549</v>
+        <v>15.06739190081403</v>
       </c>
       <c r="D325" t="n">
-        <v>14.25814657103863</v>
+        <v>14.25814565925695</v>
       </c>
       <c r="E325" t="n">
-        <v>14.34485166228703</v>
+        <v>14.34485074496072</v>
       </c>
       <c r="F325" t="n">
         <v>25461900</v>
@@ -6992,16 +6992,16 @@
         <v>44734</v>
       </c>
       <c r="B329" t="n">
-        <v>14.44118976593018</v>
+        <v>14.44119071960449</v>
       </c>
       <c r="C329" t="n">
-        <v>15.13482956889515</v>
+        <v>15.13483056837639</v>
       </c>
       <c r="D329" t="n">
-        <v>14.32558328522912</v>
+        <v>14.32558423126896</v>
       </c>
       <c r="E329" t="n">
-        <v>14.6820368304137</v>
+        <v>14.68203779999319</v>
       </c>
       <c r="F329" t="n">
         <v>8791300</v>
@@ -7032,16 +7032,16 @@
         <v>44736</v>
       </c>
       <c r="B331" t="n">
-        <v>14.4219217300415</v>
+        <v>14.42192268371582</v>
       </c>
       <c r="C331" t="n">
-        <v>14.86508034244202</v>
+        <v>14.86508132542095</v>
       </c>
       <c r="D331" t="n">
-        <v>14.25814566119184</v>
+        <v>14.25814660403618</v>
       </c>
       <c r="E331" t="n">
-        <v>14.86508034244202</v>
+        <v>14.86508132542095</v>
       </c>
       <c r="F331" t="n">
         <v>5803600</v>
@@ -7052,16 +7052,16 @@
         <v>44739</v>
       </c>
       <c r="B332" t="n">
-        <v>14.1618070602417</v>
+        <v>14.16180801391602</v>
       </c>
       <c r="C332" t="n">
-        <v>14.4989933145069</v>
+        <v>14.49899429088777</v>
       </c>
       <c r="D332" t="n">
-        <v>14.10400427987309</v>
+        <v>14.10400522965489</v>
       </c>
       <c r="E332" t="n">
-        <v>14.47972510854494</v>
+        <v>14.47972608362827</v>
       </c>
       <c r="F332" t="n">
         <v>8041800</v>
@@ -7072,16 +7072,16 @@
         <v>44740</v>
       </c>
       <c r="B333" t="n">
-        <v>14.08473491668701</v>
+        <v>14.08473587036133</v>
       </c>
       <c r="C333" t="n">
-        <v>14.48935802105732</v>
+        <v>14.48935900212858</v>
       </c>
       <c r="D333" t="n">
-        <v>13.96912844668957</v>
+        <v>13.9691293925362</v>
       </c>
       <c r="E333" t="n">
-        <v>14.2388768766836</v>
+        <v>14.23887784079483</v>
       </c>
       <c r="F333" t="n">
         <v>7081400</v>
@@ -7292,16 +7292,16 @@
         <v>44755</v>
       </c>
       <c r="B344" t="n">
-        <v>14.77837467193604</v>
+        <v>14.77837562561035</v>
       </c>
       <c r="C344" t="n">
-        <v>15.01922171438934</v>
+        <v>15.01922268360593</v>
       </c>
       <c r="D344" t="n">
-        <v>14.44118844499799</v>
+        <v>14.44118937691309</v>
       </c>
       <c r="E344" t="n">
-        <v>14.5856972217251</v>
+        <v>14.58569816296561</v>
       </c>
       <c r="F344" t="n">
         <v>3964800</v>
@@ -7392,16 +7392,16 @@
         <v>44762</v>
       </c>
       <c r="B349" t="n">
-        <v>14.82654571533203</v>
+        <v>14.82654476165771</v>
       </c>
       <c r="C349" t="n">
-        <v>15.10592827517219</v>
+        <v>15.10592730352741</v>
       </c>
       <c r="D349" t="n">
-        <v>14.57606454616261</v>
+        <v>14.57606360859976</v>
       </c>
       <c r="E349" t="n">
-        <v>14.89398259981663</v>
+        <v>14.89398164180463</v>
       </c>
       <c r="F349" t="n">
         <v>5599700</v>
@@ -7652,16 +7652,16 @@
         <v>44781</v>
       </c>
       <c r="B362" t="n">
-        <v>16.68588256835938</v>
+        <v>16.68588447570801</v>
       </c>
       <c r="C362" t="n">
-        <v>16.88819503663362</v>
+        <v>16.88819696710841</v>
       </c>
       <c r="D362" t="n">
-        <v>16.26199126520336</v>
+        <v>16.26199312409735</v>
       </c>
       <c r="E362" t="n">
-        <v>16.53174061039666</v>
+        <v>16.53174250012546</v>
       </c>
       <c r="F362" t="n">
         <v>10381400</v>
@@ -7692,16 +7692,16 @@
         <v>44783</v>
       </c>
       <c r="B364" t="n">
-        <v>16.89782905578613</v>
+        <v>16.89783096313477</v>
       </c>
       <c r="C364" t="n">
-        <v>17.20611297019896</v>
+        <v>17.20611491234526</v>
       </c>
       <c r="D364" t="n">
-        <v>16.73405299656468</v>
+        <v>16.73405488542704</v>
       </c>
       <c r="E364" t="n">
-        <v>17.16757656213882</v>
+        <v>17.1675784999353</v>
       </c>
       <c r="F364" t="n">
         <v>6533000</v>
@@ -7812,16 +7812,16 @@
         <v>44791</v>
       </c>
       <c r="B370" t="n">
-        <v>17.45659446716309</v>
+        <v>17.45659637451172</v>
       </c>
       <c r="C370" t="n">
-        <v>17.59146822309866</v>
+        <v>17.59147014518392</v>
       </c>
       <c r="D370" t="n">
-        <v>17.29281840459113</v>
+        <v>17.2928202940452</v>
       </c>
       <c r="E370" t="n">
-        <v>17.34098707813466</v>
+        <v>17.34098897285176</v>
       </c>
       <c r="F370" t="n">
         <v>13968800</v>
@@ -7832,16 +7832,16 @@
         <v>44792</v>
       </c>
       <c r="B371" t="n">
-        <v>17.12904357910156</v>
+        <v>17.12904167175293</v>
       </c>
       <c r="C371" t="n">
-        <v>17.57220128776223</v>
+        <v>17.57219933106722</v>
       </c>
       <c r="D371" t="n">
-        <v>17.07123896165407</v>
+        <v>17.07123706074208</v>
       </c>
       <c r="E371" t="n">
-        <v>17.45659572790173</v>
+        <v>17.4565937840796</v>
       </c>
       <c r="F371" t="n">
         <v>7571900</v>
@@ -7872,16 +7872,16 @@
         <v>44796</v>
       </c>
       <c r="B373" t="n">
-        <v>17.20611190795898</v>
+        <v>17.20611381530762</v>
       </c>
       <c r="C373" t="n">
-        <v>17.7937773944593</v>
+        <v>17.7937793669524</v>
       </c>
       <c r="D373" t="n">
-        <v>17.10977273127332</v>
+        <v>17.10977462794247</v>
       </c>
       <c r="E373" t="n">
-        <v>17.49512760049901</v>
+        <v>17.49512953988589</v>
       </c>
       <c r="F373" t="n">
         <v>12142000</v>
@@ -7952,16 +7952,16 @@
         <v>44802</v>
       </c>
       <c r="B377" t="n">
-        <v>17.68780899047852</v>
+        <v>17.68780708312988</v>
       </c>
       <c r="C377" t="n">
-        <v>17.98645883571042</v>
+        <v>17.98645689615716</v>
       </c>
       <c r="D377" t="n">
-        <v>17.19648075879664</v>
+        <v>17.19647890442993</v>
       </c>
       <c r="E377" t="n">
-        <v>17.29281995202162</v>
+        <v>17.29281808726627</v>
       </c>
       <c r="F377" t="n">
         <v>7263100</v>
@@ -7992,16 +7992,16 @@
         <v>44804</v>
       </c>
       <c r="B379" t="n">
-        <v>17.71670913696289</v>
+        <v>17.71671104431152</v>
       </c>
       <c r="C379" t="n">
-        <v>17.98645850553768</v>
+        <v>17.98646044192704</v>
       </c>
       <c r="D379" t="n">
-        <v>17.51439848866973</v>
+        <v>17.51440037423797</v>
       </c>
       <c r="E379" t="n">
-        <v>17.74561144565502</v>
+        <v>17.74561335611522</v>
       </c>
       <c r="F379" t="n">
         <v>9759800</v>
@@ -8032,16 +8032,16 @@
         <v>44806</v>
       </c>
       <c r="B381" t="n">
-        <v>18.20803642272949</v>
+        <v>18.20803451538086</v>
       </c>
       <c r="C381" t="n">
-        <v>18.54522265671872</v>
+        <v>18.54522071404877</v>
       </c>
       <c r="D381" t="n">
-        <v>17.95755527283799</v>
+        <v>17.95755339172804</v>
       </c>
       <c r="E381" t="n">
-        <v>18.20803642272949</v>
+        <v>18.20803451538086</v>
       </c>
       <c r="F381" t="n">
         <v>12423600</v>
@@ -8152,16 +8152,16 @@
         <v>44817</v>
       </c>
       <c r="B387" t="n">
-        <v>17.48549652099609</v>
+        <v>17.48549461364746</v>
       </c>
       <c r="C387" t="n">
-        <v>17.84195098508192</v>
+        <v>17.84194903885061</v>
       </c>
       <c r="D387" t="n">
-        <v>17.32172044358108</v>
+        <v>17.32171855409743</v>
       </c>
       <c r="E387" t="n">
-        <v>17.64927259841111</v>
+        <v>17.64927067319749</v>
       </c>
       <c r="F387" t="n">
         <v>10161300</v>
@@ -8172,16 +8172,16 @@
         <v>44818</v>
       </c>
       <c r="B388" t="n">
-        <v>17.70707511901855</v>
+        <v>17.70707702636719</v>
       </c>
       <c r="C388" t="n">
-        <v>17.8708511940252</v>
+        <v>17.87085311901526</v>
       </c>
       <c r="D388" t="n">
-        <v>17.36989070357892</v>
+        <v>17.36989257460714</v>
       </c>
       <c r="E388" t="n">
-        <v>17.44696168961044</v>
+        <v>17.4469635689405</v>
       </c>
       <c r="F388" t="n">
         <v>7347400</v>
@@ -8212,16 +8212,16 @@
         <v>44820</v>
       </c>
       <c r="B390" t="n">
-        <v>17.24464797973633</v>
+        <v>17.24464988708496</v>
       </c>
       <c r="C390" t="n">
-        <v>17.62037061781912</v>
+        <v>17.62037256672464</v>
       </c>
       <c r="D390" t="n">
-        <v>17.06160371182508</v>
+        <v>17.06160559892805</v>
       </c>
       <c r="E390" t="n">
-        <v>17.49512912595248</v>
+        <v>17.49513106100564</v>
       </c>
       <c r="F390" t="n">
         <v>10140200</v>
@@ -8232,16 +8232,16 @@
         <v>44823</v>
       </c>
       <c r="B391" t="n">
-        <v>17.46623039245605</v>
+        <v>17.46622848510742</v>
       </c>
       <c r="C391" t="n">
-        <v>17.58183780571365</v>
+        <v>17.58183588574045</v>
       </c>
       <c r="D391" t="n">
-        <v>17.14831230289454</v>
+        <v>17.14831043026322</v>
       </c>
       <c r="E391" t="n">
-        <v>17.14831230289454</v>
+        <v>17.14831043026322</v>
       </c>
       <c r="F391" t="n">
         <v>7719100</v>
@@ -8332,16 +8332,16 @@
         <v>44830</v>
       </c>
       <c r="B396" t="n">
-        <v>17.09050559997559</v>
+        <v>17.09050750732422</v>
       </c>
       <c r="C396" t="n">
-        <v>17.20611298675014</v>
+        <v>17.20611490700088</v>
       </c>
       <c r="D396" t="n">
-        <v>16.71478480861316</v>
+        <v>16.7147866740303</v>
       </c>
       <c r="E396" t="n">
-        <v>16.89782907204076</v>
+        <v>16.89783095788615</v>
       </c>
       <c r="F396" t="n">
         <v>7980700</v>
@@ -8352,16 +8352,16 @@
         <v>44831</v>
       </c>
       <c r="B397" t="n">
-        <v>17.12904357910156</v>
+        <v>17.12904167175293</v>
       </c>
       <c r="C397" t="n">
-        <v>17.49513030201615</v>
+        <v>17.49512835390313</v>
       </c>
       <c r="D397" t="n">
-        <v>16.86892831313957</v>
+        <v>16.86892643475522</v>
       </c>
       <c r="E397" t="n">
-        <v>17.25428324186998</v>
+        <v>17.2542813205757</v>
       </c>
       <c r="F397" t="n">
         <v>9260100</v>
@@ -8432,16 +8432,16 @@
         <v>44837</v>
       </c>
       <c r="B401" t="n">
-        <v>17.75524520874023</v>
+        <v>17.75524711608887</v>
       </c>
       <c r="C401" t="n">
-        <v>17.81304798750098</v>
+        <v>17.81304990105905</v>
       </c>
       <c r="D401" t="n">
-        <v>16.96526716144702</v>
+        <v>16.96526898393264</v>
       </c>
       <c r="E401" t="n">
-        <v>17.24464879005494</v>
+        <v>17.244650642553</v>
       </c>
       <c r="F401" t="n">
         <v>18011200</v>
@@ -8472,16 +8472,16 @@
         <v>44839</v>
       </c>
       <c r="B403" t="n">
-        <v>17.45659446716309</v>
+        <v>17.45659637451172</v>
       </c>
       <c r="C403" t="n">
-        <v>17.74561018345848</v>
+        <v>17.74561212238566</v>
       </c>
       <c r="D403" t="n">
-        <v>17.14830870892632</v>
+        <v>17.14831058259092</v>
       </c>
       <c r="E403" t="n">
-        <v>17.4276921605267</v>
+        <v>17.4276940647174</v>
       </c>
       <c r="F403" t="n">
         <v>8852300</v>
@@ -8492,16 +8492,16 @@
         <v>44840</v>
       </c>
       <c r="B404" t="n">
-        <v>17.44696044921875</v>
+        <v>17.44696235656738</v>
       </c>
       <c r="C404" t="n">
-        <v>17.6396369818406</v>
+        <v>17.63963891025314</v>
       </c>
       <c r="D404" t="n">
-        <v>17.30245075285597</v>
+        <v>17.30245264440641</v>
       </c>
       <c r="E404" t="n">
-        <v>17.63000287958194</v>
+        <v>17.63000480694126</v>
       </c>
       <c r="F404" t="n">
         <v>6691000</v>
@@ -8652,16 +8652,16 @@
         <v>44853</v>
       </c>
       <c r="B412" t="n">
-        <v>17.67817687988281</v>
+        <v>17.67817497253418</v>
       </c>
       <c r="C412" t="n">
-        <v>17.97682675877506</v>
+        <v>17.97682481920425</v>
       </c>
       <c r="D412" t="n">
-        <v>17.28318779690735</v>
+        <v>17.2831859321752</v>
       </c>
       <c r="E412" t="n">
-        <v>17.4758643675563</v>
+        <v>17.47586248203574</v>
       </c>
       <c r="F412" t="n">
         <v>27062400</v>
@@ -8692,16 +8692,16 @@
         <v>44855</v>
       </c>
       <c r="B414" t="n">
-        <v>17.91902160644531</v>
+        <v>17.91902351379395</v>
       </c>
       <c r="C414" t="n">
-        <v>18.25620785747724</v>
+        <v>18.25620980071688</v>
       </c>
       <c r="D414" t="n">
-        <v>17.34098829575019</v>
+        <v>17.34099014157141</v>
       </c>
       <c r="E414" t="n">
-        <v>17.53366667848764</v>
+        <v>17.53366854481807</v>
       </c>
       <c r="F414" t="n">
         <v>27105700</v>
@@ -8712,16 +8712,16 @@
         <v>44858</v>
       </c>
       <c r="B415" t="n">
-        <v>18.00572776794434</v>
+        <v>18.0057258605957</v>
       </c>
       <c r="C415" t="n">
-        <v>18.36218040847837</v>
+        <v>18.36217846337067</v>
       </c>
       <c r="D415" t="n">
-        <v>17.54329998932035</v>
+        <v>17.54329813095674</v>
       </c>
       <c r="E415" t="n">
-        <v>17.91902267429717</v>
+        <v>17.91902077613322</v>
       </c>
       <c r="F415" t="n">
         <v>16227000</v>
@@ -8732,16 +8732,16 @@
         <v>44859</v>
       </c>
       <c r="B416" t="n">
-        <v>17.04233741760254</v>
+        <v>17.04233932495117</v>
       </c>
       <c r="C416" t="n">
-        <v>18.00572559754023</v>
+        <v>18.00572761270958</v>
       </c>
       <c r="D416" t="n">
-        <v>16.80149037261812</v>
+        <v>16.80149225301157</v>
       </c>
       <c r="E416" t="n">
-        <v>18.00572559754023</v>
+        <v>18.00572761270958</v>
       </c>
       <c r="F416" t="n">
         <v>27810400</v>
@@ -8772,16 +8772,16 @@
         <v>44861</v>
       </c>
       <c r="B418" t="n">
-        <v>17.47586250305176</v>
+        <v>17.47586059570312</v>
       </c>
       <c r="C418" t="n">
-        <v>17.74561187820164</v>
+        <v>17.74560994141206</v>
       </c>
       <c r="D418" t="n">
-        <v>15.9922455335206</v>
+        <v>15.99224378809673</v>
       </c>
       <c r="E418" t="n">
-        <v>16.13675340546911</v>
+        <v>16.13675164427337</v>
       </c>
       <c r="F418" t="n">
         <v>30122400</v>
@@ -8792,16 +8792,16 @@
         <v>44862</v>
       </c>
       <c r="B419" t="n">
-        <v>18.12133026123047</v>
+        <v>18.1213321685791</v>
       </c>
       <c r="C419" t="n">
-        <v>18.21766944200201</v>
+        <v>18.21767135949075</v>
       </c>
       <c r="D419" t="n">
-        <v>17.27354951297842</v>
+        <v>17.27355133109445</v>
       </c>
       <c r="E419" t="n">
-        <v>17.40842326354835</v>
+        <v>17.40842509586043</v>
       </c>
       <c r="F419" t="n">
         <v>12193800</v>
@@ -8852,16 +8852,16 @@
         <v>44868</v>
       </c>
       <c r="B422" t="n">
-        <v>19.62422180175781</v>
+        <v>19.62421989440918</v>
       </c>
       <c r="C422" t="n">
-        <v>19.74946148068863</v>
+        <v>19.74945956116751</v>
       </c>
       <c r="D422" t="n">
-        <v>18.69936801593355</v>
+        <v>18.69936619847478</v>
       </c>
       <c r="E422" t="n">
-        <v>18.69936801593355</v>
+        <v>18.69936619847478</v>
       </c>
       <c r="F422" t="n">
         <v>9732300</v>
@@ -8892,16 +8892,16 @@
         <v>44872</v>
       </c>
       <c r="B424" t="n">
-        <v>19.51824760437012</v>
+        <v>19.51824569702148</v>
       </c>
       <c r="C424" t="n">
-        <v>19.94213898012385</v>
+        <v>19.942137031352</v>
       </c>
       <c r="D424" t="n">
-        <v>19.14252674717783</v>
+        <v>19.14252487654513</v>
       </c>
       <c r="E424" t="n">
-        <v>19.69165779615653</v>
+        <v>19.69165587186202</v>
       </c>
       <c r="F424" t="n">
         <v>17754600</v>
@@ -8972,16 +8972,16 @@
         <v>44876</v>
       </c>
       <c r="B428" t="n">
-        <v>18.64156341552734</v>
+        <v>18.64156532287598</v>
       </c>
       <c r="C428" t="n">
-        <v>18.96911557474207</v>
+        <v>18.96911751560485</v>
       </c>
       <c r="D428" t="n">
-        <v>18.03462777565176</v>
+        <v>18.03462962090057</v>
       </c>
       <c r="E428" t="n">
-        <v>18.88241048333127</v>
+        <v>18.88241241532265</v>
       </c>
       <c r="F428" t="n">
         <v>19344200</v>
@@ -9112,16 +9112,16 @@
         <v>44888</v>
       </c>
       <c r="B435" t="n">
-        <v>18.64156341552734</v>
+        <v>18.64156532287598</v>
       </c>
       <c r="C435" t="n">
-        <v>19.14252575756366</v>
+        <v>19.14252771616925</v>
       </c>
       <c r="D435" t="n">
-        <v>18.46815323270575</v>
+        <v>18.46815512231158</v>
       </c>
       <c r="E435" t="n">
-        <v>18.69936619729544</v>
+        <v>18.69936811055828</v>
       </c>
       <c r="F435" t="n">
         <v>10423000</v>
@@ -9312,16 +9312,16 @@
         <v>44902</v>
       </c>
       <c r="B445" t="n">
-        <v>19.36410522460938</v>
+        <v>19.36410331726074</v>
       </c>
       <c r="C445" t="n">
-        <v>19.48934489527705</v>
+        <v>19.48934297559241</v>
       </c>
       <c r="D445" t="n">
-        <v>18.82460829035904</v>
+        <v>18.82460643615043</v>
       </c>
       <c r="E445" t="n">
-        <v>19.17142682933272</v>
+        <v>19.17142494096275</v>
       </c>
       <c r="F445" t="n">
         <v>7439200</v>
@@ -9412,16 +9412,16 @@
         <v>44909</v>
       </c>
       <c r="B450" t="n">
-        <v>18.3718147277832</v>
+        <v>18.37181282043457</v>
       </c>
       <c r="C450" t="n">
-        <v>18.46815392602494</v>
+        <v>18.46815200867444</v>
       </c>
       <c r="D450" t="n">
-        <v>17.64927349724626</v>
+        <v>17.64927166491134</v>
       </c>
       <c r="E450" t="n">
-        <v>17.86122010088155</v>
+        <v>17.86121824654248</v>
       </c>
       <c r="F450" t="n">
         <v>10673700</v>
@@ -9612,16 +9612,16 @@
         <v>44923</v>
       </c>
       <c r="B460" t="n">
-        <v>18.71863555908203</v>
+        <v>18.7186336517334</v>
       </c>
       <c r="C460" t="n">
-        <v>18.94984853794273</v>
+        <v>18.94984660703449</v>
       </c>
       <c r="D460" t="n">
-        <v>18.26584186765209</v>
+        <v>18.26584000644119</v>
       </c>
       <c r="E460" t="n">
-        <v>18.68973324765541</v>
+        <v>18.6897313432518</v>
       </c>
       <c r="F460" t="n">
         <v>8329700</v>
@@ -27465,6 +27465,26 @@
       </c>
       <c r="F1352" t="n">
         <v>5647400</v>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B1353" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="C1353" t="n">
+        <v>8.43</v>
+      </c>
+      <c r="D1353" t="n">
+        <v>8.18</v>
+      </c>
+      <c r="E1353" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="F1353" t="n">
+        <v>6610600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-12 22:26 UTC
</commit_message>
<xml_diff>
--- a/database/ASAI3.xlsx
+++ b/database/ASAI3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1362"/>
+  <dimension ref="A1:F1361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -552,16 +552,16 @@
         <v>44263</v>
       </c>
       <c r="B7" t="n">
-        <v>13.48508644104004</v>
+        <v>13.48508548736572</v>
       </c>
       <c r="C7" t="n">
-        <v>14.2978757345337</v>
+        <v>14.29787472337838</v>
       </c>
       <c r="D7" t="n">
-        <v>13.05210579563423</v>
+        <v>13.05210487258059</v>
       </c>
       <c r="E7" t="n">
-        <v>14.21051986319279</v>
+        <v>14.21051885821534</v>
       </c>
       <c r="F7" t="n">
         <v>12366000</v>
@@ -572,16 +572,16 @@
         <v>44264</v>
       </c>
       <c r="B8" t="n">
-        <v>13.44520568847656</v>
+        <v>13.44520664215088</v>
       </c>
       <c r="C8" t="n">
-        <v>13.44520568847656</v>
+        <v>13.44520664215088</v>
       </c>
       <c r="D8" t="n">
-        <v>13.0103252694391</v>
+        <v>13.01032619226716</v>
       </c>
       <c r="E8" t="n">
-        <v>13.29138370087542</v>
+        <v>13.29138464363907</v>
       </c>
       <c r="F8" t="n">
         <v>10167000</v>
@@ -592,16 +592,16 @@
         <v>44265</v>
       </c>
       <c r="B9" t="n">
-        <v>13.48318672180176</v>
+        <v>13.48318767547607</v>
       </c>
       <c r="C9" t="n">
-        <v>13.95794682401684</v>
+        <v>13.95794781127124</v>
       </c>
       <c r="D9" t="n">
-        <v>13.23631125132199</v>
+        <v>13.23631218753465</v>
       </c>
       <c r="E9" t="n">
-        <v>13.4850856245696</v>
+        <v>13.48508657837822</v>
       </c>
       <c r="F9" t="n">
         <v>15699500</v>
@@ -652,16 +652,16 @@
         <v>44270</v>
       </c>
       <c r="B12" t="n">
-        <v>13.83451080322266</v>
+        <v>13.83450794219971</v>
       </c>
       <c r="C12" t="n">
-        <v>14.01681907452333</v>
+        <v>14.01681617579842</v>
       </c>
       <c r="D12" t="n">
-        <v>13.62181827280511</v>
+        <v>13.62181545576768</v>
       </c>
       <c r="E12" t="n">
-        <v>13.81931867366422</v>
+        <v>13.81931581578305</v>
       </c>
       <c r="F12" t="n">
         <v>11593000</v>
@@ -672,16 +672,16 @@
         <v>44271</v>
       </c>
       <c r="B13" t="n">
-        <v>13.58763408660889</v>
+        <v>13.5876350402832</v>
       </c>
       <c r="C13" t="n">
-        <v>13.91047018507921</v>
+        <v>13.9104711614124</v>
       </c>
       <c r="D13" t="n">
-        <v>13.49458060971476</v>
+        <v>13.49458155685794</v>
       </c>
       <c r="E13" t="n">
-        <v>13.84400406267841</v>
+        <v>13.84400503434655</v>
       </c>
       <c r="F13" t="n">
         <v>7789500</v>
@@ -732,16 +732,16 @@
         <v>44274</v>
       </c>
       <c r="B16" t="n">
-        <v>13.54775333404541</v>
+        <v>13.54775524139404</v>
       </c>
       <c r="C16" t="n">
-        <v>14.03580663921036</v>
+        <v>14.03580861527059</v>
       </c>
       <c r="D16" t="n">
-        <v>13.46419618282161</v>
+        <v>13.46419807840647</v>
       </c>
       <c r="E16" t="n">
-        <v>13.95414839066896</v>
+        <v>13.95415035523277</v>
       </c>
       <c r="F16" t="n">
         <v>14098000</v>
@@ -812,16 +812,16 @@
         <v>44280</v>
       </c>
       <c r="B20" t="n">
-        <v>13.64840221405029</v>
+        <v>13.64840316772461</v>
       </c>
       <c r="C20" t="n">
-        <v>13.67308975961416</v>
+        <v>13.67309071501351</v>
       </c>
       <c r="D20" t="n">
-        <v>12.83941172946964</v>
+        <v>12.83941262661621</v>
       </c>
       <c r="E20" t="n">
-        <v>12.91347436616125</v>
+        <v>12.9134752684829</v>
       </c>
       <c r="F20" t="n">
         <v>6602000</v>
@@ -832,16 +832,16 @@
         <v>44281</v>
       </c>
       <c r="B21" t="n">
-        <v>13.80602359771729</v>
+        <v>13.8060245513916</v>
       </c>
       <c r="C21" t="n">
-        <v>14.12696170612194</v>
+        <v>14.1269626819656</v>
       </c>
       <c r="D21" t="n">
-        <v>13.48888420034324</v>
+        <v>13.48888513211062</v>
       </c>
       <c r="E21" t="n">
-        <v>13.54965361596974</v>
+        <v>13.54965455193487</v>
       </c>
       <c r="F21" t="n">
         <v>4396500</v>
@@ -852,16 +852,16 @@
         <v>44284</v>
       </c>
       <c r="B22" t="n">
-        <v>13.95794677734375</v>
+        <v>13.95794773101807</v>
       </c>
       <c r="C22" t="n">
-        <v>13.95794677734375</v>
+        <v>13.95794773101807</v>
       </c>
       <c r="D22" t="n">
-        <v>13.4869853877722</v>
+        <v>13.48698630926816</v>
       </c>
       <c r="E22" t="n">
-        <v>13.7148700187455</v>
+        <v>13.71487095581164</v>
       </c>
       <c r="F22" t="n">
         <v>6557000</v>
@@ -872,16 +872,16 @@
         <v>44285</v>
       </c>
       <c r="B23" t="n">
-        <v>13.95794677734375</v>
+        <v>13.95794773101807</v>
       </c>
       <c r="C23" t="n">
-        <v>14.08138451217088</v>
+        <v>14.08138547427906</v>
       </c>
       <c r="D23" t="n">
-        <v>13.76804291819933</v>
+        <v>13.7680438588985</v>
       </c>
       <c r="E23" t="n">
-        <v>13.76804291819933</v>
+        <v>13.7680438588985</v>
       </c>
       <c r="F23" t="n">
         <v>8433000</v>
@@ -912,16 +912,16 @@
         <v>44287</v>
       </c>
       <c r="B25" t="n">
-        <v>14.2541971206665</v>
+        <v>14.25419807434082</v>
       </c>
       <c r="C25" t="n">
-        <v>14.40232240017016</v>
+        <v>14.40232336375477</v>
       </c>
       <c r="D25" t="n">
-        <v>14.02631249321458</v>
+        <v>14.02631343164232</v>
       </c>
       <c r="E25" t="n">
-        <v>14.09087971377266</v>
+        <v>14.09088065652025</v>
       </c>
       <c r="F25" t="n">
         <v>9940000</v>
@@ -932,16 +932,16 @@
         <v>44291</v>
       </c>
       <c r="B26" t="n">
-        <v>14.71756362915039</v>
+        <v>14.71756267547607</v>
       </c>
       <c r="C26" t="n">
-        <v>14.88657865823869</v>
+        <v>14.88657769361247</v>
       </c>
       <c r="D26" t="n">
-        <v>14.29977512456389</v>
+        <v>14.2997741979616</v>
       </c>
       <c r="E26" t="n">
-        <v>14.29977512456389</v>
+        <v>14.2997741979616</v>
       </c>
       <c r="F26" t="n">
         <v>6073500</v>
@@ -952,16 +952,16 @@
         <v>44292</v>
       </c>
       <c r="B27" t="n">
-        <v>14.58652877807617</v>
+        <v>14.58652973175049</v>
       </c>
       <c r="C27" t="n">
-        <v>14.72135992027025</v>
+        <v>14.72136088275989</v>
       </c>
       <c r="D27" t="n">
-        <v>14.52765826882265</v>
+        <v>14.52765921864798</v>
       </c>
       <c r="E27" t="n">
-        <v>14.71756211500646</v>
+        <v>14.7175630772478</v>
       </c>
       <c r="F27" t="n">
         <v>5821500</v>
@@ -992,16 +992,16 @@
         <v>44294</v>
       </c>
       <c r="B29" t="n">
-        <v>14.70237064361572</v>
+        <v>14.70237255096436</v>
       </c>
       <c r="C29" t="n">
-        <v>14.74035141454506</v>
+        <v>14.74035332682097</v>
       </c>
       <c r="D29" t="n">
-        <v>14.26559132516181</v>
+        <v>14.26559317584676</v>
       </c>
       <c r="E29" t="n">
-        <v>14.4327065361443</v>
+        <v>14.43270840850923</v>
       </c>
       <c r="F29" t="n">
         <v>6395000</v>
@@ -1012,16 +1012,16 @@
         <v>44295</v>
       </c>
       <c r="B30" t="n">
-        <v>14.71756362915039</v>
+        <v>14.71756267547607</v>
       </c>
       <c r="C30" t="n">
-        <v>14.73655446848903</v>
+        <v>14.73655351358414</v>
       </c>
       <c r="D30" t="n">
-        <v>14.40801982998176</v>
+        <v>14.40801889636538</v>
       </c>
       <c r="E30" t="n">
-        <v>14.63210666319261</v>
+        <v>14.63210571505577</v>
       </c>
       <c r="F30" t="n">
         <v>7012500</v>
@@ -1072,16 +1072,16 @@
         <v>44300</v>
       </c>
       <c r="B33" t="n">
-        <v>14.93785095214844</v>
+        <v>14.93785381317139</v>
       </c>
       <c r="C33" t="n">
-        <v>14.94544656259071</v>
+        <v>14.94544942506844</v>
       </c>
       <c r="D33" t="n">
-        <v>14.62260957493718</v>
+        <v>14.62261237558245</v>
       </c>
       <c r="E33" t="n">
-        <v>14.65109583069458</v>
+        <v>14.65109863679578</v>
       </c>
       <c r="F33" t="n">
         <v>5841000</v>
@@ -1092,16 +1092,16 @@
         <v>44301</v>
       </c>
       <c r="B34" t="n">
-        <v>15.18662643432617</v>
+        <v>15.18662738800049</v>
       </c>
       <c r="C34" t="n">
-        <v>15.2037165590924</v>
+        <v>15.20371751383992</v>
       </c>
       <c r="D34" t="n">
-        <v>14.84100077857334</v>
+        <v>14.84100171054341</v>
       </c>
       <c r="E34" t="n">
-        <v>14.84100077857334</v>
+        <v>14.84100171054341</v>
       </c>
       <c r="F34" t="n">
         <v>11554500</v>
@@ -1132,16 +1132,16 @@
         <v>44305</v>
       </c>
       <c r="B36" t="n">
-        <v>15.28727436065674</v>
+        <v>15.28727531433105</v>
       </c>
       <c r="C36" t="n">
-        <v>15.50756336269031</v>
+        <v>15.50756433010704</v>
       </c>
       <c r="D36" t="n">
-        <v>15.00431704491931</v>
+        <v>15.00431798094175</v>
       </c>
       <c r="E36" t="n">
-        <v>15.14484579871793</v>
+        <v>15.14484674350704</v>
       </c>
       <c r="F36" t="n">
         <v>5017000</v>
@@ -1152,16 +1152,16 @@
         <v>44306</v>
       </c>
       <c r="B37" t="n">
-        <v>15.47718048095703</v>
+        <v>15.47718143463135</v>
       </c>
       <c r="C37" t="n">
-        <v>15.65569185126732</v>
+        <v>15.65569281594117</v>
       </c>
       <c r="D37" t="n">
-        <v>15.06698845640197</v>
+        <v>15.06698938480104</v>
       </c>
       <c r="E37" t="n">
-        <v>15.35944125083699</v>
+        <v>15.35944219725644</v>
       </c>
       <c r="F37" t="n">
         <v>6029000</v>
@@ -1172,16 +1172,16 @@
         <v>44308</v>
       </c>
       <c r="B38" t="n">
-        <v>15.27967834472656</v>
+        <v>15.27967929840088</v>
       </c>
       <c r="C38" t="n">
-        <v>15.75254045321392</v>
+        <v>15.75254143640172</v>
       </c>
       <c r="D38" t="n">
-        <v>15.19422319187483</v>
+        <v>15.1942241402155</v>
       </c>
       <c r="E38" t="n">
-        <v>15.50376517258819</v>
+        <v>15.50376614024878</v>
       </c>
       <c r="F38" t="n">
         <v>8470500</v>
@@ -1192,16 +1192,16 @@
         <v>44309</v>
       </c>
       <c r="B39" t="n">
-        <v>15.41261386871338</v>
+        <v>15.41261196136475</v>
       </c>
       <c r="C39" t="n">
-        <v>15.53795051954675</v>
+        <v>15.53794859668741</v>
       </c>
       <c r="D39" t="n">
-        <v>15.21891127804373</v>
+        <v>15.21890939466627</v>
       </c>
       <c r="E39" t="n">
-        <v>15.45819116193756</v>
+        <v>15.45818924894863</v>
       </c>
       <c r="F39" t="n">
         <v>4653000</v>
@@ -1212,16 +1212,16 @@
         <v>44312</v>
       </c>
       <c r="B40" t="n">
-        <v>15.2606897354126</v>
+        <v>15.26068878173828</v>
       </c>
       <c r="C40" t="n">
-        <v>15.51705882313055</v>
+        <v>15.51705785343516</v>
       </c>
       <c r="D40" t="n">
-        <v>15.16573734944818</v>
+        <v>15.16573640170765</v>
       </c>
       <c r="E40" t="n">
-        <v>15.48477656941952</v>
+        <v>15.48477560174152</v>
       </c>
       <c r="F40" t="n">
         <v>3662000</v>
@@ -1252,16 +1252,16 @@
         <v>44314</v>
       </c>
       <c r="B42" t="n">
-        <v>15.18852519989014</v>
+        <v>15.18852615356445</v>
       </c>
       <c r="C42" t="n">
-        <v>15.35564131800169</v>
+        <v>15.35564228216909</v>
       </c>
       <c r="D42" t="n">
-        <v>15.04799553112973</v>
+        <v>15.04799647598031</v>
       </c>
       <c r="E42" t="n">
-        <v>15.14864552586341</v>
+        <v>15.14864647703371</v>
       </c>
       <c r="F42" t="n">
         <v>5371500</v>
@@ -1312,16 +1312,16 @@
         <v>44319</v>
       </c>
       <c r="B45" t="n">
-        <v>15.53295993804932</v>
+        <v>15.53295803070068</v>
       </c>
       <c r="C45" t="n">
-        <v>15.67023330010677</v>
+        <v>15.67023137590184</v>
       </c>
       <c r="D45" t="n">
-        <v>15.29463663895672</v>
+        <v>15.29463476087267</v>
       </c>
       <c r="E45" t="n">
-        <v>15.4433505085054</v>
+        <v>15.44334861216023</v>
       </c>
       <c r="F45" t="n">
         <v>8474000</v>
@@ -1332,16 +1332,16 @@
         <v>44320</v>
       </c>
       <c r="B46" t="n">
-        <v>15.72933864593506</v>
+        <v>15.72933769226074</v>
       </c>
       <c r="C46" t="n">
-        <v>15.74840494734345</v>
+        <v>15.74840399251314</v>
       </c>
       <c r="D46" t="n">
-        <v>15.35946039896755</v>
+        <v>15.35945946771906</v>
       </c>
       <c r="E46" t="n">
-        <v>15.63400895715566</v>
+        <v>15.63400800926121</v>
       </c>
       <c r="F46" t="n">
         <v>9407500</v>
@@ -1352,16 +1352,16 @@
         <v>44321</v>
       </c>
       <c r="B47" t="n">
-        <v>16.32228469848633</v>
+        <v>16.32228660583496</v>
       </c>
       <c r="C47" t="n">
-        <v>16.58730007183393</v>
+        <v>16.58730201015107</v>
       </c>
       <c r="D47" t="n">
-        <v>16.01532383109572</v>
+        <v>16.01532570257429</v>
       </c>
       <c r="E47" t="n">
-        <v>16.08396141636727</v>
+        <v>16.08396329586652</v>
       </c>
       <c r="F47" t="n">
         <v>17262500</v>
@@ -1412,16 +1412,16 @@
         <v>44326</v>
       </c>
       <c r="B50" t="n">
-        <v>16.81418418884277</v>
+        <v>16.81418609619141</v>
       </c>
       <c r="C50" t="n">
-        <v>17.01628222452739</v>
+        <v>17.0162841548014</v>
       </c>
       <c r="D50" t="n">
-        <v>16.55298171903851</v>
+        <v>16.55298359675715</v>
       </c>
       <c r="E50" t="n">
-        <v>16.97052383564365</v>
+        <v>16.97052576072697</v>
       </c>
       <c r="F50" t="n">
         <v>7669500</v>
@@ -1452,16 +1452,16 @@
         <v>44328</v>
       </c>
       <c r="B52" t="n">
-        <v>16.12590408325195</v>
+        <v>16.12590599060059</v>
       </c>
       <c r="C52" t="n">
-        <v>16.57776401598027</v>
+        <v>16.57776597677424</v>
       </c>
       <c r="D52" t="n">
-        <v>16.04201310987353</v>
+        <v>16.04201500729966</v>
       </c>
       <c r="E52" t="n">
-        <v>16.49006196539431</v>
+        <v>16.49006391581501</v>
       </c>
       <c r="F52" t="n">
         <v>6728500</v>
@@ -1472,16 +1472,16 @@
         <v>44329</v>
       </c>
       <c r="B53" t="n">
-        <v>16.43286895751953</v>
+        <v>16.43287086486816</v>
       </c>
       <c r="C53" t="n">
-        <v>16.51866367244025</v>
+        <v>16.518665589747</v>
       </c>
       <c r="D53" t="n">
-        <v>16.12781360716679</v>
+        <v>16.12781547910792</v>
       </c>
       <c r="E53" t="n">
-        <v>16.17547935796994</v>
+        <v>16.17548123544359</v>
       </c>
       <c r="F53" t="n">
         <v>6595000</v>
@@ -1492,16 +1492,16 @@
         <v>44330</v>
       </c>
       <c r="B54" t="n">
-        <v>16.52628898620605</v>
+        <v>16.52629089355469</v>
       </c>
       <c r="C54" t="n">
-        <v>16.66356232925931</v>
+        <v>16.66356425245107</v>
       </c>
       <c r="D54" t="n">
-        <v>16.13734451407442</v>
+        <v>16.13734637653381</v>
       </c>
       <c r="E54" t="n">
-        <v>16.54726082268666</v>
+        <v>16.54726273245572</v>
       </c>
       <c r="F54" t="n">
         <v>5923000</v>
@@ -1532,16 +1532,16 @@
         <v>44334</v>
       </c>
       <c r="B56" t="n">
-        <v>16.06108474731445</v>
+        <v>16.06108283996582</v>
       </c>
       <c r="C56" t="n">
-        <v>16.39092486167181</v>
+        <v>16.39092291515271</v>
       </c>
       <c r="D56" t="n">
-        <v>15.88758612704159</v>
+        <v>15.88758424029694</v>
       </c>
       <c r="E56" t="n">
-        <v>16.34897936103174</v>
+        <v>16.34897741949393</v>
       </c>
       <c r="F56" t="n">
         <v>6527500</v>
@@ -1552,16 +1552,16 @@
         <v>44335</v>
       </c>
       <c r="B57" t="n">
-        <v>15.82848262786865</v>
+        <v>15.82848072052002</v>
       </c>
       <c r="C57" t="n">
-        <v>16.36804664114567</v>
+        <v>16.36804466877901</v>
       </c>
       <c r="D57" t="n">
-        <v>15.67595583966943</v>
+        <v>15.67595395070043</v>
       </c>
       <c r="E57" t="n">
-        <v>15.98482231303345</v>
+        <v>15.98482038684572</v>
       </c>
       <c r="F57" t="n">
         <v>6358000</v>
@@ -1592,16 +1592,16 @@
         <v>44337</v>
       </c>
       <c r="B59" t="n">
-        <v>16.43477439880371</v>
+        <v>16.43477249145508</v>
       </c>
       <c r="C59" t="n">
-        <v>16.6254337643569</v>
+        <v>16.62543183488117</v>
       </c>
       <c r="D59" t="n">
-        <v>15.75984264485187</v>
+        <v>15.75984081583289</v>
       </c>
       <c r="E59" t="n">
-        <v>16.03439118575198</v>
+        <v>16.03438932487009</v>
       </c>
       <c r="F59" t="n">
         <v>10145000</v>
@@ -1652,16 +1652,16 @@
         <v>44342</v>
       </c>
       <c r="B62" t="n">
-        <v>16.94192695617676</v>
+        <v>16.94192504882812</v>
       </c>
       <c r="C62" t="n">
-        <v>17.11161449219801</v>
+        <v>17.11161256574568</v>
       </c>
       <c r="D62" t="n">
-        <v>16.65975260630318</v>
+        <v>16.65975073072218</v>
       </c>
       <c r="E62" t="n">
-        <v>17.02391059716581</v>
+        <v>17.02390868058733</v>
       </c>
       <c r="F62" t="n">
         <v>5462000</v>
@@ -1752,16 +1752,16 @@
         <v>44349</v>
       </c>
       <c r="B67" t="n">
-        <v>16.76651763916016</v>
+        <v>16.76651954650879</v>
       </c>
       <c r="C67" t="n">
-        <v>17.26032492574389</v>
+        <v>17.26032688926774</v>
       </c>
       <c r="D67" t="n">
-        <v>16.73982554996776</v>
+        <v>16.73982745427992</v>
       </c>
       <c r="E67" t="n">
-        <v>17.06394533438589</v>
+        <v>17.06394727556971</v>
       </c>
       <c r="F67" t="n">
         <v>9352500</v>
@@ -1772,16 +1772,16 @@
         <v>44351</v>
       </c>
       <c r="B68" t="n">
-        <v>16.77223968505859</v>
+        <v>16.77223777770996</v>
       </c>
       <c r="C68" t="n">
-        <v>16.81609071938215</v>
+        <v>16.81608880704675</v>
       </c>
       <c r="D68" t="n">
-        <v>16.40617437066384</v>
+        <v>16.40617250494436</v>
       </c>
       <c r="E68" t="n">
-        <v>16.72266839722167</v>
+        <v>16.72266649551031</v>
       </c>
       <c r="F68" t="n">
         <v>8097000</v>
@@ -1812,16 +1812,16 @@
         <v>44355</v>
       </c>
       <c r="B70" t="n">
-        <v>16.08205604553223</v>
+        <v>16.08205795288086</v>
       </c>
       <c r="C70" t="n">
-        <v>16.61017944054762</v>
+        <v>16.61018141053224</v>
       </c>
       <c r="D70" t="n">
-        <v>15.92952747058032</v>
+        <v>15.9295293598389</v>
       </c>
       <c r="E70" t="n">
-        <v>16.60064629097173</v>
+        <v>16.60064825982571</v>
       </c>
       <c r="F70" t="n">
         <v>9246000</v>
@@ -1832,16 +1832,16 @@
         <v>44356</v>
       </c>
       <c r="B71" t="n">
-        <v>16.16403961181641</v>
+        <v>16.16403770446777</v>
       </c>
       <c r="C71" t="n">
-        <v>16.39664448651429</v>
+        <v>16.39664255171839</v>
       </c>
       <c r="D71" t="n">
-        <v>15.82466817777308</v>
+        <v>15.82466631047011</v>
       </c>
       <c r="E71" t="n">
-        <v>16.08205778944601</v>
+        <v>16.08205589177119</v>
       </c>
       <c r="F71" t="n">
         <v>10294500</v>
@@ -1912,16 +1912,16 @@
         <v>44362</v>
       </c>
       <c r="B75" t="n">
-        <v>15.85898780822754</v>
+        <v>15.85898590087891</v>
       </c>
       <c r="C75" t="n">
-        <v>16.0267680045235</v>
+        <v>16.02676607699607</v>
       </c>
       <c r="D75" t="n">
-        <v>15.48720398490564</v>
+        <v>15.48720212227117</v>
       </c>
       <c r="E75" t="n">
-        <v>16.01532749522961</v>
+        <v>16.01532556907812</v>
       </c>
       <c r="F75" t="n">
         <v>8432500</v>
@@ -1932,16 +1932,16 @@
         <v>44363</v>
       </c>
       <c r="B76" t="n">
-        <v>15.89902400970459</v>
+        <v>15.89902210235596</v>
       </c>
       <c r="C76" t="n">
-        <v>16.11446811967458</v>
+        <v>16.1144661864799</v>
       </c>
       <c r="D76" t="n">
-        <v>15.66260805961109</v>
+        <v>15.66260618062443</v>
       </c>
       <c r="E76" t="n">
-        <v>15.70264620071735</v>
+        <v>15.70264431692745</v>
       </c>
       <c r="F76" t="n">
         <v>10606500</v>
@@ -1992,16 +1992,16 @@
         <v>44368</v>
       </c>
       <c r="B79" t="n">
-        <v>16.48434448242188</v>
+        <v>16.48434638977051</v>
       </c>
       <c r="C79" t="n">
-        <v>16.59302020374093</v>
+        <v>16.59302212366407</v>
       </c>
       <c r="D79" t="n">
-        <v>16.00007212945171</v>
+        <v>16.0000739807668</v>
       </c>
       <c r="E79" t="n">
-        <v>16.20789042268334</v>
+        <v>16.20789229804439</v>
       </c>
       <c r="F79" t="n">
         <v>6798000</v>
@@ -2012,16 +2012,16 @@
         <v>44369</v>
       </c>
       <c r="B80" t="n">
-        <v>16.47290420532227</v>
+        <v>16.4729061126709</v>
       </c>
       <c r="C80" t="n">
-        <v>16.49578339803871</v>
+        <v>16.49578530803645</v>
       </c>
       <c r="D80" t="n">
-        <v>16.13162548984007</v>
+        <v>16.13162735767305</v>
       </c>
       <c r="E80" t="n">
-        <v>16.46718395257762</v>
+        <v>16.46718585926392</v>
       </c>
       <c r="F80" t="n">
         <v>6518000</v>
@@ -2032,16 +2032,16 @@
         <v>44370</v>
       </c>
       <c r="B81" t="n">
-        <v>16.39664459228516</v>
+        <v>16.39664268493652</v>
       </c>
       <c r="C81" t="n">
-        <v>16.45574721722616</v>
+        <v>16.45574530300238</v>
       </c>
       <c r="D81" t="n">
-        <v>16.20979811200328</v>
+        <v>16.20979622638967</v>
       </c>
       <c r="E81" t="n">
-        <v>16.4004574889011</v>
+        <v>16.40045558110893</v>
       </c>
       <c r="F81" t="n">
         <v>5819500</v>
@@ -2052,16 +2052,16 @@
         <v>44371</v>
       </c>
       <c r="B82" t="n">
-        <v>16.64640235900879</v>
+        <v>16.64640426635742</v>
       </c>
       <c r="C82" t="n">
-        <v>16.72647862235864</v>
+        <v>16.72648053888243</v>
       </c>
       <c r="D82" t="n">
-        <v>16.39664042071346</v>
+        <v>16.39664229944431</v>
       </c>
       <c r="E82" t="n">
-        <v>16.46908907450944</v>
+        <v>16.46909096154148</v>
       </c>
       <c r="F82" t="n">
         <v>8527500</v>
@@ -2092,16 +2092,16 @@
         <v>44375</v>
       </c>
       <c r="B84" t="n">
-        <v>16.3737621307373</v>
+        <v>16.37376403808594</v>
       </c>
       <c r="C84" t="n">
-        <v>16.37948056539015</v>
+        <v>16.37948247340491</v>
       </c>
       <c r="D84" t="n">
-        <v>15.9390592744375</v>
+        <v>15.93906113114842</v>
       </c>
       <c r="E84" t="n">
-        <v>16.2250482827814</v>
+        <v>16.22505017280664</v>
       </c>
       <c r="F84" t="n">
         <v>6202500</v>
@@ -2112,16 +2112,16 @@
         <v>44376</v>
       </c>
       <c r="B85" t="n">
-        <v>16.42333602905273</v>
+        <v>16.42333793640137</v>
       </c>
       <c r="C85" t="n">
-        <v>16.53963755336238</v>
+        <v>16.53963947421787</v>
       </c>
       <c r="D85" t="n">
-        <v>16.120188031945</v>
+        <v>16.12018990408709</v>
       </c>
       <c r="E85" t="n">
-        <v>16.3680444846797</v>
+        <v>16.36804638560697</v>
       </c>
       <c r="F85" t="n">
         <v>8958000</v>
@@ -2132,16 +2132,16 @@
         <v>44377</v>
       </c>
       <c r="B86" t="n">
-        <v>16.49959945678711</v>
+        <v>16.49959754943848</v>
       </c>
       <c r="C86" t="n">
-        <v>16.49959945678711</v>
+        <v>16.49959754943848</v>
       </c>
       <c r="D86" t="n">
-        <v>16.19073120503556</v>
+        <v>16.19072933339201</v>
       </c>
       <c r="E86" t="n">
-        <v>16.38901636774828</v>
+        <v>16.38901447318302</v>
       </c>
       <c r="F86" t="n">
         <v>6685000</v>
@@ -2172,16 +2172,16 @@
         <v>44379</v>
       </c>
       <c r="B88" t="n">
-        <v>16.39664459228516</v>
+        <v>16.39664268493652</v>
       </c>
       <c r="C88" t="n">
-        <v>16.45765457466542</v>
+        <v>16.45765266021977</v>
       </c>
       <c r="D88" t="n">
-        <v>16.21551836605848</v>
+        <v>16.21551647977946</v>
       </c>
       <c r="E88" t="n">
-        <v>16.36804514027171</v>
+        <v>16.36804323624992</v>
       </c>
       <c r="F88" t="n">
         <v>5948000</v>
@@ -2192,16 +2192,16 @@
         <v>44382</v>
       </c>
       <c r="B89" t="n">
-        <v>16.41570663452148</v>
+        <v>16.41570854187012</v>
       </c>
       <c r="C89" t="n">
-        <v>16.54726154865489</v>
+        <v>16.54726347128895</v>
       </c>
       <c r="D89" t="n">
-        <v>16.25174119484036</v>
+        <v>16.25174308313778</v>
       </c>
       <c r="E89" t="n">
-        <v>16.40808084242347</v>
+        <v>16.40808274888606</v>
       </c>
       <c r="F89" t="n">
         <v>3871000</v>
@@ -2212,16 +2212,16 @@
         <v>44383</v>
       </c>
       <c r="B90" t="n">
-        <v>16.33944320678711</v>
+        <v>16.33944511413574</v>
       </c>
       <c r="C90" t="n">
-        <v>16.38901449179115</v>
+        <v>16.38901640492637</v>
       </c>
       <c r="D90" t="n">
-        <v>16.11256043736321</v>
+        <v>16.11256231822719</v>
       </c>
       <c r="E90" t="n">
-        <v>16.38901449179115</v>
+        <v>16.38901640492637</v>
       </c>
       <c r="F90" t="n">
         <v>3828000</v>
@@ -2252,16 +2252,16 @@
         <v>44385</v>
       </c>
       <c r="B92" t="n">
-        <v>16.43477439880371</v>
+        <v>16.43477249145508</v>
       </c>
       <c r="C92" t="n">
-        <v>16.79893236876558</v>
+        <v>16.79893041915436</v>
       </c>
       <c r="D92" t="n">
-        <v>16.24411685151298</v>
+        <v>16.24411496629124</v>
       </c>
       <c r="E92" t="n">
-        <v>16.26318133345833</v>
+        <v>16.26317944602405</v>
       </c>
       <c r="F92" t="n">
         <v>7435000</v>
@@ -2312,16 +2312,16 @@
         <v>44391</v>
       </c>
       <c r="B95" t="n">
-        <v>16.72266960144043</v>
+        <v>16.7226676940918</v>
       </c>
       <c r="C95" t="n">
-        <v>17.08873494219598</v>
+        <v>17.08873299309478</v>
       </c>
       <c r="D95" t="n">
-        <v>16.67309831003382</v>
+        <v>16.67309640833917</v>
       </c>
       <c r="E95" t="n">
-        <v>16.93048791752151</v>
+        <v>16.9304859864696</v>
       </c>
       <c r="F95" t="n">
         <v>5548000</v>
@@ -2332,16 +2332,16 @@
         <v>44392</v>
       </c>
       <c r="B96" t="n">
-        <v>16.45002555847168</v>
+        <v>16.45002746582031</v>
       </c>
       <c r="C96" t="n">
-        <v>16.86375476157448</v>
+        <v>16.86375671689422</v>
       </c>
       <c r="D96" t="n">
-        <v>16.44049240966831</v>
+        <v>16.44049431591159</v>
       </c>
       <c r="E96" t="n">
-        <v>16.72266670485169</v>
+        <v>16.72266864381253</v>
       </c>
       <c r="F96" t="n">
         <v>3746000</v>
@@ -2372,16 +2372,16 @@
         <v>44396</v>
       </c>
       <c r="B98" t="n">
-        <v>16.65402984619141</v>
+        <v>16.65403175354004</v>
       </c>
       <c r="C98" t="n">
-        <v>16.79702526617702</v>
+        <v>16.7970271899026</v>
       </c>
       <c r="D98" t="n">
-        <v>16.40426788246265</v>
+        <v>16.40426976120661</v>
       </c>
       <c r="E98" t="n">
-        <v>16.58539408105208</v>
+        <v>16.58539598054001</v>
       </c>
       <c r="F98" t="n">
         <v>7763500</v>
@@ -2392,16 +2392,16 @@
         <v>44397</v>
       </c>
       <c r="B99" t="n">
-        <v>16.51103401184082</v>
+        <v>16.51103782653809</v>
       </c>
       <c r="C99" t="n">
-        <v>16.71694491594005</v>
+        <v>16.71694877821082</v>
       </c>
       <c r="D99" t="n">
-        <v>16.45955719494704</v>
+        <v>16.45956099775114</v>
       </c>
       <c r="E99" t="n">
-        <v>16.65402759422851</v>
+        <v>16.6540314419629</v>
       </c>
       <c r="F99" t="n">
         <v>3835500</v>
@@ -2432,16 +2432,16 @@
         <v>44399</v>
       </c>
       <c r="B101" t="n">
-        <v>16.64449501037598</v>
+        <v>16.64449691772461</v>
       </c>
       <c r="C101" t="n">
-        <v>16.68072024642313</v>
+        <v>16.68072215792294</v>
       </c>
       <c r="D101" t="n">
-        <v>16.44430435190125</v>
+        <v>16.44430623630937</v>
       </c>
       <c r="E101" t="n">
-        <v>16.58729793913493</v>
+        <v>16.58729983992916</v>
       </c>
       <c r="F101" t="n">
         <v>2829500</v>
@@ -2472,16 +2472,16 @@
         <v>44403</v>
       </c>
       <c r="B103" t="n">
-        <v>17.19741058349609</v>
+        <v>17.19740867614746</v>
       </c>
       <c r="C103" t="n">
-        <v>17.21647506604089</v>
+        <v>17.21647315657783</v>
       </c>
       <c r="D103" t="n">
-        <v>16.56060959167434</v>
+        <v>16.5606077549527</v>
       </c>
       <c r="E103" t="n">
-        <v>16.75126896322247</v>
+        <v>16.75126710535498</v>
       </c>
       <c r="F103" t="n">
         <v>9987000</v>
@@ -2512,16 +2512,16 @@
         <v>44405</v>
       </c>
       <c r="B105" t="n">
-        <v>16.793212890625</v>
+        <v>16.79321479797363</v>
       </c>
       <c r="C105" t="n">
-        <v>17.38044259996134</v>
+        <v>17.38044457400667</v>
       </c>
       <c r="D105" t="n">
-        <v>16.42333646812846</v>
+        <v>16.42333833346707</v>
       </c>
       <c r="E105" t="n">
-        <v>17.34993760917749</v>
+        <v>17.3499395797581</v>
       </c>
       <c r="F105" t="n">
         <v>14614500</v>
@@ -2552,16 +2552,16 @@
         <v>44407</v>
       </c>
       <c r="B107" t="n">
-        <v>16.52628898620605</v>
+        <v>16.52629089355469</v>
       </c>
       <c r="C107" t="n">
-        <v>16.73219990991705</v>
+        <v>16.73220184103048</v>
       </c>
       <c r="D107" t="n">
-        <v>16.30893755658766</v>
+        <v>16.30893943885111</v>
       </c>
       <c r="E107" t="n">
-        <v>16.62543155217983</v>
+        <v>16.6254334709708</v>
       </c>
       <c r="F107" t="n">
         <v>16469000</v>
@@ -2592,16 +2592,16 @@
         <v>44411</v>
       </c>
       <c r="B109" t="n">
-        <v>16.53010368347168</v>
+        <v>16.53010177612305</v>
       </c>
       <c r="C109" t="n">
-        <v>16.68072308765598</v>
+        <v>16.68072116292792</v>
       </c>
       <c r="D109" t="n">
-        <v>16.26127540276083</v>
+        <v>16.26127352643131</v>
       </c>
       <c r="E109" t="n">
-        <v>16.68072308765598</v>
+        <v>16.68072116292792</v>
       </c>
       <c r="F109" t="n">
         <v>5450500</v>
@@ -2652,16 +2652,16 @@
         <v>44414</v>
       </c>
       <c r="B112" t="n">
-        <v>16.73982810974121</v>
+        <v>16.73982620239258</v>
       </c>
       <c r="C112" t="n">
-        <v>16.78368096434495</v>
+        <v>16.78367905199969</v>
       </c>
       <c r="D112" t="n">
-        <v>16.37567013584921</v>
+        <v>16.37566826999301</v>
       </c>
       <c r="E112" t="n">
-        <v>16.63115237929877</v>
+        <v>16.63115048433273</v>
       </c>
       <c r="F112" t="n">
         <v>15424500</v>
@@ -2672,16 +2672,16 @@
         <v>44417</v>
       </c>
       <c r="B113" t="n">
-        <v>17.31942749023438</v>
+        <v>17.31942939758301</v>
       </c>
       <c r="C113" t="n">
-        <v>17.35756008512363</v>
+        <v>17.35756199667172</v>
       </c>
       <c r="D113" t="n">
-        <v>16.61780374497947</v>
+        <v>16.6178055750599</v>
       </c>
       <c r="E113" t="n">
-        <v>16.61780374497947</v>
+        <v>16.6178055750599</v>
       </c>
       <c r="F113" t="n">
         <v>10558500</v>
@@ -2712,16 +2712,16 @@
         <v>44419</v>
       </c>
       <c r="B115" t="n">
-        <v>17.20884895324707</v>
+        <v>17.20884704589844</v>
       </c>
       <c r="C115" t="n">
-        <v>17.57872718168084</v>
+        <v>17.57872523333663</v>
       </c>
       <c r="D115" t="n">
-        <v>17.19741026393275</v>
+        <v>17.19740835785192</v>
       </c>
       <c r="E115" t="n">
-        <v>17.57872718168084</v>
+        <v>17.57872523333663</v>
       </c>
       <c r="F115" t="n">
         <v>6265000</v>
@@ -2732,16 +2732,16 @@
         <v>44420</v>
       </c>
       <c r="B116" t="n">
-        <v>16.92095184326172</v>
+        <v>16.92095375061035</v>
       </c>
       <c r="C116" t="n">
-        <v>17.24507162966405</v>
+        <v>17.24507357354782</v>
       </c>
       <c r="D116" t="n">
-        <v>16.68262857786367</v>
+        <v>16.68263045834824</v>
       </c>
       <c r="E116" t="n">
-        <v>16.98768206665122</v>
+        <v>16.98768398152176</v>
       </c>
       <c r="F116" t="n">
         <v>14059400</v>
@@ -2752,16 +2752,16 @@
         <v>44421</v>
       </c>
       <c r="B117" t="n">
-        <v>16.91141891479492</v>
+        <v>16.91142082214355</v>
       </c>
       <c r="C117" t="n">
-        <v>17.27367130114663</v>
+        <v>17.27367324935177</v>
       </c>
       <c r="D117" t="n">
-        <v>16.53010204884227</v>
+        <v>16.53010391318421</v>
       </c>
       <c r="E117" t="n">
-        <v>16.82562239267279</v>
+        <v>16.82562429034489</v>
       </c>
       <c r="F117" t="n">
         <v>5547600</v>
@@ -2832,16 +2832,16 @@
         <v>44427</v>
       </c>
       <c r="B121" t="n">
-        <v>16.6635627746582</v>
+        <v>16.66356658935547</v>
       </c>
       <c r="C121" t="n">
-        <v>16.87328841811889</v>
+        <v>16.87329228082749</v>
       </c>
       <c r="D121" t="n">
-        <v>15.57680923404292</v>
+        <v>15.57681279995571</v>
       </c>
       <c r="E121" t="n">
-        <v>15.71026968478171</v>
+        <v>15.71027328124686</v>
       </c>
       <c r="F121" t="n">
         <v>14455000</v>
@@ -2872,16 +2872,16 @@
         <v>44431</v>
       </c>
       <c r="B123" t="n">
-        <v>16.69216537475586</v>
+        <v>16.69216346740723</v>
       </c>
       <c r="C123" t="n">
-        <v>17.16881200972343</v>
+        <v>17.16881004791025</v>
       </c>
       <c r="D123" t="n">
-        <v>16.52057229524551</v>
+        <v>16.52057040750415</v>
       </c>
       <c r="E123" t="n">
-        <v>16.97815262843136</v>
+        <v>16.97815068840407</v>
       </c>
       <c r="F123" t="n">
         <v>5050600</v>
@@ -2892,16 +2892,16 @@
         <v>44432</v>
       </c>
       <c r="B124" t="n">
-        <v>16.91141891479492</v>
+        <v>16.91142082214355</v>
       </c>
       <c r="C124" t="n">
-        <v>17.05441251224439</v>
+        <v>17.05441443572051</v>
       </c>
       <c r="D124" t="n">
-        <v>16.66356249736014</v>
+        <v>16.66356437675437</v>
       </c>
       <c r="E124" t="n">
-        <v>16.78749161520865</v>
+        <v>16.78749350858018</v>
       </c>
       <c r="F124" t="n">
         <v>4198100</v>
@@ -3012,16 +3012,16 @@
         <v>44440</v>
       </c>
       <c r="B130" t="n">
-        <v>16.23458290100098</v>
+        <v>16.23458099365234</v>
       </c>
       <c r="C130" t="n">
-        <v>16.77795970229644</v>
+        <v>16.77795773110823</v>
       </c>
       <c r="D130" t="n">
-        <v>15.89139678723021</v>
+        <v>15.8913949202014</v>
       </c>
       <c r="E130" t="n">
-        <v>16.30131313017587</v>
+        <v>16.30131121498732</v>
       </c>
       <c r="F130" t="n">
         <v>7651500</v>
@@ -3032,16 +3032,16 @@
         <v>44441</v>
       </c>
       <c r="B131" t="n">
-        <v>16.72076225280762</v>
+        <v>16.72076416015625</v>
       </c>
       <c r="C131" t="n">
-        <v>17.03534891071645</v>
+        <v>17.03535085395019</v>
       </c>
       <c r="D131" t="n">
-        <v>16.10112026815059</v>
+        <v>16.10112210481625</v>
       </c>
       <c r="E131" t="n">
-        <v>16.16785049584908</v>
+        <v>16.1678523401267</v>
       </c>
       <c r="F131" t="n">
         <v>17566400</v>
@@ -3052,16 +3052,16 @@
         <v>44442</v>
       </c>
       <c r="B132" t="n">
-        <v>17.31180381774902</v>
+        <v>17.31180572509766</v>
       </c>
       <c r="C132" t="n">
-        <v>17.35946774893307</v>
+        <v>17.35946966153313</v>
       </c>
       <c r="D132" t="n">
-        <v>16.69216362104432</v>
+        <v>16.69216546012336</v>
       </c>
       <c r="E132" t="n">
-        <v>16.90188746382151</v>
+        <v>16.90188932600712</v>
       </c>
       <c r="F132" t="n">
         <v>19565300</v>
@@ -3092,16 +3092,16 @@
         <v>44447</v>
       </c>
       <c r="B134" t="n">
-        <v>17.0734806060791</v>
+        <v>17.07347869873047</v>
       </c>
       <c r="C134" t="n">
-        <v>17.55012719322427</v>
+        <v>17.55012523262749</v>
       </c>
       <c r="D134" t="n">
-        <v>16.84469046244091</v>
+        <v>16.84468858065136</v>
       </c>
       <c r="E134" t="n">
-        <v>17.49293011188033</v>
+        <v>17.49292815767328</v>
       </c>
       <c r="F134" t="n">
         <v>11069100</v>
@@ -3112,16 +3112,16 @@
         <v>44448</v>
       </c>
       <c r="B135" t="n">
-        <v>17.34993934631348</v>
+        <v>17.34993553161621</v>
       </c>
       <c r="C135" t="n">
-        <v>17.44526722477477</v>
+        <v>17.44526338911795</v>
       </c>
       <c r="D135" t="n">
-        <v>16.92095662018675</v>
+        <v>16.92095289980908</v>
       </c>
       <c r="E135" t="n">
-        <v>17.07348340764009</v>
+        <v>17.07347965372665</v>
       </c>
       <c r="F135" t="n">
         <v>12544000</v>
@@ -3152,16 +3152,16 @@
         <v>44452</v>
       </c>
       <c r="B137" t="n">
-        <v>17.79798316955566</v>
+        <v>17.79798126220703</v>
       </c>
       <c r="C137" t="n">
-        <v>17.9695762273458</v>
+        <v>17.96957430160813</v>
       </c>
       <c r="D137" t="n">
-        <v>17.49292965271203</v>
+        <v>17.49292777805493</v>
       </c>
       <c r="E137" t="n">
-        <v>17.5787261816071</v>
+        <v>17.57872429775548</v>
       </c>
       <c r="F137" t="n">
         <v>17075500</v>
@@ -3172,16 +3172,16 @@
         <v>44453</v>
       </c>
       <c r="B138" t="n">
-        <v>17.47386360168457</v>
+        <v>17.47386169433594</v>
       </c>
       <c r="C138" t="n">
-        <v>18.1507026927803</v>
+        <v>18.15070071155172</v>
       </c>
       <c r="D138" t="n">
-        <v>17.3976002213898</v>
+        <v>17.39759832236565</v>
       </c>
       <c r="E138" t="n">
-        <v>17.82658287196191</v>
+        <v>17.82658092611242</v>
       </c>
       <c r="F138" t="n">
         <v>6594500</v>
@@ -3272,16 +3272,16 @@
         <v>44460</v>
       </c>
       <c r="B143" t="n">
-        <v>18.57968139648438</v>
+        <v>18.57968330383301</v>
       </c>
       <c r="C143" t="n">
-        <v>18.74174128832697</v>
+        <v>18.7417432123123</v>
       </c>
       <c r="D143" t="n">
-        <v>17.82658082963624</v>
+        <v>17.82658265967325</v>
       </c>
       <c r="E143" t="n">
-        <v>18.06490409303639</v>
+        <v>18.06490594753913</v>
       </c>
       <c r="F143" t="n">
         <v>17756900</v>
@@ -3332,16 +3332,16 @@
         <v>44463</v>
       </c>
       <c r="B146" t="n">
-        <v>18.09350395202637</v>
+        <v>18.09350204467773</v>
       </c>
       <c r="C146" t="n">
-        <v>18.26509701375519</v>
+        <v>18.26509508831786</v>
       </c>
       <c r="D146" t="n">
-        <v>17.87424695904506</v>
+        <v>17.87424507480967</v>
       </c>
       <c r="E146" t="n">
-        <v>18.13163655163829</v>
+        <v>18.13163464026987</v>
       </c>
       <c r="F146" t="n">
         <v>18657800</v>
@@ -3372,16 +3372,16 @@
         <v>44467</v>
       </c>
       <c r="B148" t="n">
-        <v>18.2841625213623</v>
+        <v>18.28416061401367</v>
       </c>
       <c r="C148" t="n">
-        <v>18.29369567085224</v>
+        <v>18.29369376250914</v>
       </c>
       <c r="D148" t="n">
-        <v>18.01723979043107</v>
+        <v>18.01723791092701</v>
       </c>
       <c r="E148" t="n">
-        <v>18.23649677391261</v>
+        <v>18.23649487153633</v>
       </c>
       <c r="F148" t="n">
         <v>11310100</v>
@@ -3392,16 +3392,16 @@
         <v>44468</v>
       </c>
       <c r="B149" t="n">
-        <v>18.08396911621094</v>
+        <v>18.08397102355957</v>
       </c>
       <c r="C149" t="n">
-        <v>18.4271552076744</v>
+        <v>18.42715715121949</v>
       </c>
       <c r="D149" t="n">
-        <v>17.96957496456462</v>
+        <v>17.9695768598479</v>
       </c>
       <c r="E149" t="n">
-        <v>18.29369475799961</v>
+        <v>18.29369668746839</v>
       </c>
       <c r="F149" t="n">
         <v>10203400</v>
@@ -3412,16 +3412,16 @@
         <v>44469</v>
       </c>
       <c r="B150" t="n">
-        <v>18.15070343017578</v>
+        <v>18.15070152282715</v>
       </c>
       <c r="C150" t="n">
-        <v>18.6273500309481</v>
+        <v>18.62734807351153</v>
       </c>
       <c r="D150" t="n">
-        <v>18.04584059616188</v>
+        <v>18.04583869983265</v>
       </c>
       <c r="E150" t="n">
-        <v>18.30323019696192</v>
+        <v>18.30322827358517</v>
       </c>
       <c r="F150" t="n">
         <v>10293000</v>
@@ -3432,16 +3432,16 @@
         <v>44470</v>
       </c>
       <c r="B151" t="n">
-        <v>18.45575714111328</v>
+        <v>18.45575523376465</v>
       </c>
       <c r="C151" t="n">
-        <v>18.56061815787245</v>
+        <v>18.56061623968673</v>
       </c>
       <c r="D151" t="n">
-        <v>18.00770816839343</v>
+        <v>18.00770630734936</v>
       </c>
       <c r="E151" t="n">
-        <v>18.19836753783964</v>
+        <v>18.19836565709148</v>
       </c>
       <c r="F151" t="n">
         <v>5841800</v>
@@ -3452,16 +3452,16 @@
         <v>44473</v>
       </c>
       <c r="B152" t="n">
-        <v>18.4176197052002</v>
+        <v>18.41762351989746</v>
       </c>
       <c r="C152" t="n">
-        <v>18.49388306930666</v>
+        <v>18.49388689979976</v>
       </c>
       <c r="D152" t="n">
-        <v>18.0744336575901</v>
+        <v>18.07443740120593</v>
       </c>
       <c r="E152" t="n">
-        <v>18.38902208007404</v>
+        <v>18.3890258888481</v>
       </c>
       <c r="F152" t="n">
         <v>9789400</v>
@@ -3592,16 +3592,16 @@
         <v>44483</v>
       </c>
       <c r="B159" t="n">
-        <v>17.06758308410645</v>
+        <v>17.06758117675781</v>
       </c>
       <c r="C159" t="n">
-        <v>17.14403354871527</v>
+        <v>17.14403163282309</v>
       </c>
       <c r="D159" t="n">
-        <v>16.60887847373064</v>
+        <v>16.6088766176435</v>
       </c>
       <c r="E159" t="n">
-        <v>16.96246301174824</v>
+        <v>16.96246111614706</v>
       </c>
       <c r="F159" t="n">
         <v>10051300</v>
@@ -3772,16 +3772,16 @@
         <v>44496</v>
       </c>
       <c r="B168" t="n">
-        <v>14.94607830047607</v>
+        <v>14.94607734680176</v>
       </c>
       <c r="C168" t="n">
-        <v>15.38566886553011</v>
+        <v>15.38566788380655</v>
       </c>
       <c r="D168" t="n">
-        <v>14.81228955063831</v>
+        <v>14.81228860550074</v>
       </c>
       <c r="E168" t="n">
-        <v>15.38566886553011</v>
+        <v>15.38566788380655</v>
       </c>
       <c r="F168" t="n">
         <v>9783700</v>
@@ -3812,16 +3812,16 @@
         <v>44498</v>
       </c>
       <c r="B170" t="n">
-        <v>14.61160850524902</v>
+        <v>14.61160755157471</v>
       </c>
       <c r="C170" t="n">
-        <v>15.21365657937846</v>
+        <v>15.21365558640951</v>
       </c>
       <c r="D170" t="n">
-        <v>14.50648934742759</v>
+        <v>14.50648840061422</v>
       </c>
       <c r="E170" t="n">
-        <v>15.0034173523742</v>
+        <v>15.0034163731272</v>
       </c>
       <c r="F170" t="n">
         <v>13706000</v>
@@ -3832,16 +3832,16 @@
         <v>44501</v>
       </c>
       <c r="B171" t="n">
-        <v>14.31536197662354</v>
+        <v>14.31536102294922</v>
       </c>
       <c r="C171" t="n">
-        <v>14.77406565205061</v>
+        <v>14.77406466781794</v>
       </c>
       <c r="D171" t="n">
-        <v>14.20068628560711</v>
+        <v>14.20068533957237</v>
       </c>
       <c r="E171" t="n">
-        <v>14.76450911662556</v>
+        <v>14.76450813302954</v>
       </c>
       <c r="F171" t="n">
         <v>10277500</v>
@@ -3912,16 +3912,16 @@
         <v>44508</v>
       </c>
       <c r="B175" t="n">
-        <v>14.73583889007568</v>
+        <v>14.73583984375</v>
       </c>
       <c r="C175" t="n">
-        <v>14.89829632997021</v>
+        <v>14.89829729415845</v>
       </c>
       <c r="D175" t="n">
-        <v>14.28669179675779</v>
+        <v>14.2866927213642</v>
       </c>
       <c r="E175" t="n">
-        <v>14.39181185278442</v>
+        <v>14.39181278419399</v>
       </c>
       <c r="F175" t="n">
         <v>8290300</v>
@@ -3952,16 +3952,16 @@
         <v>44510</v>
       </c>
       <c r="B177" t="n">
-        <v>15.26143836975098</v>
+        <v>15.26143932342529</v>
       </c>
       <c r="C177" t="n">
-        <v>15.38567059902005</v>
+        <v>15.38567156045753</v>
       </c>
       <c r="D177" t="n">
-        <v>14.7167276858233</v>
+        <v>14.71672860545911</v>
       </c>
       <c r="E177" t="n">
-        <v>14.84095991509237</v>
+        <v>14.84096084249134</v>
       </c>
       <c r="F177" t="n">
         <v>10223900</v>
@@ -3992,16 +3992,16 @@
         <v>44512</v>
       </c>
       <c r="B179" t="n">
-        <v>14.84096050262451</v>
+        <v>14.8409595489502</v>
       </c>
       <c r="C179" t="n">
-        <v>15.23276936586659</v>
+        <v>15.23276838701479</v>
       </c>
       <c r="D179" t="n">
-        <v>14.82184834194417</v>
+        <v>14.82184738949799</v>
       </c>
       <c r="E179" t="n">
-        <v>15.089424970999</v>
+        <v>15.08942400135846</v>
       </c>
       <c r="F179" t="n">
         <v>7831400</v>
@@ -4012,16 +4012,16 @@
         <v>44516</v>
       </c>
       <c r="B180" t="n">
-        <v>14.18157386779785</v>
+        <v>14.18157482147217</v>
       </c>
       <c r="C180" t="n">
-        <v>14.86007237747372</v>
+        <v>14.86007337677532</v>
       </c>
       <c r="D180" t="n">
-        <v>14.00000334347483</v>
+        <v>14.00000428493899</v>
       </c>
       <c r="E180" t="n">
-        <v>14.81229061258022</v>
+        <v>14.81229160866862</v>
       </c>
       <c r="F180" t="n">
         <v>11424100</v>
@@ -4052,16 +4052,16 @@
         <v>44518</v>
       </c>
       <c r="B182" t="n">
-        <v>13.3597297668457</v>
+        <v>13.35973072052002</v>
       </c>
       <c r="C182" t="n">
-        <v>13.69420120231332</v>
+        <v>13.69420217986363</v>
       </c>
       <c r="D182" t="n">
-        <v>13.13993492912112</v>
+        <v>13.13993586710555</v>
       </c>
       <c r="E182" t="n">
-        <v>13.65597597351942</v>
+        <v>13.65597694834105</v>
       </c>
       <c r="F182" t="n">
         <v>21252300</v>
@@ -4112,16 +4112,16 @@
         <v>44523</v>
       </c>
       <c r="B185" t="n">
-        <v>13.24505424499512</v>
+        <v>13.2450532913208</v>
       </c>
       <c r="C185" t="n">
-        <v>13.4170682323851</v>
+        <v>13.41706726632538</v>
       </c>
       <c r="D185" t="n">
-        <v>12.99659071042901</v>
+        <v>12.99658977464464</v>
       </c>
       <c r="E185" t="n">
-        <v>13.23549862119895</v>
+        <v>13.23549766821266</v>
       </c>
       <c r="F185" t="n">
         <v>3755200</v>
@@ -4212,16 +4212,16 @@
         <v>44530</v>
       </c>
       <c r="B190" t="n">
-        <v>12.18430328369141</v>
+        <v>12.18430423736572</v>
       </c>
       <c r="C190" t="n">
-        <v>12.44232426127008</v>
+        <v>12.44232523513989</v>
       </c>
       <c r="D190" t="n">
-        <v>11.84027622494785</v>
+        <v>11.84027715169492</v>
       </c>
       <c r="E190" t="n">
-        <v>12.38498596246548</v>
+        <v>12.38498693184738</v>
       </c>
       <c r="F190" t="n">
         <v>16793700</v>
@@ -4232,16 +4232,16 @@
         <v>44531</v>
       </c>
       <c r="B191" t="n">
-        <v>11.91672706604004</v>
+        <v>11.91672801971436</v>
       </c>
       <c r="C191" t="n">
-        <v>12.37542982579687</v>
+        <v>12.37543081618034</v>
       </c>
       <c r="D191" t="n">
-        <v>11.81160700007474</v>
+        <v>11.81160794533648</v>
       </c>
       <c r="E191" t="n">
-        <v>12.2989793658374</v>
+        <v>12.29898035010268</v>
       </c>
       <c r="F191" t="n">
         <v>5991300</v>
@@ -4252,16 +4252,16 @@
         <v>44532</v>
       </c>
       <c r="B192" t="n">
-        <v>11.89761447906494</v>
+        <v>11.89761352539062</v>
       </c>
       <c r="C192" t="n">
-        <v>12.14607893971519</v>
+        <v>12.14607796612476</v>
       </c>
       <c r="D192" t="n">
-        <v>11.71604485711986</v>
+        <v>11.71604391799958</v>
       </c>
       <c r="E192" t="n">
-        <v>12.14607893971519</v>
+        <v>12.14607796612476</v>
       </c>
       <c r="F192" t="n">
         <v>7306700</v>
@@ -4392,16 +4392,16 @@
         <v>44543</v>
       </c>
       <c r="B199" t="n">
-        <v>13.74198341369629</v>
+        <v>13.74198246002197</v>
       </c>
       <c r="C199" t="n">
-        <v>14.12423571408451</v>
+        <v>14.12423473388242</v>
       </c>
       <c r="D199" t="n">
-        <v>13.66553295361865</v>
+        <v>13.66553200524988</v>
       </c>
       <c r="E199" t="n">
-        <v>13.96177825857917</v>
+        <v>13.9617772896514</v>
       </c>
       <c r="F199" t="n">
         <v>11783000</v>
@@ -4432,16 +4432,16 @@
         <v>44545</v>
       </c>
       <c r="B201" t="n">
-        <v>14.03822898864746</v>
+        <v>14.03822803497314</v>
       </c>
       <c r="C201" t="n">
-        <v>14.05734205971515</v>
+        <v>14.0573411047424</v>
       </c>
       <c r="D201" t="n">
-        <v>13.73242714245554</v>
+        <v>13.7324262095556</v>
       </c>
       <c r="E201" t="n">
-        <v>13.92355329632549</v>
+        <v>13.92355235044156</v>
       </c>
       <c r="F201" t="n">
         <v>6373000</v>
@@ -4492,16 +4492,16 @@
         <v>44550</v>
       </c>
       <c r="B204" t="n">
-        <v>13.47440528869629</v>
+        <v>13.47440624237061</v>
       </c>
       <c r="C204" t="n">
-        <v>13.86621408038928</v>
+        <v>13.86621506179454</v>
       </c>
       <c r="D204" t="n">
-        <v>13.29283478290215</v>
+        <v>13.29283572372549</v>
       </c>
       <c r="E204" t="n">
-        <v>13.81843232037181</v>
+        <v>13.81843329839523</v>
       </c>
       <c r="F204" t="n">
         <v>6680500</v>
@@ -4592,16 +4592,16 @@
         <v>44558</v>
       </c>
       <c r="B209" t="n">
-        <v>12.51877498626709</v>
+        <v>12.51877403259277</v>
       </c>
       <c r="C209" t="n">
-        <v>13.12082212409239</v>
+        <v>13.12082112455441</v>
       </c>
       <c r="D209" t="n">
-        <v>12.31809230320487</v>
+        <v>12.31809136481846</v>
       </c>
       <c r="E209" t="n">
-        <v>13.12082212409239</v>
+        <v>13.12082112455441</v>
       </c>
       <c r="F209" t="n">
         <v>22962600</v>
@@ -4632,16 +4632,16 @@
         <v>44560</v>
       </c>
       <c r="B211" t="n">
-        <v>12.38498592376709</v>
+        <v>12.38498497009277</v>
       </c>
       <c r="C211" t="n">
-        <v>12.49966160965662</v>
+        <v>12.499660647152</v>
       </c>
       <c r="D211" t="n">
-        <v>12.25119716788196</v>
+        <v>12.25119622450971</v>
       </c>
       <c r="E211" t="n">
-        <v>12.32764762514165</v>
+        <v>12.32764667588253</v>
       </c>
       <c r="F211" t="n">
         <v>5913100</v>
@@ -4752,16 +4752,16 @@
         <v>44571</v>
       </c>
       <c r="B217" t="n">
-        <v>10.7986364364624</v>
+        <v>10.79863739013672</v>
       </c>
       <c r="C217" t="n">
-        <v>10.85597381771528</v>
+        <v>10.8559747764533</v>
       </c>
       <c r="D217" t="n">
-        <v>10.54061548674074</v>
+        <v>10.54061641762812</v>
       </c>
       <c r="E217" t="n">
-        <v>10.76041121184007</v>
+        <v>10.76041216213855</v>
       </c>
       <c r="F217" t="n">
         <v>8755800</v>
@@ -4872,16 +4872,16 @@
         <v>44579</v>
       </c>
       <c r="B223" t="n">
-        <v>11.39112854003906</v>
+        <v>11.39112949371338</v>
       </c>
       <c r="C223" t="n">
-        <v>11.49624768605842</v>
+        <v>11.49624864853339</v>
       </c>
       <c r="D223" t="n">
-        <v>11.29556501721325</v>
+        <v>11.29556596288691</v>
       </c>
       <c r="E223" t="n">
-        <v>11.47713552831003</v>
+        <v>11.47713648918492</v>
       </c>
       <c r="F223" t="n">
         <v>7771300</v>
@@ -4892,16 +4892,16 @@
         <v>44580</v>
       </c>
       <c r="B224" t="n">
-        <v>11.49624824523926</v>
+        <v>11.49624919891357</v>
       </c>
       <c r="C224" t="n">
-        <v>11.69693092384569</v>
+        <v>11.69693189416769</v>
       </c>
       <c r="D224" t="n">
-        <v>11.41979778780455</v>
+        <v>11.4197987351369</v>
       </c>
       <c r="E224" t="n">
-        <v>11.41979778780455</v>
+        <v>11.4197987351369</v>
       </c>
       <c r="F224" t="n">
         <v>5074700</v>
@@ -4952,16 +4952,16 @@
         <v>44585</v>
       </c>
       <c r="B227" t="n">
-        <v>11.50580501556396</v>
+        <v>11.50580406188965</v>
       </c>
       <c r="C227" t="n">
-        <v>11.63959377449148</v>
+        <v>11.6395928097279</v>
       </c>
       <c r="D227" t="n">
-        <v>11.3242354032836</v>
+        <v>11.32423446465893</v>
       </c>
       <c r="E227" t="n">
-        <v>11.46757978606487</v>
+        <v>11.4675788355589</v>
       </c>
       <c r="F227" t="n">
         <v>6551900</v>
@@ -4972,16 +4972,16 @@
         <v>44586</v>
       </c>
       <c r="B228" t="n">
-        <v>11.75427055358887</v>
+        <v>11.75426959991455</v>
       </c>
       <c r="C228" t="n">
-        <v>11.8880584135683</v>
+        <v>11.8880574490392</v>
       </c>
       <c r="D228" t="n">
-        <v>10.98020844521045</v>
+        <v>10.98020755433911</v>
       </c>
       <c r="E228" t="n">
-        <v>11.4293556170192</v>
+        <v>11.42935468970662</v>
       </c>
       <c r="F228" t="n">
         <v>40426700</v>
@@ -4992,16 +4992,16 @@
         <v>44587</v>
       </c>
       <c r="B229" t="n">
-        <v>11.73515701293945</v>
+        <v>11.73515605926514</v>
       </c>
       <c r="C229" t="n">
-        <v>12.21297286261863</v>
+        <v>12.21297187011393</v>
       </c>
       <c r="D229" t="n">
-        <v>11.73515701293945</v>
+        <v>11.73515605926514</v>
       </c>
       <c r="E229" t="n">
-        <v>11.81160747597921</v>
+        <v>11.81160651609204</v>
       </c>
       <c r="F229" t="n">
         <v>11052300</v>
@@ -5032,16 +5032,16 @@
         <v>44589</v>
       </c>
       <c r="B231" t="n">
-        <v>11.83071994781494</v>
+        <v>11.83071899414062</v>
       </c>
       <c r="C231" t="n">
-        <v>12.04095916619962</v>
+        <v>12.04095819557792</v>
       </c>
       <c r="D231" t="n">
-        <v>11.4580232758641</v>
+        <v>11.45802235223286</v>
       </c>
       <c r="E231" t="n">
-        <v>11.94539563656258</v>
+        <v>11.94539467364426</v>
       </c>
       <c r="F231" t="n">
         <v>14924100</v>
@@ -5072,16 +5072,16 @@
         <v>44593</v>
       </c>
       <c r="B233" t="n">
-        <v>12.0218448638916</v>
+        <v>12.02184581756592</v>
       </c>
       <c r="C233" t="n">
-        <v>12.09829531522309</v>
+        <v>12.0982962749621</v>
       </c>
       <c r="D233" t="n">
-        <v>11.83071873556289</v>
+        <v>11.83071967407547</v>
       </c>
       <c r="E233" t="n">
-        <v>11.93583787830337</v>
+        <v>11.93583882515488</v>
       </c>
       <c r="F233" t="n">
         <v>5991900</v>
@@ -5172,16 +5172,16 @@
         <v>44600</v>
       </c>
       <c r="B238" t="n">
-        <v>11.9549503326416</v>
+        <v>11.95495223999023</v>
       </c>
       <c r="C238" t="n">
-        <v>12.20341474238491</v>
+        <v>12.20341668937472</v>
       </c>
       <c r="D238" t="n">
-        <v>11.83071812776995</v>
+        <v>11.83072001529799</v>
       </c>
       <c r="E238" t="n">
-        <v>12.14607645115137</v>
+        <v>12.14607838899316</v>
       </c>
       <c r="F238" t="n">
         <v>8002100</v>
@@ -5192,16 +5192,16 @@
         <v>44601</v>
       </c>
       <c r="B239" t="n">
-        <v>12.05051517486572</v>
+        <v>12.05051422119141</v>
       </c>
       <c r="C239" t="n">
-        <v>12.28942309522567</v>
+        <v>12.28942212264425</v>
       </c>
       <c r="D239" t="n">
-        <v>11.91672732273544</v>
+        <v>11.91672637964906</v>
       </c>
       <c r="E239" t="n">
-        <v>11.95495255353858</v>
+        <v>11.95495160742706</v>
       </c>
       <c r="F239" t="n">
         <v>9060800</v>
@@ -5232,16 +5232,16 @@
         <v>44603</v>
       </c>
       <c r="B241" t="n">
-        <v>11.79249382019043</v>
+        <v>11.79249477386475</v>
       </c>
       <c r="C241" t="n">
-        <v>12.21297131357752</v>
+        <v>12.2129723012564</v>
       </c>
       <c r="D241" t="n">
-        <v>11.74471205901066</v>
+        <v>11.74471300882081</v>
       </c>
       <c r="E241" t="n">
-        <v>12.18430262141418</v>
+        <v>12.18430360677458</v>
       </c>
       <c r="F241" t="n">
         <v>7316000</v>
@@ -5252,16 +5252,16 @@
         <v>44606</v>
       </c>
       <c r="B242" t="n">
-        <v>11.78293800354004</v>
+        <v>11.78293895721436</v>
       </c>
       <c r="C242" t="n">
-        <v>11.97406414854188</v>
+        <v>11.97406511768535</v>
       </c>
       <c r="D242" t="n">
-        <v>11.639593622629</v>
+        <v>11.63959456470146</v>
       </c>
       <c r="E242" t="n">
-        <v>11.79249453863047</v>
+        <v>11.79249549307826</v>
       </c>
       <c r="F242" t="n">
         <v>5445000</v>
@@ -5272,16 +5272,16 @@
         <v>44607</v>
       </c>
       <c r="B243" t="n">
-        <v>11.63959503173828</v>
+        <v>11.63959312438965</v>
       </c>
       <c r="C243" t="n">
-        <v>11.95495343700949</v>
+        <v>11.95495147798393</v>
       </c>
       <c r="D243" t="n">
-        <v>11.53447495574024</v>
+        <v>11.53447306561735</v>
       </c>
       <c r="E243" t="n">
-        <v>11.92628382826741</v>
+        <v>11.92628187393986</v>
       </c>
       <c r="F243" t="n">
         <v>11329100</v>
@@ -5312,16 +5312,16 @@
         <v>44609</v>
       </c>
       <c r="B245" t="n">
-        <v>12.66211700439453</v>
+        <v>12.66211795806885</v>
       </c>
       <c r="C245" t="n">
-        <v>12.9488066282757</v>
+        <v>12.94880760354266</v>
       </c>
       <c r="D245" t="n">
-        <v>12.46143435881383</v>
+        <v>12.46143529737331</v>
       </c>
       <c r="E245" t="n">
-        <v>12.46143435881383</v>
+        <v>12.46143529737331</v>
       </c>
       <c r="F245" t="n">
         <v>10362100</v>
@@ -5372,16 +5372,16 @@
         <v>44614</v>
       </c>
       <c r="B248" t="n">
-        <v>12.51877498626709</v>
+        <v>12.51877403259277</v>
       </c>
       <c r="C248" t="n">
-        <v>12.63345067496531</v>
+        <v>12.63344971255505</v>
       </c>
       <c r="D248" t="n">
-        <v>12.08874001444707</v>
+        <v>12.08873909353262</v>
       </c>
       <c r="E248" t="n">
-        <v>12.14607831447686</v>
+        <v>12.1460773891944</v>
       </c>
       <c r="F248" t="n">
         <v>15416600</v>
@@ -5392,16 +5392,16 @@
         <v>44615</v>
       </c>
       <c r="B249" t="n">
-        <v>12.73856925964355</v>
+        <v>12.73857021331787</v>
       </c>
       <c r="C249" t="n">
-        <v>12.87235801283171</v>
+        <v>12.87235897652213</v>
       </c>
       <c r="D249" t="n">
-        <v>12.51877442729301</v>
+        <v>12.51877536451236</v>
       </c>
       <c r="E249" t="n">
-        <v>12.51877442729301</v>
+        <v>12.51877536451236</v>
       </c>
       <c r="F249" t="n">
         <v>5598100</v>
@@ -5472,16 +5472,16 @@
         <v>44623</v>
       </c>
       <c r="B253" t="n">
-        <v>12.56655406951904</v>
+        <v>12.56655502319336</v>
       </c>
       <c r="C253" t="n">
-        <v>12.95836375658081</v>
+        <v>12.95836473998952</v>
       </c>
       <c r="D253" t="n">
-        <v>12.33720272443013</v>
+        <v>12.337203660699</v>
       </c>
       <c r="E253" t="n">
-        <v>12.80546194849363</v>
+        <v>12.80546292029864</v>
       </c>
       <c r="F253" t="n">
         <v>12631200</v>
@@ -5512,16 +5512,16 @@
         <v>44627</v>
       </c>
       <c r="B255" t="n">
-        <v>11.73515701293945</v>
+        <v>11.73515605926514</v>
       </c>
       <c r="C255" t="n">
-        <v>12.17474763109875</v>
+        <v>12.17474664170048</v>
       </c>
       <c r="D255" t="n">
-        <v>11.68737524569925</v>
+        <v>11.68737429590799</v>
       </c>
       <c r="E255" t="n">
-        <v>12.08874063233868</v>
+        <v>12.08873964992988</v>
       </c>
       <c r="F255" t="n">
         <v>12255900</v>
@@ -5532,16 +5532,16 @@
         <v>44628</v>
       </c>
       <c r="B256" t="n">
-        <v>11.75427055358887</v>
+        <v>11.75426959991455</v>
       </c>
       <c r="C256" t="n">
-        <v>11.99317848796522</v>
+        <v>11.99317751490728</v>
       </c>
       <c r="D256" t="n">
-        <v>11.52491915531431</v>
+        <v>11.52491822024826</v>
       </c>
       <c r="E256" t="n">
-        <v>11.74471401748707</v>
+        <v>11.74471306458811</v>
       </c>
       <c r="F256" t="n">
         <v>10151100</v>
@@ -5612,16 +5612,16 @@
         <v>44634</v>
       </c>
       <c r="B260" t="n">
-        <v>12.51877498626709</v>
+        <v>12.51877403259277</v>
       </c>
       <c r="C260" t="n">
-        <v>12.74812636366353</v>
+        <v>12.74812539251733</v>
       </c>
       <c r="D260" t="n">
-        <v>12.38498622710516</v>
+        <v>12.3849852836228</v>
       </c>
       <c r="E260" t="n">
-        <v>12.43276799190309</v>
+        <v>12.43276704478074</v>
       </c>
       <c r="F260" t="n">
         <v>4274300</v>
@@ -5632,16 +5632,16 @@
         <v>44635</v>
       </c>
       <c r="B261" t="n">
-        <v>12.82457542419434</v>
+        <v>12.82457637786865</v>
       </c>
       <c r="C261" t="n">
-        <v>12.90102587498907</v>
+        <v>12.90102683434848</v>
       </c>
       <c r="D261" t="n">
-        <v>12.29897789145957</v>
+        <v>12.29897880604886</v>
       </c>
       <c r="E261" t="n">
-        <v>12.29897789145957</v>
+        <v>12.29897880604886</v>
       </c>
       <c r="F261" t="n">
         <v>8181800</v>
@@ -5652,16 +5652,16 @@
         <v>44636</v>
       </c>
       <c r="B262" t="n">
-        <v>12.99659156799316</v>
+        <v>12.99659061431885</v>
       </c>
       <c r="C262" t="n">
-        <v>13.09215419178991</v>
+        <v>13.09215323110332</v>
       </c>
       <c r="D262" t="n">
-        <v>12.73857056988299</v>
+        <v>12.73856963514194</v>
       </c>
       <c r="E262" t="n">
-        <v>12.91058456862311</v>
+        <v>12.91058362125988</v>
       </c>
       <c r="F262" t="n">
         <v>7731200</v>
@@ -5672,16 +5672,16 @@
         <v>44637</v>
       </c>
       <c r="B263" t="n">
-        <v>13.12082099914551</v>
+        <v>13.12082195281982</v>
       </c>
       <c r="C263" t="n">
-        <v>13.24505321242422</v>
+        <v>13.24505417512824</v>
       </c>
       <c r="D263" t="n">
-        <v>12.87235748394937</v>
+        <v>12.87235841956435</v>
       </c>
       <c r="E263" t="n">
-        <v>13.09215230726928</v>
+        <v>13.09215325885984</v>
       </c>
       <c r="F263" t="n">
         <v>6159800</v>
@@ -5752,16 +5752,16 @@
         <v>44643</v>
       </c>
       <c r="B267" t="n">
-        <v>14.38225650787354</v>
+        <v>14.38225555419922</v>
       </c>
       <c r="C267" t="n">
-        <v>14.59249572595387</v>
+        <v>14.59249475833878</v>
       </c>
       <c r="D267" t="n">
-        <v>13.87577198879766</v>
+        <v>13.87577106870787</v>
       </c>
       <c r="E267" t="n">
-        <v>14.0286729069065</v>
+        <v>14.02867197667799</v>
       </c>
       <c r="F267" t="n">
         <v>8813400</v>
@@ -5832,16 +5832,16 @@
         <v>44649</v>
       </c>
       <c r="B271" t="n">
-        <v>15.50034523010254</v>
+        <v>15.50034427642822</v>
       </c>
       <c r="C271" t="n">
-        <v>15.93038021620936</v>
+        <v>15.93037923607671</v>
       </c>
       <c r="D271" t="n">
-        <v>15.43345130397987</v>
+        <v>15.43345035442127</v>
       </c>
       <c r="E271" t="n">
-        <v>15.72969661511858</v>
+        <v>15.72969564733319</v>
       </c>
       <c r="F271" t="n">
         <v>7323700</v>
@@ -5892,16 +5892,16 @@
         <v>44652</v>
       </c>
       <c r="B274" t="n">
-        <v>15.74880695343018</v>
+        <v>15.74880599975586</v>
       </c>
       <c r="C274" t="n">
-        <v>15.97815829864838</v>
+        <v>15.97815733108562</v>
       </c>
       <c r="D274" t="n">
-        <v>15.4716747614791</v>
+        <v>15.47167382458661</v>
       </c>
       <c r="E274" t="n">
-        <v>15.72013917447944</v>
+        <v>15.72013822254111</v>
       </c>
       <c r="F274" t="n">
         <v>8302400</v>
@@ -5992,16 +5992,16 @@
         <v>44659</v>
       </c>
       <c r="B279" t="n">
-        <v>15.40478229522705</v>
+        <v>15.40478134155273</v>
       </c>
       <c r="C279" t="n">
-        <v>15.57679445327038</v>
+        <v>15.5767934889472</v>
       </c>
       <c r="D279" t="n">
-        <v>15.07031086848462</v>
+        <v>15.07030993551665</v>
       </c>
       <c r="E279" t="n">
-        <v>15.32833183963358</v>
+        <v>15.32833089069213</v>
       </c>
       <c r="F279" t="n">
         <v>3069100</v>
@@ -6012,16 +6012,16 @@
         <v>44662</v>
       </c>
       <c r="B280" t="n">
-        <v>15.29010581970215</v>
+        <v>15.29010677337646</v>
       </c>
       <c r="C280" t="n">
-        <v>15.49078758367887</v>
+        <v>15.4907885498701</v>
       </c>
       <c r="D280" t="n">
-        <v>15.21365536351254</v>
+        <v>15.21365631241849</v>
       </c>
       <c r="E280" t="n">
-        <v>15.38566934561982</v>
+        <v>15.38567030525462</v>
       </c>
       <c r="F280" t="n">
         <v>10289300</v>
@@ -6032,16 +6032,16 @@
         <v>44663</v>
       </c>
       <c r="B281" t="n">
-        <v>15.720139503479</v>
+        <v>15.72014141082764</v>
       </c>
       <c r="C281" t="n">
-        <v>15.82525773303578</v>
+        <v>15.82525965313857</v>
       </c>
       <c r="D281" t="n">
-        <v>15.3952246352726</v>
+        <v>15.39522650319881</v>
       </c>
       <c r="E281" t="n">
-        <v>15.48123161936973</v>
+        <v>15.48123349773131</v>
       </c>
       <c r="F281" t="n">
         <v>9798400</v>
@@ -6052,16 +6052,16 @@
         <v>44664</v>
       </c>
       <c r="B282" t="n">
-        <v>15.76792335510254</v>
+        <v>15.76792144775391</v>
       </c>
       <c r="C282" t="n">
-        <v>16.02594435654861</v>
+        <v>16.02594241798877</v>
       </c>
       <c r="D282" t="n">
-        <v>15.69147289053217</v>
+        <v>15.69147099243128</v>
       </c>
       <c r="E282" t="n">
-        <v>15.78703642692584</v>
+        <v>15.78703451726522</v>
       </c>
       <c r="F282" t="n">
         <v>7212700</v>
@@ -6072,16 +6072,16 @@
         <v>44665</v>
       </c>
       <c r="B283" t="n">
-        <v>15.64369106292725</v>
+        <v>15.64369201660156</v>
       </c>
       <c r="C283" t="n">
-        <v>15.79659198257972</v>
+        <v>15.79659294557522</v>
       </c>
       <c r="D283" t="n">
-        <v>15.48123360795615</v>
+        <v>15.4812345517267</v>
       </c>
       <c r="E283" t="n">
-        <v>15.72014152275348</v>
+        <v>15.72014248108839</v>
       </c>
       <c r="F283" t="n">
         <v>4607000</v>
@@ -6092,16 +6092,16 @@
         <v>44669</v>
       </c>
       <c r="B284" t="n">
-        <v>15.3187780380249</v>
+        <v>15.31877708435059</v>
       </c>
       <c r="C284" t="n">
-        <v>15.67236077471006</v>
+        <v>15.67235979902336</v>
       </c>
       <c r="D284" t="n">
-        <v>15.3187780380249</v>
+        <v>15.31877708435059</v>
       </c>
       <c r="E284" t="n">
-        <v>15.56724251871545</v>
+        <v>15.56724154957292</v>
       </c>
       <c r="F284" t="n">
         <v>3539900</v>
@@ -6112,16 +6112,16 @@
         <v>44670</v>
       </c>
       <c r="B285" t="n">
-        <v>15.61502170562744</v>
+        <v>15.61502075195312</v>
       </c>
       <c r="C285" t="n">
-        <v>15.77747916318553</v>
+        <v>15.77747819958926</v>
       </c>
       <c r="D285" t="n">
-        <v>15.18498763441659</v>
+        <v>15.18498670700624</v>
       </c>
       <c r="E285" t="n">
-        <v>15.32833293239446</v>
+        <v>15.32833199622942</v>
       </c>
       <c r="F285" t="n">
         <v>7756800</v>
@@ -6152,16 +6152,16 @@
         <v>44673</v>
       </c>
       <c r="B287" t="n">
-        <v>15.3187780380249</v>
+        <v>15.31877708435059</v>
       </c>
       <c r="C287" t="n">
-        <v>15.74881124394384</v>
+        <v>15.7488102634977</v>
       </c>
       <c r="D287" t="n">
-        <v>15.14676402656814</v>
+        <v>15.1467630836026</v>
       </c>
       <c r="E287" t="n">
-        <v>15.74881124394384</v>
+        <v>15.7488102634977</v>
       </c>
       <c r="F287" t="n">
         <v>8878800</v>
@@ -6192,16 +6192,16 @@
         <v>44677</v>
       </c>
       <c r="B289" t="n">
-        <v>15.12764930725098</v>
+        <v>15.12765026092529</v>
       </c>
       <c r="C289" t="n">
-        <v>15.30921983544218</v>
+        <v>15.30922080056303</v>
       </c>
       <c r="D289" t="n">
-        <v>15.02253015133491</v>
+        <v>15.02253109838233</v>
       </c>
       <c r="E289" t="n">
-        <v>15.2136563036193</v>
+        <v>15.21365726271565</v>
       </c>
       <c r="F289" t="n">
         <v>9387600</v>
@@ -6232,16 +6232,16 @@
         <v>44679</v>
       </c>
       <c r="B291" t="n">
-        <v>14.84096050262451</v>
+        <v>14.8409595489502</v>
       </c>
       <c r="C291" t="n">
-        <v>15.3856712081165</v>
+        <v>15.38567021943929</v>
       </c>
       <c r="D291" t="n">
-        <v>14.84096050262451</v>
+        <v>14.8409595489502</v>
       </c>
       <c r="E291" t="n">
-        <v>15.32833381471404</v>
+        <v>15.3283328297213</v>
       </c>
       <c r="F291" t="n">
         <v>5384600</v>
@@ -6272,16 +6272,16 @@
         <v>44683</v>
       </c>
       <c r="B293" t="n">
-        <v>14.69167137145996</v>
+        <v>14.69167041778564</v>
       </c>
       <c r="C293" t="n">
-        <v>14.97105393783902</v>
+        <v>14.97105296602926</v>
       </c>
       <c r="D293" t="n">
-        <v>14.44119019642807</v>
+        <v>14.44118925901314</v>
       </c>
       <c r="E293" t="n">
-        <v>14.54716349596546</v>
+        <v>14.54716255167152</v>
       </c>
       <c r="F293" t="n">
         <v>5536000</v>
@@ -6292,16 +6292,16 @@
         <v>44684</v>
       </c>
       <c r="B294" t="n">
-        <v>14.62423419952393</v>
+        <v>14.62423324584961</v>
       </c>
       <c r="C294" t="n">
-        <v>14.85544716329886</v>
+        <v>14.85544619454671</v>
       </c>
       <c r="D294" t="n">
-        <v>14.4797254080956</v>
+        <v>14.47972446384498</v>
       </c>
       <c r="E294" t="n">
-        <v>14.70130518744891</v>
+        <v>14.70130422874864</v>
       </c>
       <c r="F294" t="n">
         <v>5388000</v>
@@ -6372,16 +6372,16 @@
         <v>44690</v>
       </c>
       <c r="B298" t="n">
-        <v>14.21961116790771</v>
+        <v>14.21961212158203</v>
       </c>
       <c r="C298" t="n">
-        <v>14.32558354746724</v>
+        <v>14.32558450824887</v>
       </c>
       <c r="D298" t="n">
-        <v>13.92096039822737</v>
+        <v>13.92096133187191</v>
       </c>
       <c r="E298" t="n">
-        <v>14.04620098430244</v>
+        <v>14.04620192634656</v>
       </c>
       <c r="F298" t="n">
         <v>11844800</v>
@@ -6392,16 +6392,16 @@
         <v>44691</v>
       </c>
       <c r="B299" t="n">
-        <v>14.71093845367432</v>
+        <v>14.71093940734863</v>
       </c>
       <c r="C299" t="n">
-        <v>14.97105279343268</v>
+        <v>14.97105376396958</v>
       </c>
       <c r="D299" t="n">
-        <v>14.14253926099675</v>
+        <v>14.14254017782313</v>
       </c>
       <c r="E299" t="n">
-        <v>14.2196102445369</v>
+        <v>14.21961116635961</v>
       </c>
       <c r="F299" t="n">
         <v>13119700</v>
@@ -6452,16 +6452,16 @@
         <v>44694</v>
       </c>
       <c r="B302" t="n">
-        <v>14.91324996948242</v>
+        <v>14.91324901580811</v>
       </c>
       <c r="C302" t="n">
-        <v>15.09629425517541</v>
+        <v>15.09629328979575</v>
       </c>
       <c r="D302" t="n">
-        <v>14.62423422366596</v>
+        <v>14.62423328847366</v>
       </c>
       <c r="E302" t="n">
-        <v>14.7205724993519</v>
+        <v>14.72057155799894</v>
       </c>
       <c r="F302" t="n">
         <v>5016200</v>
@@ -6572,16 +6572,16 @@
         <v>44704</v>
       </c>
       <c r="B308" t="n">
-        <v>15.28897285461426</v>
+        <v>15.28897190093994</v>
       </c>
       <c r="C308" t="n">
-        <v>15.63579232646676</v>
+        <v>15.63579135115902</v>
       </c>
       <c r="D308" t="n">
-        <v>15.17336636399676</v>
+        <v>15.17336541753358</v>
       </c>
       <c r="E308" t="n">
-        <v>15.52982085851578</v>
+        <v>15.52981988981818</v>
       </c>
       <c r="F308" t="n">
         <v>8474400</v>
@@ -6612,16 +6612,16 @@
         <v>44706</v>
       </c>
       <c r="B310" t="n">
-        <v>15.14446258544922</v>
+        <v>15.1444616317749</v>
       </c>
       <c r="C310" t="n">
-        <v>15.44311332823613</v>
+        <v>15.44311235575524</v>
       </c>
       <c r="D310" t="n">
-        <v>14.94215102904739</v>
+        <v>14.942150088113</v>
       </c>
       <c r="E310" t="n">
-        <v>15.16372987147109</v>
+        <v>15.16372891658348</v>
       </c>
       <c r="F310" t="n">
         <v>8129200</v>
@@ -6652,16 +6652,16 @@
         <v>44708</v>
       </c>
       <c r="B312" t="n">
-        <v>15.22153472900391</v>
+        <v>15.22153377532959</v>
       </c>
       <c r="C312" t="n">
-        <v>15.51055139146295</v>
+        <v>15.51055041968089</v>
       </c>
       <c r="D312" t="n">
-        <v>15.13482963839033</v>
+        <v>15.13482869014834</v>
       </c>
       <c r="E312" t="n">
-        <v>15.43348040397503</v>
+        <v>15.43347943702168</v>
       </c>
       <c r="F312" t="n">
         <v>3408100</v>
@@ -6692,16 +6692,16 @@
         <v>44712</v>
       </c>
       <c r="B314" t="n">
-        <v>15.26006984710693</v>
+        <v>15.26007080078125</v>
       </c>
       <c r="C314" t="n">
-        <v>15.39494361251144</v>
+        <v>15.39494457461466</v>
       </c>
       <c r="D314" t="n">
-        <v>15.05775828024155</v>
+        <v>15.05775922127246</v>
       </c>
       <c r="E314" t="n">
-        <v>15.29860533990231</v>
+        <v>15.29860629598489</v>
       </c>
       <c r="F314" t="n">
         <v>5708500</v>
@@ -6712,16 +6712,16 @@
         <v>44713</v>
       </c>
       <c r="B315" t="n">
-        <v>14.85544586181641</v>
+        <v>14.85544681549072</v>
       </c>
       <c r="C315" t="n">
-        <v>15.53945059003543</v>
+        <v>15.53945158762076</v>
       </c>
       <c r="D315" t="n">
-        <v>14.73020528772095</v>
+        <v>14.73020623335521</v>
       </c>
       <c r="E315" t="n">
-        <v>15.39494273002606</v>
+        <v>15.39494371833443</v>
       </c>
       <c r="F315" t="n">
         <v>6096700</v>
@@ -6732,16 +6732,16 @@
         <v>44714</v>
       </c>
       <c r="B316" t="n">
-        <v>15.30823993682861</v>
+        <v>15.30824089050293</v>
       </c>
       <c r="C316" t="n">
-        <v>15.41421231574625</v>
+        <v>15.41421327602245</v>
       </c>
       <c r="D316" t="n">
-        <v>14.88434858364075</v>
+        <v>14.88434951090744</v>
       </c>
       <c r="E316" t="n">
-        <v>15.06739286939508</v>
+        <v>15.06739380806508</v>
       </c>
       <c r="F316" t="n">
         <v>5285700</v>
@@ -6852,16 +6852,16 @@
         <v>44722</v>
       </c>
       <c r="B322" t="n">
-        <v>14.48935985565186</v>
+        <v>14.48936080932617</v>
       </c>
       <c r="C322" t="n">
-        <v>15.01922359929862</v>
+        <v>15.019224587848</v>
       </c>
       <c r="D322" t="n">
-        <v>14.22924549491244</v>
+        <v>14.22924643146631</v>
       </c>
       <c r="E322" t="n">
-        <v>14.85544751637582</v>
+        <v>14.85544849414564</v>
       </c>
       <c r="F322" t="n">
         <v>15101900</v>
@@ -6872,16 +6872,16 @@
         <v>44725</v>
       </c>
       <c r="B323" t="n">
-        <v>14.03656578063965</v>
+        <v>14.03656673431396</v>
       </c>
       <c r="C323" t="n">
-        <v>14.35448381315351</v>
+        <v>14.35448478842786</v>
       </c>
       <c r="D323" t="n">
-        <v>13.89205791813647</v>
+        <v>13.89205886199261</v>
       </c>
       <c r="E323" t="n">
-        <v>14.25814554440425</v>
+        <v>14.25814651313317</v>
       </c>
       <c r="F323" t="n">
         <v>9104400</v>
@@ -6912,16 +6912,16 @@
         <v>44727</v>
       </c>
       <c r="B325" t="n">
-        <v>14.91324996948242</v>
+        <v>14.91324901580811</v>
       </c>
       <c r="C325" t="n">
-        <v>15.06739286434549</v>
+        <v>15.06739190081403</v>
       </c>
       <c r="D325" t="n">
-        <v>14.25814657103863</v>
+        <v>14.25814565925695</v>
       </c>
       <c r="E325" t="n">
-        <v>14.34485166228703</v>
+        <v>14.34485074496072</v>
       </c>
       <c r="F325" t="n">
         <v>25461900</v>
@@ -6932,16 +6932,16 @@
         <v>44729</v>
       </c>
       <c r="B326" t="n">
-        <v>14.94215202331543</v>
+        <v>14.94215297698975</v>
       </c>
       <c r="C326" t="n">
-        <v>15.18299908654582</v>
+        <v>15.18300005559206</v>
       </c>
       <c r="D326" t="n">
-        <v>14.56643027392291</v>
+        <v>14.56643120361701</v>
       </c>
       <c r="E326" t="n">
-        <v>14.63386715762466</v>
+        <v>14.63386809162287</v>
       </c>
       <c r="F326" t="n">
         <v>14099900</v>
@@ -6972,16 +6972,16 @@
         <v>44733</v>
       </c>
       <c r="B328" t="n">
-        <v>14.84581279754639</v>
+        <v>14.84581184387207</v>
       </c>
       <c r="C328" t="n">
-        <v>15.6454249721946</v>
+        <v>15.64542396715431</v>
       </c>
       <c r="D328" t="n">
-        <v>14.81691140727535</v>
+        <v>14.81691045545762</v>
       </c>
       <c r="E328" t="n">
-        <v>15.37567651922811</v>
+        <v>15.37567553151609</v>
       </c>
       <c r="F328" t="n">
         <v>9398400</v>
@@ -7032,16 +7032,16 @@
         <v>44736</v>
       </c>
       <c r="B331" t="n">
-        <v>14.4219217300415</v>
+        <v>14.42192268371582</v>
       </c>
       <c r="C331" t="n">
-        <v>14.86508034244202</v>
+        <v>14.86508132542095</v>
       </c>
       <c r="D331" t="n">
-        <v>14.25814566119184</v>
+        <v>14.25814660403618</v>
       </c>
       <c r="E331" t="n">
-        <v>14.86508034244202</v>
+        <v>14.86508132542095</v>
       </c>
       <c r="F331" t="n">
         <v>5803600</v>
@@ -7052,16 +7052,16 @@
         <v>44739</v>
       </c>
       <c r="B332" t="n">
-        <v>14.16180801391602</v>
+        <v>14.1618070602417</v>
       </c>
       <c r="C332" t="n">
-        <v>14.49899429088777</v>
+        <v>14.4989933145069</v>
       </c>
       <c r="D332" t="n">
-        <v>14.10400522965489</v>
+        <v>14.10400427987309</v>
       </c>
       <c r="E332" t="n">
-        <v>14.47972608362827</v>
+        <v>14.47972510854494</v>
       </c>
       <c r="F332" t="n">
         <v>8041800</v>
@@ -7092,16 +7092,16 @@
         <v>44741</v>
       </c>
       <c r="B334" t="n">
-        <v>13.85352325439453</v>
+        <v>13.85352230072021</v>
       </c>
       <c r="C334" t="n">
-        <v>14.1810754089765</v>
+        <v>14.18107443275354</v>
       </c>
       <c r="D334" t="n">
-        <v>13.5934079838411</v>
+        <v>13.59340704807308</v>
       </c>
       <c r="E334" t="n">
-        <v>14.1810754089765</v>
+        <v>14.18107443275354</v>
       </c>
       <c r="F334" t="n">
         <v>8408900</v>
@@ -7132,16 +7132,16 @@
         <v>44743</v>
       </c>
       <c r="B336" t="n">
-        <v>14.06546878814697</v>
+        <v>14.06546974182129</v>
       </c>
       <c r="C336" t="n">
-        <v>14.28704764418037</v>
+        <v>14.28704861287829</v>
       </c>
       <c r="D336" t="n">
-        <v>13.54523917098311</v>
+        <v>13.54524008938454</v>
       </c>
       <c r="E336" t="n">
-        <v>13.64157744452686</v>
+        <v>13.64157836946027</v>
       </c>
       <c r="F336" t="n">
         <v>10271400</v>
@@ -7152,16 +7152,16 @@
         <v>44746</v>
       </c>
       <c r="B337" t="n">
-        <v>13.8727912902832</v>
+        <v>13.87279033660889</v>
       </c>
       <c r="C337" t="n">
-        <v>14.14254067846864</v>
+        <v>14.14253970625061</v>
       </c>
       <c r="D337" t="n">
-        <v>13.76681890698379</v>
+        <v>13.76681796059447</v>
       </c>
       <c r="E337" t="n">
-        <v>13.95949638514576</v>
+        <v>13.95949542551097</v>
       </c>
       <c r="F337" t="n">
         <v>1980900</v>
@@ -7172,16 +7172,16 @@
         <v>44747</v>
       </c>
       <c r="B338" t="n">
-        <v>14.17144107818604</v>
+        <v>14.17144012451172</v>
       </c>
       <c r="C338" t="n">
-        <v>14.19070836527375</v>
+        <v>14.19070741030283</v>
       </c>
       <c r="D338" t="n">
-        <v>13.46816718369137</v>
+        <v>13.46816627734423</v>
       </c>
       <c r="E338" t="n">
-        <v>13.67047875128478</v>
+        <v>13.67047783132298</v>
       </c>
       <c r="F338" t="n">
         <v>7354200</v>
@@ -7192,16 +7192,16 @@
         <v>44748</v>
       </c>
       <c r="B339" t="n">
-        <v>14.35448455810547</v>
+        <v>14.35448551177979</v>
       </c>
       <c r="C339" t="n">
-        <v>14.63386711386697</v>
+        <v>14.63386808610274</v>
       </c>
       <c r="D339" t="n">
-        <v>13.9209600293388</v>
+        <v>13.92096095421089</v>
       </c>
       <c r="E339" t="n">
-        <v>13.96912962559257</v>
+        <v>13.96913055366492</v>
       </c>
       <c r="F339" t="n">
         <v>11107300</v>
@@ -7252,16 +7252,16 @@
         <v>44753</v>
       </c>
       <c r="B342" t="n">
-        <v>14.78800964355469</v>
+        <v>14.788010597229</v>
       </c>
       <c r="C342" t="n">
-        <v>14.8939820177114</v>
+        <v>14.89398297821984</v>
       </c>
       <c r="D342" t="n">
-        <v>14.52789438140829</v>
+        <v>14.52789531830785</v>
       </c>
       <c r="E342" t="n">
-        <v>14.57606397648265</v>
+        <v>14.57606491648865</v>
       </c>
       <c r="F342" t="n">
         <v>3654100</v>
@@ -7312,16 +7312,16 @@
         <v>44756</v>
       </c>
       <c r="B345" t="n">
-        <v>14.75910758972168</v>
+        <v>14.75910663604736</v>
       </c>
       <c r="C345" t="n">
-        <v>14.99995465048742</v>
+        <v>14.99995368125053</v>
       </c>
       <c r="D345" t="n">
-        <v>14.51826052895594</v>
+        <v>14.5182595908442</v>
       </c>
       <c r="E345" t="n">
-        <v>14.52789463188864</v>
+        <v>14.52789369315438</v>
       </c>
       <c r="F345" t="n">
         <v>8175300</v>
@@ -7332,16 +7332,16 @@
         <v>44757</v>
       </c>
       <c r="B346" t="n">
-        <v>15.00958824157715</v>
+        <v>15.00958919525146</v>
       </c>
       <c r="C346" t="n">
-        <v>15.16373020820944</v>
+        <v>15.16373117167757</v>
       </c>
       <c r="D346" t="n">
-        <v>14.56642962813003</v>
+        <v>14.56643055364708</v>
       </c>
       <c r="E346" t="n">
-        <v>14.83617806973653</v>
+        <v>14.83617901239277</v>
       </c>
       <c r="F346" t="n">
         <v>3973400</v>
@@ -7352,16 +7352,16 @@
         <v>44760</v>
       </c>
       <c r="B347" t="n">
-        <v>14.87471294403076</v>
+        <v>14.87471389770508</v>
       </c>
       <c r="C347" t="n">
-        <v>15.19263188546311</v>
+        <v>15.19263285952041</v>
       </c>
       <c r="D347" t="n">
-        <v>14.8072760661177</v>
+        <v>14.80727701546838</v>
       </c>
       <c r="E347" t="n">
-        <v>15.0770244965285</v>
+        <v>15.07702546317377</v>
       </c>
       <c r="F347" t="n">
         <v>3805700</v>
@@ -7392,16 +7392,16 @@
         <v>44762</v>
       </c>
       <c r="B349" t="n">
-        <v>14.82654571533203</v>
+        <v>14.82654476165771</v>
       </c>
       <c r="C349" t="n">
-        <v>15.10592827517219</v>
+        <v>15.10592730352741</v>
       </c>
       <c r="D349" t="n">
-        <v>14.57606454616261</v>
+        <v>14.57606360859976</v>
       </c>
       <c r="E349" t="n">
-        <v>14.89398259981663</v>
+        <v>14.89398164180463</v>
       </c>
       <c r="F349" t="n">
         <v>5599700</v>
@@ -7412,16 +7412,16 @@
         <v>44763</v>
       </c>
       <c r="B350" t="n">
-        <v>14.84581279754639</v>
+        <v>14.84581184387207</v>
       </c>
       <c r="C350" t="n">
-        <v>14.95178609313791</v>
+        <v>14.95178513265602</v>
       </c>
       <c r="D350" t="n">
-        <v>14.60496573485093</v>
+        <v>14.6049647966483</v>
       </c>
       <c r="E350" t="n">
-        <v>14.74947452372338</v>
+        <v>14.7494735762377</v>
       </c>
       <c r="F350" t="n">
         <v>4662200</v>
@@ -7472,16 +7472,16 @@
         <v>44768</v>
       </c>
       <c r="B353" t="n">
-        <v>14.95178508758545</v>
+        <v>14.95178604125977</v>
       </c>
       <c r="C353" t="n">
-        <v>15.03848925256745</v>
+        <v>15.03849021177204</v>
       </c>
       <c r="D353" t="n">
-        <v>14.76874081774235</v>
+        <v>14.76874175974149</v>
       </c>
       <c r="E353" t="n">
-        <v>14.82654451315558</v>
+        <v>14.82654545884164</v>
       </c>
       <c r="F353" t="n">
         <v>3874000</v>
@@ -7632,16 +7632,16 @@
         <v>44778</v>
       </c>
       <c r="B361" t="n">
-        <v>16.40650367736816</v>
+        <v>16.40650177001953</v>
       </c>
       <c r="C361" t="n">
-        <v>16.57027976453278</v>
+        <v>16.57027783814425</v>
       </c>
       <c r="D361" t="n">
-        <v>16.10785197649791</v>
+        <v>16.10785010386923</v>
       </c>
       <c r="E361" t="n">
-        <v>16.26199396000374</v>
+        <v>16.26199206945518</v>
       </c>
       <c r="F361" t="n">
         <v>6244900</v>
@@ -7652,16 +7652,16 @@
         <v>44781</v>
       </c>
       <c r="B362" t="n">
-        <v>16.68588256835938</v>
+        <v>16.68588447570801</v>
       </c>
       <c r="C362" t="n">
-        <v>16.88819503663362</v>
+        <v>16.88819696710841</v>
       </c>
       <c r="D362" t="n">
-        <v>16.26199126520336</v>
+        <v>16.26199312409735</v>
       </c>
       <c r="E362" t="n">
-        <v>16.53174061039666</v>
+        <v>16.53174250012546</v>
       </c>
       <c r="F362" t="n">
         <v>10381400</v>
@@ -7672,16 +7672,16 @@
         <v>44782</v>
       </c>
       <c r="B363" t="n">
-        <v>16.61844825744629</v>
+        <v>16.61845016479492</v>
       </c>
       <c r="C363" t="n">
-        <v>16.87856354074092</v>
+        <v>16.87856547794376</v>
       </c>
       <c r="D363" t="n">
-        <v>16.51247495591499</v>
+        <v>16.51247685110075</v>
       </c>
       <c r="E363" t="n">
-        <v>16.65698467164581</v>
+        <v>16.65698658341738</v>
       </c>
       <c r="F363" t="n">
         <v>6314800</v>
@@ -7712,16 +7712,16 @@
         <v>44784</v>
       </c>
       <c r="B365" t="n">
-        <v>16.99416732788086</v>
+        <v>16.99416923522949</v>
       </c>
       <c r="C365" t="n">
-        <v>17.34098766927179</v>
+        <v>17.34098961554597</v>
       </c>
       <c r="D365" t="n">
-        <v>16.86892766988812</v>
+        <v>16.86892956318042</v>
       </c>
       <c r="E365" t="n">
-        <v>16.91709634507367</v>
+        <v>16.91709824377221</v>
       </c>
       <c r="F365" t="n">
         <v>8667500</v>
@@ -7732,16 +7732,16 @@
         <v>44785</v>
       </c>
       <c r="B366" t="n">
-        <v>17.34099006652832</v>
+        <v>17.34098815917969</v>
       </c>
       <c r="C366" t="n">
-        <v>17.64927404037492</v>
+        <v>17.6492720991179</v>
       </c>
       <c r="D366" t="n">
-        <v>17.06160656678144</v>
+        <v>17.06160469016241</v>
       </c>
       <c r="E366" t="n">
-        <v>17.16757987186025</v>
+        <v>17.16757798358513</v>
       </c>
       <c r="F366" t="n">
         <v>11729000</v>
@@ -7832,16 +7832,16 @@
         <v>44792</v>
       </c>
       <c r="B371" t="n">
-        <v>17.12904167175293</v>
+        <v>17.12904357910156</v>
       </c>
       <c r="C371" t="n">
-        <v>17.57219933106722</v>
+        <v>17.57220128776223</v>
       </c>
       <c r="D371" t="n">
-        <v>17.07123706074208</v>
+        <v>17.07123896165407</v>
       </c>
       <c r="E371" t="n">
-        <v>17.4565937840796</v>
+        <v>17.45659572790173</v>
       </c>
       <c r="F371" t="n">
         <v>7571900</v>
@@ -8012,16 +8012,16 @@
         <v>44805</v>
       </c>
       <c r="B380" t="n">
-        <v>18.08279800415039</v>
+        <v>18.08279609680176</v>
       </c>
       <c r="C380" t="n">
-        <v>18.24657408115321</v>
+        <v>18.2465721565297</v>
       </c>
       <c r="D380" t="n">
-        <v>17.71670943790068</v>
+        <v>17.71670756916656</v>
       </c>
       <c r="E380" t="n">
-        <v>17.81304863099362</v>
+        <v>17.81304675209778</v>
       </c>
       <c r="F380" t="n">
         <v>12942800</v>
@@ -8032,16 +8032,16 @@
         <v>44806</v>
       </c>
       <c r="B381" t="n">
-        <v>18.20803833007812</v>
+        <v>18.20803642272949</v>
       </c>
       <c r="C381" t="n">
-        <v>18.54522459938866</v>
+        <v>18.54522265671872</v>
       </c>
       <c r="D381" t="n">
-        <v>17.95755715394794</v>
+        <v>17.95755527283799</v>
       </c>
       <c r="E381" t="n">
-        <v>18.20803833007812</v>
+        <v>18.20803642272949</v>
       </c>
       <c r="F381" t="n">
         <v>12423600</v>
@@ -8052,16 +8052,16 @@
         <v>44809</v>
       </c>
       <c r="B382" t="n">
-        <v>18.73790168762207</v>
+        <v>18.7379035949707</v>
       </c>
       <c r="C382" t="n">
-        <v>18.91131002438889</v>
+        <v>18.91131194938891</v>
       </c>
       <c r="D382" t="n">
-        <v>18.12133197488807</v>
+        <v>18.12133381947549</v>
       </c>
       <c r="E382" t="n">
-        <v>18.39108133905402</v>
+        <v>18.39108321109948</v>
       </c>
       <c r="F382" t="n">
         <v>11861400</v>
@@ -8092,16 +8092,16 @@
         <v>44812</v>
       </c>
       <c r="B384" t="n">
-        <v>18.40071487426758</v>
+        <v>18.40071678161621</v>
       </c>
       <c r="C384" t="n">
-        <v>18.94984585088554</v>
+        <v>18.94984781515502</v>
       </c>
       <c r="D384" t="n">
-        <v>18.3429120971281</v>
+        <v>18.34291399848511</v>
       </c>
       <c r="E384" t="n">
-        <v>18.91130944111445</v>
+        <v>18.91131140138939</v>
       </c>
       <c r="F384" t="n">
         <v>6653400</v>
@@ -8172,16 +8172,16 @@
         <v>44818</v>
       </c>
       <c r="B388" t="n">
-        <v>17.70707511901855</v>
+        <v>17.70707321166992</v>
       </c>
       <c r="C388" t="n">
-        <v>17.8708511940252</v>
+        <v>17.87084926903514</v>
       </c>
       <c r="D388" t="n">
-        <v>17.36989070357892</v>
+        <v>17.3698888325507</v>
       </c>
       <c r="E388" t="n">
-        <v>17.44696168961044</v>
+        <v>17.44695981028038</v>
       </c>
       <c r="F388" t="n">
         <v>7347400</v>
@@ -8352,16 +8352,16 @@
         <v>44831</v>
       </c>
       <c r="B397" t="n">
-        <v>17.12904167175293</v>
+        <v>17.12904357910156</v>
       </c>
       <c r="C397" t="n">
-        <v>17.49512835390313</v>
+        <v>17.49513030201615</v>
       </c>
       <c r="D397" t="n">
-        <v>16.86892643475522</v>
+        <v>16.86892831313957</v>
       </c>
       <c r="E397" t="n">
-        <v>17.2542813205757</v>
+        <v>17.25428324186998</v>
       </c>
       <c r="F397" t="n">
         <v>9260100</v>
@@ -8512,16 +8512,16 @@
         <v>44841</v>
       </c>
       <c r="B405" t="n">
-        <v>17.49513053894043</v>
+        <v>17.49513244628906</v>
       </c>
       <c r="C405" t="n">
-        <v>17.68780892467357</v>
+        <v>17.68781085302832</v>
       </c>
       <c r="D405" t="n">
-        <v>17.32172035928406</v>
+        <v>17.32172224772722</v>
       </c>
       <c r="E405" t="n">
-        <v>17.44696186126578</v>
+        <v>17.44696376336298</v>
       </c>
       <c r="F405" t="n">
         <v>11897600</v>
@@ -8532,16 +8532,16 @@
         <v>44844</v>
       </c>
       <c r="B406" t="n">
-        <v>18.10206604003906</v>
+        <v>18.1020679473877</v>
       </c>
       <c r="C406" t="n">
-        <v>18.12133240846265</v>
+        <v>18.12133431784131</v>
       </c>
       <c r="D406" t="n">
-        <v>17.58183550473985</v>
+        <v>17.58183735727369</v>
       </c>
       <c r="E406" t="n">
-        <v>17.73597747723208</v>
+        <v>17.73597934600729</v>
       </c>
       <c r="F406" t="n">
         <v>7333800</v>
@@ -8592,16 +8592,16 @@
         <v>44848</v>
       </c>
       <c r="B409" t="n">
-        <v>18.39108085632324</v>
+        <v>18.39108276367188</v>
       </c>
       <c r="C409" t="n">
-        <v>18.94021183546421</v>
+        <v>18.9402137997635</v>
       </c>
       <c r="D409" t="n">
-        <v>18.29474166897004</v>
+        <v>18.29474356632728</v>
       </c>
       <c r="E409" t="n">
-        <v>18.80533807568002</v>
+        <v>18.80534002599148</v>
       </c>
       <c r="F409" t="n">
         <v>11391600</v>
@@ -8632,16 +8632,16 @@
         <v>44852</v>
       </c>
       <c r="B411" t="n">
-        <v>17.263916015625</v>
+        <v>17.26391792297363</v>
       </c>
       <c r="C411" t="n">
-        <v>19.16179004195282</v>
+        <v>19.16179215898201</v>
       </c>
       <c r="D411" t="n">
-        <v>17.263916015625</v>
+        <v>17.26391792297363</v>
       </c>
       <c r="E411" t="n">
-        <v>19.10398726647282</v>
+        <v>19.10398937711585</v>
       </c>
       <c r="F411" t="n">
         <v>33355700</v>
@@ -8712,16 +8712,16 @@
         <v>44858</v>
       </c>
       <c r="B415" t="n">
-        <v>18.00572776794434</v>
+        <v>18.0057258605957</v>
       </c>
       <c r="C415" t="n">
-        <v>18.36218040847837</v>
+        <v>18.36217846337067</v>
       </c>
       <c r="D415" t="n">
-        <v>17.54329998932035</v>
+        <v>17.54329813095674</v>
       </c>
       <c r="E415" t="n">
-        <v>17.91902267429717</v>
+        <v>17.91902077613322</v>
       </c>
       <c r="F415" t="n">
         <v>16227000</v>
@@ -8732,16 +8732,16 @@
         <v>44859</v>
       </c>
       <c r="B416" t="n">
-        <v>17.04233932495117</v>
+        <v>17.04233741760254</v>
       </c>
       <c r="C416" t="n">
-        <v>18.00572761270958</v>
+        <v>18.00572559754023</v>
       </c>
       <c r="D416" t="n">
-        <v>16.80149225301157</v>
+        <v>16.80149037261812</v>
       </c>
       <c r="E416" t="n">
-        <v>18.00572761270958</v>
+        <v>18.00572559754023</v>
       </c>
       <c r="F416" t="n">
         <v>27810400</v>
@@ -8752,16 +8752,16 @@
         <v>44860</v>
       </c>
       <c r="B417" t="n">
-        <v>16.45466995239258</v>
+        <v>16.45467185974121</v>
       </c>
       <c r="C417" t="n">
-        <v>17.07123779627069</v>
+        <v>17.07123977508899</v>
       </c>
       <c r="D417" t="n">
-        <v>16.36796486965758</v>
+        <v>16.36796676695576</v>
       </c>
       <c r="E417" t="n">
-        <v>17.0423373270371</v>
+        <v>17.0423393025054</v>
       </c>
       <c r="F417" t="n">
         <v>12823000</v>
@@ -8792,16 +8792,16 @@
         <v>44862</v>
       </c>
       <c r="B419" t="n">
-        <v>18.12133026123047</v>
+        <v>18.1213321685791</v>
       </c>
       <c r="C419" t="n">
-        <v>18.21766944200201</v>
+        <v>18.21767135949075</v>
       </c>
       <c r="D419" t="n">
-        <v>17.27354951297842</v>
+        <v>17.27355133109445</v>
       </c>
       <c r="E419" t="n">
-        <v>17.40842326354835</v>
+        <v>17.40842509586043</v>
       </c>
       <c r="F419" t="n">
         <v>12193800</v>
@@ -8932,16 +8932,16 @@
         <v>44874</v>
       </c>
       <c r="B426" t="n">
-        <v>19.65312004089355</v>
+        <v>19.65311813354492</v>
       </c>
       <c r="C426" t="n">
-        <v>20.09627959384678</v>
+        <v>20.09627764348921</v>
       </c>
       <c r="D426" t="n">
-        <v>19.1328913385332</v>
+        <v>19.13288948167312</v>
       </c>
       <c r="E426" t="n">
-        <v>19.1328913385332</v>
+        <v>19.13288948167312</v>
       </c>
       <c r="F426" t="n">
         <v>19633400</v>
@@ -9032,16 +9032,16 @@
         <v>44882</v>
       </c>
       <c r="B431" t="n">
-        <v>18.78607368469238</v>
+        <v>18.78607177734375</v>
       </c>
       <c r="C431" t="n">
-        <v>18.90168110049051</v>
+        <v>18.90167918140427</v>
       </c>
       <c r="D431" t="n">
-        <v>18.05389828468432</v>
+        <v>18.0538964516734</v>
       </c>
       <c r="E431" t="n">
-        <v>18.66083400196882</v>
+        <v>18.66083210733576</v>
       </c>
       <c r="F431" t="n">
         <v>10826800</v>
@@ -9232,16 +9232,16 @@
         <v>44896</v>
       </c>
       <c r="B441" t="n">
-        <v>18.95948219299316</v>
+        <v>18.95948028564453</v>
       </c>
       <c r="C441" t="n">
-        <v>19.08472186450934</v>
+        <v>19.08471994456143</v>
       </c>
       <c r="D441" t="n">
-        <v>18.41998525508773</v>
+        <v>18.41998340201319</v>
       </c>
       <c r="E441" t="n">
-        <v>19.0750877609285</v>
+        <v>19.0750858419498</v>
       </c>
       <c r="F441" t="n">
         <v>25518700</v>
@@ -9252,16 +9252,16 @@
         <v>44897</v>
       </c>
       <c r="B442" t="n">
-        <v>19.78799438476562</v>
+        <v>19.78799247741699</v>
       </c>
       <c r="C442" t="n">
-        <v>19.97103681859475</v>
+        <v>19.97103489360281</v>
       </c>
       <c r="D442" t="n">
-        <v>19.01728272713333</v>
+        <v>19.01728089407297</v>
       </c>
       <c r="E442" t="n">
-        <v>19.11362191402701</v>
+        <v>19.11362007168059</v>
       </c>
       <c r="F442" t="n">
         <v>24428900</v>
@@ -9352,16 +9352,16 @@
         <v>44904</v>
       </c>
       <c r="B447" t="n">
-        <v>18.57412528991699</v>
+        <v>18.57412719726562</v>
       </c>
       <c r="C447" t="n">
-        <v>18.7571677262095</v>
+        <v>18.75716965235448</v>
       </c>
       <c r="D447" t="n">
-        <v>18.25620725515131</v>
+        <v>18.25620912985342</v>
       </c>
       <c r="E447" t="n">
-        <v>18.57412528991699</v>
+        <v>18.57412719726562</v>
       </c>
       <c r="F447" t="n">
         <v>14833900</v>
@@ -9372,16 +9372,16 @@
         <v>44907</v>
       </c>
       <c r="B448" t="n">
-        <v>18.2562084197998</v>
+        <v>18.25621032714844</v>
       </c>
       <c r="C448" t="n">
-        <v>18.6704638316658</v>
+        <v>18.67046578229448</v>
       </c>
       <c r="D448" t="n">
-        <v>17.87085164245525</v>
+        <v>17.87085350954307</v>
       </c>
       <c r="E448" t="n">
-        <v>18.45851907414013</v>
+        <v>18.45852100262552</v>
       </c>
       <c r="F448" t="n">
         <v>10851800</v>
@@ -9392,16 +9392,16 @@
         <v>44908</v>
       </c>
       <c r="B449" t="n">
-        <v>17.94792175292969</v>
+        <v>17.94792366027832</v>
       </c>
       <c r="C449" t="n">
-        <v>18.52595505316863</v>
+        <v>18.5259570219456</v>
       </c>
       <c r="D449" t="n">
-        <v>17.89975307687528</v>
+        <v>17.89975497910497</v>
       </c>
       <c r="E449" t="n">
-        <v>18.52595505316863</v>
+        <v>18.5259570219456</v>
       </c>
       <c r="F449" t="n">
         <v>13648600</v>
@@ -9472,16 +9472,16 @@
         <v>44914</v>
       </c>
       <c r="B453" t="n">
-        <v>18.8342399597168</v>
+        <v>18.83424186706543</v>
       </c>
       <c r="C453" t="n">
-        <v>18.90167868218942</v>
+        <v>18.90168059636759</v>
       </c>
       <c r="D453" t="n">
-        <v>18.13096696301515</v>
+        <v>18.13096879914314</v>
       </c>
       <c r="E453" t="n">
-        <v>18.1502351694359</v>
+        <v>18.15023700751518</v>
       </c>
       <c r="F453" t="n">
         <v>7150400</v>
@@ -9652,16 +9652,16 @@
         <v>44928</v>
       </c>
       <c r="B462" t="n">
-        <v>18.32970237731934</v>
+        <v>18.32970428466797</v>
       </c>
       <c r="C462" t="n">
-        <v>18.50344392873929</v>
+        <v>18.50344585416709</v>
       </c>
       <c r="D462" t="n">
-        <v>17.90500101174039</v>
+        <v>17.90500287489553</v>
       </c>
       <c r="E462" t="n">
-        <v>18.33935489029029</v>
+        <v>18.33935679864334</v>
       </c>
       <c r="F462" t="n">
         <v>4837200</v>
@@ -9692,16 +9692,16 @@
         <v>44930</v>
       </c>
       <c r="B464" t="n">
-        <v>18.41657447814941</v>
+        <v>18.41657257080078</v>
       </c>
       <c r="C464" t="n">
-        <v>18.54205347374314</v>
+        <v>18.54205155339903</v>
       </c>
       <c r="D464" t="n">
-        <v>17.87604660008386</v>
+        <v>17.87604474871605</v>
       </c>
       <c r="E464" t="n">
-        <v>18.1752671595987</v>
+        <v>18.17526527724153</v>
       </c>
       <c r="F464" t="n">
         <v>9017200</v>
@@ -9732,16 +9732,16 @@
         <v>44932</v>
       </c>
       <c r="B466" t="n">
-        <v>18.37796592712402</v>
+        <v>18.37796401977539</v>
       </c>
       <c r="C466" t="n">
-        <v>18.85092804187709</v>
+        <v>18.85092608544231</v>
       </c>
       <c r="D466" t="n">
-        <v>18.20422436639255</v>
+        <v>18.2042224770756</v>
       </c>
       <c r="E466" t="n">
-        <v>18.33935587317094</v>
+        <v>18.33935396982943</v>
       </c>
       <c r="F466" t="n">
         <v>4999100</v>
@@ -9752,16 +9752,16 @@
         <v>44935</v>
       </c>
       <c r="B467" t="n">
-        <v>18.56135940551758</v>
+        <v>18.56135749816895</v>
       </c>
       <c r="C467" t="n">
-        <v>18.77371103444791</v>
+        <v>18.77370910527821</v>
       </c>
       <c r="D467" t="n">
-        <v>18.20422558763648</v>
+        <v>18.20422371698659</v>
       </c>
       <c r="E467" t="n">
-        <v>18.29109637383</v>
+        <v>18.29109449425335</v>
       </c>
       <c r="F467" t="n">
         <v>4878500</v>
@@ -9772,16 +9772,16 @@
         <v>44936</v>
       </c>
       <c r="B468" t="n">
-        <v>18.57101058959961</v>
+        <v>18.57101249694824</v>
       </c>
       <c r="C468" t="n">
-        <v>18.68683890990498</v>
+        <v>18.68684082914984</v>
       </c>
       <c r="D468" t="n">
-        <v>18.14630920318485</v>
+        <v>18.14631106691423</v>
       </c>
       <c r="E468" t="n">
-        <v>18.29109506382374</v>
+        <v>18.29109694242345</v>
       </c>
       <c r="F468" t="n">
         <v>7152400</v>
@@ -9992,16 +9992,16 @@
         <v>44951</v>
       </c>
       <c r="B479" t="n">
-        <v>20.37598991394043</v>
+        <v>20.37599182128906</v>
       </c>
       <c r="C479" t="n">
-        <v>20.6172972247506</v>
+        <v>20.61729915468745</v>
       </c>
       <c r="D479" t="n">
-        <v>20.12503008977441</v>
+        <v>20.12503197363128</v>
       </c>
       <c r="E479" t="n">
-        <v>20.57868717132721</v>
+        <v>20.57868909764986</v>
       </c>
       <c r="F479" t="n">
         <v>2807800</v>
@@ -10052,16 +10052,16 @@
         <v>44956</v>
       </c>
       <c r="B482" t="n">
-        <v>20.05746459960938</v>
+        <v>20.05746269226074</v>
       </c>
       <c r="C482" t="n">
-        <v>20.50146917361271</v>
+        <v>20.50146722404181</v>
       </c>
       <c r="D482" t="n">
-        <v>19.85476549854316</v>
+        <v>19.85476361047004</v>
       </c>
       <c r="E482" t="n">
-        <v>20.35668515343896</v>
+        <v>20.35668321763618</v>
       </c>
       <c r="F482" t="n">
         <v>14094800</v>
@@ -10152,16 +10152,16 @@
         <v>44963</v>
       </c>
       <c r="B487" t="n">
-        <v>18.55170631408691</v>
+        <v>18.55170440673828</v>
       </c>
       <c r="C487" t="n">
-        <v>18.66753463908353</v>
+        <v>18.66753271982629</v>
       </c>
       <c r="D487" t="n">
-        <v>18.24283323546763</v>
+        <v>18.24283135987503</v>
       </c>
       <c r="E487" t="n">
-        <v>18.45518485778996</v>
+        <v>18.45518296036495</v>
       </c>
       <c r="F487" t="n">
         <v>7136600</v>
@@ -10192,16 +10192,16 @@
         <v>44965</v>
       </c>
       <c r="B489" t="n">
-        <v>18.10770225524902</v>
+        <v>18.10770034790039</v>
       </c>
       <c r="C489" t="n">
-        <v>18.39727031469558</v>
+        <v>18.39726837684571</v>
       </c>
       <c r="D489" t="n">
-        <v>17.76987162520883</v>
+        <v>17.76986975344509</v>
       </c>
       <c r="E489" t="n">
-        <v>18.29109634144721</v>
+        <v>18.29109441478103</v>
       </c>
       <c r="F489" t="n">
         <v>14424900</v>
@@ -10212,16 +10212,16 @@
         <v>44966</v>
       </c>
       <c r="B490" t="n">
-        <v>17.87604904174805</v>
+        <v>17.87604713439941</v>
       </c>
       <c r="C490" t="n">
-        <v>18.04979062940028</v>
+        <v>18.04978870351367</v>
       </c>
       <c r="D490" t="n">
-        <v>17.69265493911191</v>
+        <v>17.69265305133117</v>
       </c>
       <c r="E490" t="n">
-        <v>17.91465726065466</v>
+        <v>17.91465534918659</v>
       </c>
       <c r="F490" t="n">
         <v>11653900</v>
@@ -10232,16 +10232,16 @@
         <v>44967</v>
       </c>
       <c r="B491" t="n">
-        <v>17.98221969604492</v>
+        <v>17.98222160339355</v>
       </c>
       <c r="C491" t="n">
-        <v>18.09804801338318</v>
+        <v>18.09804993301756</v>
       </c>
       <c r="D491" t="n">
-        <v>17.6250859128902</v>
+        <v>17.62508778235816</v>
       </c>
       <c r="E491" t="n">
-        <v>17.79882746838327</v>
+        <v>17.79882935627974</v>
       </c>
       <c r="F491" t="n">
         <v>6326900</v>
@@ -10272,16 +10272,16 @@
         <v>44971</v>
       </c>
       <c r="B493" t="n">
-        <v>17.80848121643066</v>
+        <v>17.80847930908203</v>
       </c>
       <c r="C493" t="n">
-        <v>18.11735429604525</v>
+        <v>18.11735235561527</v>
       </c>
       <c r="D493" t="n">
-        <v>17.71195791879391</v>
+        <v>17.71195602178325</v>
       </c>
       <c r="E493" t="n">
-        <v>18.0208309984085</v>
+        <v>18.02082906831649</v>
       </c>
       <c r="F493" t="n">
         <v>9612400</v>
@@ -10292,16 +10292,16 @@
         <v>44972</v>
       </c>
       <c r="B494" t="n">
-        <v>18.55170631408691</v>
+        <v>18.55170440673828</v>
       </c>
       <c r="C494" t="n">
-        <v>18.7737104502447</v>
+        <v>18.77370852007125</v>
       </c>
       <c r="D494" t="n">
-        <v>17.7602185898678</v>
+        <v>17.76021676389406</v>
       </c>
       <c r="E494" t="n">
-        <v>17.80848115904505</v>
+        <v>17.8084793281093</v>
       </c>
       <c r="F494" t="n">
         <v>12677500</v>
@@ -10312,16 +10312,16 @@
         <v>44973</v>
       </c>
       <c r="B495" t="n">
-        <v>18.3490104675293</v>
+        <v>18.34900856018066</v>
       </c>
       <c r="C495" t="n">
-        <v>18.55170775068378</v>
+        <v>18.5517058222651</v>
       </c>
       <c r="D495" t="n">
-        <v>17.88570081372285</v>
+        <v>17.88569895453448</v>
       </c>
       <c r="E495" t="n">
-        <v>18.43588125774662</v>
+        <v>18.43587934136792</v>
       </c>
       <c r="F495" t="n">
         <v>33990600</v>
@@ -10372,16 +10372,16 @@
         <v>44980</v>
       </c>
       <c r="B498" t="n">
-        <v>18.11735343933105</v>
+        <v>18.11735153198242</v>
       </c>
       <c r="C498" t="n">
-        <v>18.27178997183552</v>
+        <v>18.2717880482282</v>
       </c>
       <c r="D498" t="n">
-        <v>17.8470885869339</v>
+        <v>17.84708670803806</v>
       </c>
       <c r="E498" t="n">
-        <v>18.17526667876306</v>
+        <v>18.17526476531746</v>
       </c>
       <c r="F498" t="n">
         <v>5103300</v>
@@ -10392,16 +10392,16 @@
         <v>44981</v>
       </c>
       <c r="B499" t="n">
-        <v>18.04013633728027</v>
+        <v>18.04013442993164</v>
       </c>
       <c r="C499" t="n">
-        <v>18.16561533765205</v>
+        <v>18.16561341703677</v>
       </c>
       <c r="D499" t="n">
-        <v>17.82778471061123</v>
+        <v>17.82778282571412</v>
       </c>
       <c r="E499" t="n">
-        <v>18.10770209448268</v>
+        <v>18.10770017999045</v>
       </c>
       <c r="F499" t="n">
         <v>6522200</v>
@@ -10452,16 +10452,16 @@
         <v>44986</v>
       </c>
       <c r="B502" t="n">
-        <v>17.02664184570312</v>
+        <v>17.02664375305176</v>
       </c>
       <c r="C502" t="n">
-        <v>17.77952125559183</v>
+        <v>17.77952324727908</v>
       </c>
       <c r="D502" t="n">
-        <v>16.67916059893248</v>
+        <v>16.67916246735577</v>
       </c>
       <c r="E502" t="n">
-        <v>17.5092564271893</v>
+        <v>17.5092583886011</v>
       </c>
       <c r="F502" t="n">
         <v>19714300</v>
@@ -10652,16 +10652,16 @@
         <v>45000</v>
       </c>
       <c r="B512" t="n">
-        <v>16.15793800354004</v>
+        <v>16.15793609619141</v>
       </c>
       <c r="C512" t="n">
-        <v>16.43785537977234</v>
+        <v>16.43785343938112</v>
       </c>
       <c r="D512" t="n">
-        <v>15.6077576058738</v>
+        <v>15.6077557634707</v>
       </c>
       <c r="E512" t="n">
-        <v>15.7911516854388</v>
+        <v>15.79114982138712</v>
       </c>
       <c r="F512" t="n">
         <v>24755700</v>
@@ -10672,16 +10672,16 @@
         <v>45001</v>
       </c>
       <c r="B513" t="n">
-        <v>15.68497467041016</v>
+        <v>15.68497562408447</v>
       </c>
       <c r="C513" t="n">
-        <v>16.33167831507744</v>
+        <v>16.33167930807249</v>
       </c>
       <c r="D513" t="n">
-        <v>15.64636461829695</v>
+        <v>15.64636556962371</v>
       </c>
       <c r="E513" t="n">
-        <v>16.03245777531455</v>
+        <v>16.03245875011646</v>
       </c>
       <c r="F513" t="n">
         <v>11501700</v>
@@ -10712,16 +10712,16 @@
         <v>45005</v>
       </c>
       <c r="B515" t="n">
-        <v>15.49192810058594</v>
+        <v>15.49192905426025</v>
       </c>
       <c r="C515" t="n">
-        <v>15.59810390292816</v>
+        <v>15.5981048631386</v>
       </c>
       <c r="D515" t="n">
-        <v>15.31818746855065</v>
+        <v>15.31818841152959</v>
       </c>
       <c r="E515" t="n">
-        <v>15.44366737644599</v>
+        <v>15.4436683271494</v>
       </c>
       <c r="F515" t="n">
         <v>20828100</v>
@@ -10772,16 +10772,16 @@
         <v>45008</v>
       </c>
       <c r="B518" t="n">
-        <v>14.71974658966064</v>
+        <v>14.71974563598633</v>
       </c>
       <c r="C518" t="n">
-        <v>15.01896807290302</v>
+        <v>15.01896709984251</v>
       </c>
       <c r="D518" t="n">
-        <v>14.25643697491495</v>
+        <v>14.25643605125789</v>
       </c>
       <c r="E518" t="n">
-        <v>14.74870321045366</v>
+        <v>14.74870225490328</v>
       </c>
       <c r="F518" t="n">
         <v>25394300</v>
@@ -10792,16 +10792,16 @@
         <v>45009</v>
       </c>
       <c r="B519" t="n">
-        <v>14.43017768859863</v>
+        <v>14.43017673492432</v>
       </c>
       <c r="C519" t="n">
-        <v>14.95140146791577</v>
+        <v>14.95140047979436</v>
       </c>
       <c r="D519" t="n">
-        <v>14.01512972021653</v>
+        <v>14.01512879397227</v>
       </c>
       <c r="E519" t="n">
-        <v>14.74870328037497</v>
+        <v>14.74870230564966</v>
       </c>
       <c r="F519" t="n">
         <v>32819700</v>
@@ -10812,16 +10812,16 @@
         <v>45012</v>
       </c>
       <c r="B520" t="n">
-        <v>14.65218162536621</v>
+        <v>14.65218067169189</v>
       </c>
       <c r="C520" t="n">
-        <v>14.72939989865945</v>
+        <v>14.72939893995919</v>
       </c>
       <c r="D520" t="n">
-        <v>14.23713271602922</v>
+        <v>14.23713178936941</v>
       </c>
       <c r="E520" t="n">
-        <v>14.48809256448947</v>
+        <v>14.4880916214953</v>
       </c>
       <c r="F520" t="n">
         <v>14200700</v>
@@ -10852,16 +10852,16 @@
         <v>45014</v>
       </c>
       <c r="B522" t="n">
-        <v>14.89348697662354</v>
+        <v>14.89348793029785</v>
       </c>
       <c r="C522" t="n">
-        <v>14.96105272663084</v>
+        <v>14.96105368463159</v>
       </c>
       <c r="D522" t="n">
-        <v>14.4205239650295</v>
+        <v>14.42052488841858</v>
       </c>
       <c r="E522" t="n">
-        <v>14.84522533211219</v>
+        <v>14.84522628269617</v>
       </c>
       <c r="F522" t="n">
         <v>19793200</v>
@@ -10932,16 +10932,16 @@
         <v>45020</v>
       </c>
       <c r="B526" t="n">
-        <v>14.15991306304932</v>
+        <v>14.15991401672363</v>
       </c>
       <c r="C526" t="n">
-        <v>14.57496193194557</v>
+        <v>14.57496291357355</v>
       </c>
       <c r="D526" t="n">
-        <v>14.05373817774498</v>
+        <v>14.05373912426839</v>
       </c>
       <c r="E526" t="n">
-        <v>14.37226375417232</v>
+        <v>14.37226472214852</v>
       </c>
       <c r="F526" t="n">
         <v>12462300</v>
@@ -10972,16 +10972,16 @@
         <v>45022</v>
       </c>
       <c r="B528" t="n">
-        <v>13.1560754776001</v>
+        <v>13.15607452392578</v>
       </c>
       <c r="C528" t="n">
-        <v>13.57112437142145</v>
+        <v>13.57112338766055</v>
       </c>
       <c r="D528" t="n">
-        <v>13.00163893678686</v>
+        <v>13.00163799430754</v>
       </c>
       <c r="E528" t="n">
-        <v>13.33946863968721</v>
+        <v>13.33946767271886</v>
       </c>
       <c r="F528" t="n">
         <v>26117400</v>
@@ -11012,16 +11012,16 @@
         <v>45027</v>
       </c>
       <c r="B530" t="n">
-        <v>14.19852256774902</v>
+        <v>14.19852161407471</v>
       </c>
       <c r="C530" t="n">
-        <v>14.3240024830388</v>
+        <v>14.32400152093636</v>
       </c>
       <c r="D530" t="n">
-        <v>13.51320975071368</v>
+        <v>13.51320884306988</v>
       </c>
       <c r="E530" t="n">
-        <v>13.52286226431621</v>
+        <v>13.52286135602407</v>
       </c>
       <c r="F530" t="n">
         <v>23105700</v>
@@ -11052,16 +11052,16 @@
         <v>45029</v>
       </c>
       <c r="B532" t="n">
-        <v>13.27190208435059</v>
+        <v>13.2719030380249</v>
       </c>
       <c r="C532" t="n">
-        <v>14.14060803439325</v>
+        <v>14.14060905048986</v>
       </c>
       <c r="D532" t="n">
-        <v>13.27190208435059</v>
+        <v>13.2719030380249</v>
       </c>
       <c r="E532" t="n">
-        <v>14.09234730867981</v>
+        <v>14.09234832130857</v>
       </c>
       <c r="F532" t="n">
         <v>20136100</v>
@@ -11112,16 +11112,16 @@
         <v>45034</v>
       </c>
       <c r="B535" t="n">
-        <v>12.70241737365723</v>
+        <v>12.70241641998291</v>
       </c>
       <c r="C535" t="n">
-        <v>12.95337721125578</v>
+        <v>12.95337623873985</v>
       </c>
       <c r="D535" t="n">
-        <v>12.61554658983354</v>
+        <v>12.61554564268133</v>
       </c>
       <c r="E535" t="n">
-        <v>12.87615894130459</v>
+        <v>12.87615797458607</v>
       </c>
       <c r="F535" t="n">
         <v>12417000</v>
@@ -27509,162 +27509,142 @@
     </row>
     <row r="1355">
       <c r="A1355" s="1" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="B1355" t="n">
-        <v>8.5</v>
+        <v>8.550000190734863</v>
       </c>
       <c r="C1355" t="n">
-        <v>8.510000228881836</v>
+        <v>8.680000305175781</v>
       </c>
       <c r="D1355" t="n">
-        <v>8.340000152587891</v>
+        <v>8.439999580383301</v>
       </c>
       <c r="E1355" t="n">
-        <v>8.510000228881836</v>
+        <v>8.600000381469727</v>
       </c>
       <c r="F1355" t="n">
-        <v>3774300</v>
+        <v>5991300</v>
       </c>
     </row>
     <row r="1356">
       <c r="A1356" s="1" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B1356" t="n">
-        <v>8.550000190734863</v>
+        <v>8.659999847412109</v>
       </c>
       <c r="C1356" t="n">
-        <v>8.680000305175781</v>
+        <v>8.770000457763672</v>
       </c>
       <c r="D1356" t="n">
-        <v>8.439999580383301</v>
+        <v>8.590000152587891</v>
       </c>
       <c r="E1356" t="n">
-        <v>8.600000381469727</v>
+        <v>8.729999542236328</v>
       </c>
       <c r="F1356" t="n">
-        <v>5991300</v>
+        <v>5728800</v>
       </c>
     </row>
     <row r="1357">
       <c r="A1357" s="1" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="B1357" t="n">
-        <v>8.659999847412109</v>
+        <v>8.829999923706055</v>
       </c>
       <c r="C1357" t="n">
-        <v>8.770000457763672</v>
+        <v>8.909999847412109</v>
       </c>
       <c r="D1357" t="n">
-        <v>8.590000152587891</v>
+        <v>8.670000076293945</v>
       </c>
       <c r="E1357" t="n">
-        <v>8.729999542236328</v>
+        <v>8.710000038146973</v>
       </c>
       <c r="F1357" t="n">
-        <v>5728800</v>
+        <v>8653300</v>
       </c>
     </row>
     <row r="1358">
       <c r="A1358" s="1" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="B1358" t="n">
-        <v>8.829999923706055</v>
+        <v>8.489999771118164</v>
       </c>
       <c r="C1358" t="n">
-        <v>8.909999847412109</v>
+        <v>8.869999885559082</v>
       </c>
       <c r="D1358" t="n">
-        <v>8.670000076293945</v>
+        <v>8.489999771118164</v>
       </c>
       <c r="E1358" t="n">
-        <v>8.710000038146973</v>
+        <v>8.739999771118164</v>
       </c>
       <c r="F1358" t="n">
-        <v>8653300</v>
+        <v>9598300</v>
       </c>
     </row>
     <row r="1359">
       <c r="A1359" s="1" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="B1359" t="n">
-        <v>8.489999771118164</v>
+        <v>8.239999771118164</v>
       </c>
       <c r="C1359" t="n">
-        <v>8.869999885559082</v>
+        <v>8.630000114440918</v>
       </c>
       <c r="D1359" t="n">
-        <v>8.489999771118164</v>
+        <v>7.929999828338623</v>
       </c>
       <c r="E1359" t="n">
-        <v>8.739999771118164</v>
+        <v>8.619999885559082</v>
       </c>
       <c r="F1359" t="n">
-        <v>9598300</v>
+        <v>15405900</v>
       </c>
     </row>
     <row r="1360">
       <c r="A1360" s="1" t="n">
-        <v>46241</v>
+        <v>46245</v>
       </c>
       <c r="B1360" t="n">
-        <v>8.239999771118164</v>
+        <v>8.079999923706055</v>
       </c>
       <c r="C1360" t="n">
-        <v>8.630000114440918</v>
+        <v>8.189999580383301</v>
       </c>
       <c r="D1360" t="n">
-        <v>7.929999828338623</v>
+        <v>7.949999809265137</v>
       </c>
       <c r="E1360" t="n">
-        <v>8.619999885559082</v>
+        <v>8.060000419616699</v>
       </c>
       <c r="F1360" t="n">
-        <v>15405900</v>
+        <v>14248700</v>
       </c>
     </row>
     <row r="1361">
       <c r="A1361" s="1" t="n">
-        <v>46244</v>
+        <v>46246</v>
       </c>
       <c r="B1361" t="n">
-        <v>8.060000419616699</v>
+        <v>8</v>
       </c>
       <c r="C1361" t="n">
-        <v>8.229999542236328</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="D1361" t="n">
-        <v>7.960000038146973</v>
+        <v>7.95</v>
       </c>
       <c r="E1361" t="n">
-        <v>8.229999542236328</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="F1361" t="n">
-        <v>10741500</v>
-      </c>
-    </row>
-    <row r="1362">
-      <c r="A1362" s="1" t="n">
-        <v>46245</v>
-      </c>
-      <c r="B1362" t="n">
-        <v>8.08</v>
-      </c>
-      <c r="C1362" t="n">
-        <v>8.19</v>
-      </c>
-      <c r="D1362" t="n">
-        <v>7.95</v>
-      </c>
-      <c r="E1362" t="n">
-        <v>8.06</v>
-      </c>
-      <c r="F1362" t="n">
-        <v>14248700</v>
+        <v>8426200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>